<commit_message>
Atualização automática - 2026-08-20
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148308.64</v>
+        <v>148383.04</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150178.39</v>
+        <v>150253.73</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149243.51</v>
+        <v>149318.38</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113520.62</v>
+        <v>113577.57</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114292.45</v>
+        <v>114349.79</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>113906.53</v>
+        <v>113963.68</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>80942.86</v>
+        <v>80983.46000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81447.23</v>
+        <v>81488.09</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81195.05</v>
+        <v>81235.78</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57356.09</v>
+        <v>57384.86</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>56921.4</v>
+        <v>56949.95</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57138.74</v>
+        <v>57167.41</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37049.76</v>
+        <v>37068.34</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37352.84</v>
+        <v>37371.58</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37201.3</v>
+        <v>37219.96</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4962</v>
+        <v>13.4964</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16850.92</v>
+        <v>16859.37</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16740.27</v>
+        <v>16748.66</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16795.59</v>
+        <v>16804.02</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161092.5</v>
+        <v>161174.91</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160228.1</v>
+        <v>160310.07</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>160660.3</v>
+        <v>160742.49</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>120980.96</v>
+        <v>121042.85</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119272.27</v>
+        <v>119333.29</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120126.62</v>
+        <v>120188.07</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86433.37</v>
+        <v>86477.59</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85363.07000000001</v>
+        <v>85406.74000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>85898.22</v>
+        <v>85942.16</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>65840.57000000001</v>
+        <v>65874.25</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65377.72</v>
+        <v>65411.16</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65609.14</v>
+        <v>65642.71000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51435.72</v>
+        <v>51462.03</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49587.17</v>
+        <v>49612.53</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50511.44</v>
+        <v>50537.28</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.5219</v>
+        <v>13.5203</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>38991.06</v>
+        <v>39011.01</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>39954.55</v>
+        <v>39974.99</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39472.81</v>
+        <v>39493</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>165810.96</v>
+        <v>165896.2</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167338.35</v>
+        <v>167424.38</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>166574.65</v>
+        <v>166660.29</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119526.61</v>
+        <v>119588.06</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118098.01</v>
+        <v>118158.72</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>118812.31</v>
+        <v>118873.39</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>81877.61</v>
+        <v>81919.71000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81568.36</v>
+        <v>81610.28999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81722.98</v>
+        <v>81765</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54550.79</v>
+        <v>54578.84</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>54851.79</v>
+        <v>54879.99</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54701.29</v>
+        <v>54729.41</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>32924.19</v>
+        <v>32941.11</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32538.82</v>
+        <v>32555.55</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32731.5</v>
+        <v>32748.33</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5584</v>
+        <v>13.5567</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17092.84</v>
+        <v>17101.63</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17770.48</v>
+        <v>17779.62</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17431.66</v>
+        <v>17440.62</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128100.53</v>
+        <v>128166.72</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128194.4</v>
+        <v>128260.63</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128147.46</v>
+        <v>128213.67</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>88716.33</v>
+        <v>88762.17</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87339.71000000001</v>
+        <v>87384.83</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88028.02</v>
+        <v>88073.5</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55763.19</v>
+        <v>55792.01</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56047.78</v>
+        <v>56076.74</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>55905.49</v>
+        <v>55934.37</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29521.08</v>
+        <v>29536.33</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29719.78</v>
+        <v>29735.14</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29620.43</v>
+        <v>29635.73</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6770.9</v>
+        <v>6774.4</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6769.61</v>
+        <v>6773.11</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6770.25</v>
+        <v>6773.75</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.5948</v>
+        <v>13.5932</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3762.21</v>
+        <v>3764.16</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3673.47</v>
+        <v>3675.37</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3717.84</v>
+        <v>3719.76</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108117.94</v>
+        <v>108174.06</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108592.26</v>
+        <v>108648.63</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108355.1</v>
+        <v>108411.35</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>75821.67</v>
+        <v>75861.03</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75282.23</v>
+        <v>75321.31</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75551.95</v>
+        <v>75591.17</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>45879.79</v>
+        <v>45903.61</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>46976.72</v>
+        <v>47001.1</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46428.25</v>
+        <v>46452.35</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28503.23</v>
+        <v>28518.03</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28397</v>
+        <v>28411.75</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28450.12</v>
+        <v>28464.89</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>13982.43</v>
+        <v>13989.69</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14103.65</v>
+        <v>14110.98</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14043.04</v>
+        <v>14050.33</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.6296</v>
+        <v>13.628</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6482.26</v>
+        <v>6485.63</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6322.12</v>
+        <v>6325.4</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6402.19</v>
+        <v>6405.51</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49190.36</v>
+        <v>49216.02</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>48861.04</v>
+        <v>48886.52</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49025.7</v>
+        <v>49051.27</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43274.38</v>
+        <v>43296.95</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43466.5</v>
+        <v>43489.17</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43370.44</v>
+        <v>43393.06</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31670.34</v>
+        <v>31686.86</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32007.61</v>
+        <v>32024.31</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31838.98</v>
+        <v>31855.58</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22268.32</v>
+        <v>22279.94</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22421.25</v>
+        <v>22432.95</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22344.79</v>
+        <v>22356.44</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14312.56</v>
+        <v>14320.02</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14516.23</v>
+        <v>14523.8</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14414.39</v>
+        <v>14421.91</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.6661</v>
+        <v>13.6644</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8225.440000000001</v>
+        <v>8229.73</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8279.93</v>
+        <v>8284.25</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8252.690000000001</v>
+        <v>8256.99</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48373.84</v>
+        <v>48399.21</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47661.91</v>
+        <v>47686.89</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48017.87</v>
+        <v>48043.05</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43319.46</v>
+        <v>43342.17</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>42986.68</v>
+        <v>43009.22</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43153.07</v>
+        <v>43175.69</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31285.33</v>
+        <v>31301.73</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30722.92</v>
+        <v>30739.03</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31004.13</v>
+        <v>31020.38</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23317.95</v>
+        <v>23330.17</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23213.98</v>
+        <v>23226.15</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23265.97</v>
+        <v>23278.16</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18292.63</v>
+        <v>18302.22</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18108.8</v>
+        <v>18118.3</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18200.72</v>
+        <v>18210.26</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.7042</v>
+        <v>13.7025</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15385.35</v>
+        <v>15393.42</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15330.42</v>
+        <v>15338.46</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15357.89</v>
+        <v>15365.94</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>122747.62</v>
+        <v>122810.07</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123369.24</v>
+        <v>123432.01</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123058.43</v>
+        <v>123121.04</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88023.17</v>
+        <v>88067.96000000001</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88379.00999999999</v>
+        <v>88423.97</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88201.09</v>
+        <v>88245.97</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57500.5</v>
+        <v>57529.76</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57012.16</v>
+        <v>57041.16</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57256.33</v>
+        <v>57285.46</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33058.88</v>
+        <v>33075.7</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32820.67</v>
+        <v>32837.37</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>32939.77</v>
+        <v>32956.53</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18787.02</v>
+        <v>18796.58</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18712.79</v>
+        <v>18722.31</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18749.91</v>
+        <v>18759.45</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7616.95</v>
+        <v>7620.83</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7375.93</v>
+        <v>7379.68</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7496.44</v>
+        <v>7500.26</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>399429.41</v>
+        <v>399629.31</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>394487.48</v>
+        <v>394684.9</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>396958.45</v>
+        <v>397157.1</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>299863.44</v>
+        <v>300013.51</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>300835.97</v>
+        <v>300986.52</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>300349.71</v>
+        <v>300500.01</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>209815.38</v>
+        <v>209920.38</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>209688.8</v>
+        <v>209793.74</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>209752.09</v>
+        <v>209857.06</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127555.54</v>
+        <v>127619.37</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>127836.68</v>
+        <v>127900.66</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>127696.11</v>
+        <v>127760.01</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>61827.82</v>
+        <v>61858.76</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61538.98</v>
+        <v>61569.78</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61683.4</v>
+        <v>61714.27</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6088</v>
+        <v>13.614</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31576.49</v>
+        <v>31592.29</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31600.33</v>
+        <v>31616.15</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31588.41</v>
+        <v>31604.22</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>402953.75</v>
+        <v>403154.41</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>403495.36</v>
+        <v>403696.29</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>403224.55</v>
+        <v>403425.35</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299108.28</v>
+        <v>299257.23</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>297240.68</v>
+        <v>297388.69</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>298174.48</v>
+        <v>298322.96</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>202885.41</v>
+        <v>202986.45</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>202954.82</v>
+        <v>203055.89</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>202920.12</v>
+        <v>203021.17</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>122773.01</v>
+        <v>122834.15</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123284.91</v>
+        <v>123346.3</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123028.96</v>
+        <v>123090.23</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49030.07</v>
+        <v>49054.49</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>48971.64</v>
+        <v>48996.03</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49000.86</v>
+        <v>49025.26</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5248</v>
+        <v>13.5277</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5393.15</v>
+        <v>5395.83</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5428.71</v>
+        <v>5431.42</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5410.93</v>
+        <v>5413.63</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168281.22</v>
+        <v>168365.75</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168308.14</v>
+        <v>168392.68</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168294.68</v>
+        <v>168379.21</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110588.71</v>
+        <v>110644.25</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110203.99</v>
+        <v>110259.35</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110396.35</v>
+        <v>110451.8</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>61934.56</v>
+        <v>61965.67</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62285.85</v>
+        <v>62317.14</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62110.21</v>
+        <v>62141.4</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26514.78</v>
+        <v>26528.1</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26712.32</v>
+        <v>26725.74</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26613.55</v>
+        <v>26626.92</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6241.3</v>
+        <v>6244.43</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6391.33</v>
+        <v>6394.54</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6316.31</v>
+        <v>6319.49</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5051</v>
+        <v>13.5053</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3696.42</v>
+        <v>3698.28</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3690.01</v>
+        <v>3691.86</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3693.22</v>
+        <v>3695.07</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188206.48</v>
+        <v>188300.95</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189125.47</v>
+        <v>189220.4</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>188665.97</v>
+        <v>188760.68</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136453.68</v>
+        <v>136522.17</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137405.9</v>
+        <v>137474.87</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>136929.79</v>
+        <v>136998.52</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86252.39999999999</v>
+        <v>86295.69</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>86950.39999999999</v>
+        <v>86994.05</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86601.39999999999</v>
+        <v>86644.87</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41199.53</v>
+        <v>41220.21</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41133.45</v>
+        <v>41154.1</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41166.49</v>
+        <v>41187.15</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12847.4</v>
+        <v>12853.85</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12705.89</v>
+        <v>12712.27</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12776.65</v>
+        <v>12783.06</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5006</v>
+        <v>13.5008</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4458.85</v>
+        <v>4461.09</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4350.01</v>
+        <v>4352.19</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4404.43</v>
+        <v>4406.64</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-22
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148439.9</v>
+        <v>148459.42</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150311.31</v>
+        <v>150331.07</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149375.6</v>
+        <v>149395.24</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113621.09</v>
+        <v>113636.03</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114393.6</v>
+        <v>114408.64</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114007.35</v>
+        <v>114022.34</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81014.5</v>
+        <v>81025.14999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81519.32000000001</v>
+        <v>81530.03999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81266.91</v>
+        <v>81277.59</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57406.85</v>
+        <v>57414.4</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>56971.77</v>
+        <v>56979.27</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57189.31</v>
+        <v>57196.83</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37082.55</v>
+        <v>37087.43</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37385.9</v>
+        <v>37390.81</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37234.22</v>
+        <v>37239.12</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.5248</v>
+        <v>13.4935</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16865.84</v>
+        <v>16868.05</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16755.08</v>
+        <v>16757.29</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16810.46</v>
+        <v>16812.67</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161236.88</v>
+        <v>161265.21</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160371.71</v>
+        <v>160399.89</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>160804.3</v>
+        <v>160832.55</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121089.39</v>
+        <v>121110.66</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119379.17</v>
+        <v>119400.15</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120234.28</v>
+        <v>120255.41</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86510.84</v>
+        <v>86526.03999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85439.58</v>
+        <v>85454.59</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>85975.21000000001</v>
+        <v>85990.31</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>65899.58</v>
+        <v>65911.16</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65436.31</v>
+        <v>65447.81</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65667.95</v>
+        <v>65679.48</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51481.82</v>
+        <v>51490.86</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49631.61</v>
+        <v>49640.33</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50556.71</v>
+        <v>50565.6</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.5445</v>
+        <v>13.5086</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39026.01</v>
+        <v>39032.86</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>39990.36</v>
+        <v>39997.39</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39508.18</v>
+        <v>39515.13</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>165957.21</v>
+        <v>165995.37</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167485.95</v>
+        <v>167524.47</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>166721.58</v>
+        <v>166759.92</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119632.03</v>
+        <v>119659.54</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118202.17</v>
+        <v>118229.35</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>118917.1</v>
+        <v>118944.45</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>81949.83</v>
+        <v>81968.67999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81640.31</v>
+        <v>81659.08</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81795.07000000001</v>
+        <v>81813.88</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54598.91</v>
+        <v>54611.47</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>54900.17</v>
+        <v>54912.79</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54749.54</v>
+        <v>54762.13</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>32953.23</v>
+        <v>32960.8</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32567.52</v>
+        <v>32575.01</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32760.37</v>
+        <v>32767.91</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5809</v>
+        <v>13.5403</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17107.91</v>
+        <v>17111.85</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17786.16</v>
+        <v>17790.25</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17447.04</v>
+        <v>17451.05</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128211.72</v>
+        <v>128249.09</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128305.67</v>
+        <v>128343.06</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128258.7</v>
+        <v>128296.07</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>88793.34</v>
+        <v>88819.21000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87415.52</v>
+        <v>87440.99000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88104.42999999999</v>
+        <v>88130.10000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55811.6</v>
+        <v>55827.86</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56096.43</v>
+        <v>56112.77</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>55954.01</v>
+        <v>55970.32</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29546.7</v>
+        <v>29555.31</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29745.58</v>
+        <v>29754.25</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29646.14</v>
+        <v>29654.78</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6776.78</v>
+        <v>6778.75</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6775.49</v>
+        <v>6777.46</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6776.13</v>
+        <v>6778.11</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.6172</v>
+        <v>13.5719</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3765.48</v>
+        <v>3766.57</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3676.66</v>
+        <v>3677.73</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3721.07</v>
+        <v>3722.15</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108210.35</v>
+        <v>108248.96</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108685.08</v>
+        <v>108723.86</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108447.72</v>
+        <v>108486.41</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>75886.48</v>
+        <v>75913.56</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75346.58</v>
+        <v>75373.47</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75616.53</v>
+        <v>75643.50999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>45919.01</v>
+        <v>45935.39</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47016.87</v>
+        <v>47033.65</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46467.94</v>
+        <v>46484.52</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28527.59</v>
+        <v>28537.77</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28421.28</v>
+        <v>28431.42</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28474.43</v>
+        <v>28484.59</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>13994.38</v>
+        <v>13999.38</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14115.71</v>
+        <v>14120.75</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14055.05</v>
+        <v>14060.06</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.6519</v>
+        <v>13.6021</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6487.8</v>
+        <v>6490.12</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6327.52</v>
+        <v>6329.78</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6407.66</v>
+        <v>6409.95</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49231.73</v>
+        <v>49253.01</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>48902.13</v>
+        <v>48923.27</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49066.93</v>
+        <v>49088.14</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43310.77</v>
+        <v>43329.5</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43503.05</v>
+        <v>43521.86</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43406.91</v>
+        <v>43425.68</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31696.97</v>
+        <v>31710.68</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32034.53</v>
+        <v>32048.38</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31865.75</v>
+        <v>31879.53</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22287.05</v>
+        <v>22296.68</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22440.11</v>
+        <v>22449.81</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22363.58</v>
+        <v>22373.25</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14324.59</v>
+        <v>14330.79</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14528.44</v>
+        <v>14534.72</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14426.52</v>
+        <v>14432.75</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.6883</v>
+        <v>13.6337</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8232.360000000001</v>
+        <v>8235.92</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8286.9</v>
+        <v>8290.48</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8259.629999999999</v>
+        <v>8263.200000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48413.84</v>
+        <v>48438.97</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47701.32</v>
+        <v>47726.08</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48057.58</v>
+        <v>48082.52</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43355.28</v>
+        <v>43377.78</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43022.22</v>
+        <v>43044.56</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43188.75</v>
+        <v>43211.17</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31311.2</v>
+        <v>31327.45</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30748.33</v>
+        <v>30764.29</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31029.76</v>
+        <v>31045.87</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23337.23</v>
+        <v>23349.34</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23233.18</v>
+        <v>23245.24</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23285.2</v>
+        <v>23297.29</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18307.76</v>
+        <v>18317.26</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18123.78</v>
+        <v>18133.18</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18215.77</v>
+        <v>18225.22</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.7263</v>
+        <v>13.6668</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15398.07</v>
+        <v>15406.07</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15343.1</v>
+        <v>15351.06</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15370.59</v>
+        <v>15378.56</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>122869.33</v>
+        <v>122868.94</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123491.57</v>
+        <v>123491.18</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123180.45</v>
+        <v>123180.06</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88110.46000000001</v>
+        <v>88110.17999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88466.64</v>
+        <v>88466.36</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88288.55</v>
+        <v>88288.27</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57557.52</v>
+        <v>57557.34</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57068.69</v>
+        <v>57068.51</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57313.1</v>
+        <v>57312.92</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33091.66</v>
+        <v>33091.55</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32853.22</v>
+        <v>32853.11</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>32972.44</v>
+        <v>32972.33</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18805.65</v>
+        <v>18805.59</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18731.34</v>
+        <v>18731.28</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18768.5</v>
+        <v>18768.44</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.7515</v>
+        <v>13.7606</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7624.51</v>
+        <v>7624.48</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7383.24</v>
+        <v>7383.22</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7503.88</v>
+        <v>7503.85</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>399798.99</v>
+        <v>399798.6</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>394852.49</v>
+        <v>394852.1</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>397325.74</v>
+        <v>397325.35</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300140.9</v>
+        <v>300140.6</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301114.32</v>
+        <v>301114.02</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>300627.61</v>
+        <v>300627.31</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210009.51</v>
+        <v>210009.3</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>209882.82</v>
+        <v>209882.61</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>209946.16</v>
+        <v>209945.96</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127673.56</v>
+        <v>127673.43</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>127954.96</v>
+        <v>127954.84</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>127814.26</v>
+        <v>127814.14</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>61885.02</v>
+        <v>61884.96</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61595.92</v>
+        <v>61595.86</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61740.47</v>
+        <v>61740.41</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6873</v>
+        <v>13.6882</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31605.7</v>
+        <v>31605.67</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31629.57</v>
+        <v>31629.54</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31617.64</v>
+        <v>31617.61</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>403313.29</v>
+        <v>403323.16</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>403855.39</v>
+        <v>403865.27</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>403584.34</v>
+        <v>403594.21</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299375.16</v>
+        <v>299382.49</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>297505.9</v>
+        <v>297513.17</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>298440.53</v>
+        <v>298447.83</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203066.44</v>
+        <v>203071.41</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203135.91</v>
+        <v>203140.88</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203101.18</v>
+        <v>203106.15</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>122882.56</v>
+        <v>122885.57</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123394.91</v>
+        <v>123397.93</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123138.74</v>
+        <v>123141.75</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49073.82</v>
+        <v>49075.02</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49015.34</v>
+        <v>49016.54</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49044.58</v>
+        <v>49045.78</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5846</v>
+        <v>13.5719</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5397.96</v>
+        <v>5398.09</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5433.56</v>
+        <v>5433.69</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5415.76</v>
+        <v>5415.89</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168430.47</v>
+        <v>168439.14</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168457.41</v>
+        <v>168466.08</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168443.94</v>
+        <v>168452.61</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110686.79</v>
+        <v>110692.48</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110301.73</v>
+        <v>110307.41</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110494.26</v>
+        <v>110499.95</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>61989.49</v>
+        <v>61992.68</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62341.1</v>
+        <v>62344.3</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62165.29</v>
+        <v>62168.49</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26538.3</v>
+        <v>26539.67</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26736.01</v>
+        <v>26737.39</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26637.16</v>
+        <v>26638.53</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6246.83</v>
+        <v>6247.16</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6397</v>
+        <v>6397.33</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6321.92</v>
+        <v>6322.24</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5505</v>
+        <v>13.5308</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3699.7</v>
+        <v>3699.89</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3693.28</v>
+        <v>3693.47</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3696.49</v>
+        <v>3696.68</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188371.99</v>
+        <v>188388.51</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189291.78</v>
+        <v>189308.39</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>188831.88</v>
+        <v>188848.45</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136573.67</v>
+        <v>136585.66</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137526.73</v>
+        <v>137538.8</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137050.2</v>
+        <v>137062.23</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86328.25</v>
+        <v>86335.82000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87026.87</v>
+        <v>87034.5</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86677.56</v>
+        <v>86685.16</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41235.76</v>
+        <v>41239.37</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41169.62</v>
+        <v>41173.24</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41202.69</v>
+        <v>41206.31</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12858.7</v>
+        <v>12859.83</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12717.07</v>
+        <v>12718.18</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12787.88</v>
+        <v>12789</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5374</v>
+        <v>13.5117</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4462.77</v>
+        <v>4463.16</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4353.83</v>
+        <v>4354.21</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4408.3</v>
+        <v>4408.69</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-25
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148459.42</v>
+        <v>148600.27</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150331.07</v>
+        <v>150473.7</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149395.24</v>
+        <v>149536.99</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113636.03</v>
+        <v>113743.84</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114408.64</v>
+        <v>114517.19</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114022.34</v>
+        <v>114130.52</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81025.14999999999</v>
+        <v>81102.02</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81530.03999999999</v>
+        <v>81607.39</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81277.59</v>
+        <v>81354.71000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57414.4</v>
+        <v>57468.87</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>56979.27</v>
+        <v>57033.33</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57196.83</v>
+        <v>57251.1</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37087.43</v>
+        <v>37122.61</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37390.81</v>
+        <v>37426.29</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37239.12</v>
+        <v>37274.45</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4935</v>
+        <v>13.5071</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16868.05</v>
+        <v>16884.06</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16757.29</v>
+        <v>16773.18</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16812.67</v>
+        <v>16828.62</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161265.21</v>
+        <v>161417.96</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160399.89</v>
+        <v>160551.82</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>160832.55</v>
+        <v>160984.89</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121110.66</v>
+        <v>121225.38</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119400.15</v>
+        <v>119513.25</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120255.41</v>
+        <v>120369.31</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86526.03999999999</v>
+        <v>86608</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85454.59</v>
+        <v>85535.53</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>85990.31</v>
+        <v>86071.77</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>65911.16</v>
+        <v>65973.59</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65447.81</v>
+        <v>65509.8</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65679.48</v>
+        <v>65741.7</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51490.86</v>
+        <v>51539.64</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49640.33</v>
+        <v>49687.35</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50565.6</v>
+        <v>50613.49</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.5086</v>
+        <v>13.5208</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39032.86</v>
+        <v>39069.84</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>39997.39</v>
+        <v>40035.27</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39515.13</v>
+        <v>39552.55</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>165995.37</v>
+        <v>166150.61</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167524.47</v>
+        <v>167681.13</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>166759.92</v>
+        <v>166915.87</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119659.54</v>
+        <v>119771.44</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118229.35</v>
+        <v>118339.92</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>118944.45</v>
+        <v>119055.68</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>81968.67999999999</v>
+        <v>82045.33</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81659.08</v>
+        <v>81735.44</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81813.88</v>
+        <v>81890.39</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54611.47</v>
+        <v>54662.54</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>54912.79</v>
+        <v>54964.15</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54762.13</v>
+        <v>54813.34</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>32960.8</v>
+        <v>32991.63</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32575.01</v>
+        <v>32605.47</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32767.91</v>
+        <v>32798.55</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5403</v>
+        <v>13.5533</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17111.85</v>
+        <v>17127.85</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17790.25</v>
+        <v>17806.89</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17451.05</v>
+        <v>17467.37</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128249.09</v>
+        <v>128367.3</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128343.06</v>
+        <v>128461.36</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128296.07</v>
+        <v>128414.33</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>88819.21000000001</v>
+        <v>88901.08</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87440.99000000001</v>
+        <v>87521.59</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88130.10000000001</v>
+        <v>88211.34</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55827.86</v>
+        <v>55879.32</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56112.77</v>
+        <v>56164.5</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>55970.32</v>
+        <v>56021.91</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29555.31</v>
+        <v>29582.55</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29754.25</v>
+        <v>29781.68</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29654.78</v>
+        <v>29682.11</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6778.75</v>
+        <v>6785</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6777.46</v>
+        <v>6783.71</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6778.11</v>
+        <v>6784.35</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5859</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3766.57</v>
+        <v>3770.05</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3677.73</v>
+        <v>3681.12</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3722.15</v>
+        <v>3725.59</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108248.96</v>
+        <v>108347.23</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108723.86</v>
+        <v>108822.55</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108486.41</v>
+        <v>108584.89</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>75913.56</v>
+        <v>75982.47</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75373.47</v>
+        <v>75441.89</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75643.50999999999</v>
+        <v>75712.17999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>45935.39</v>
+        <v>45977.09</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47033.65</v>
+        <v>47076.34</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46484.52</v>
+        <v>46526.72</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28537.77</v>
+        <v>28563.68</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28431.42</v>
+        <v>28457.23</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28484.59</v>
+        <v>28510.45</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>13999.38</v>
+        <v>14012.08</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14120.75</v>
+        <v>14133.56</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14060.06</v>
+        <v>14072.82</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.6021</v>
+        <v>13.6169</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6490.12</v>
+        <v>6496.01</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6329.78</v>
+        <v>6335.53</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6409.95</v>
+        <v>6415.77</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49253.01</v>
+        <v>49296.94</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>48923.27</v>
+        <v>48966.9</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49088.14</v>
+        <v>49131.92</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43329.5</v>
+        <v>43368.14</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43521.86</v>
+        <v>43560.68</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43425.68</v>
+        <v>43464.41</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31710.68</v>
+        <v>31738.96</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32048.38</v>
+        <v>32076.96</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31879.53</v>
+        <v>31907.96</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22296.68</v>
+        <v>22316.57</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22449.81</v>
+        <v>22469.83</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22373.25</v>
+        <v>22393.2</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14330.79</v>
+        <v>14343.57</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14534.72</v>
+        <v>14547.68</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14432.75</v>
+        <v>14445.63</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.6337</v>
+        <v>13.6494</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8235.92</v>
+        <v>8243.26</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8290.48</v>
+        <v>8297.870000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8263.200000000001</v>
+        <v>8270.57</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48438.97</v>
+        <v>48481.29</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47726.08</v>
+        <v>47767.77</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48082.52</v>
+        <v>48124.53</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43377.78</v>
+        <v>43415.68</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43044.56</v>
+        <v>43082.16</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43211.17</v>
+        <v>43248.92</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31327.45</v>
+        <v>31354.82</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30764.29</v>
+        <v>30791.16</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31045.87</v>
+        <v>31072.99</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23349.34</v>
+        <v>23369.74</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23245.24</v>
+        <v>23265.55</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23297.29</v>
+        <v>23317.64</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18317.26</v>
+        <v>18333.26</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18133.18</v>
+        <v>18149.02</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18225.22</v>
+        <v>18241.14</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.6668</v>
+        <v>13.6834</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15406.07</v>
+        <v>15419.53</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15351.06</v>
+        <v>15364.47</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15378.56</v>
+        <v>15392</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>122868.94</v>
+        <v>122996.72</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123491.18</v>
+        <v>123619.6</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123180.06</v>
+        <v>123308.16</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88110.17999999999</v>
+        <v>88201.81</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88466.36</v>
+        <v>88558.36</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88288.27</v>
+        <v>88380.09</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57557.34</v>
+        <v>57617.19</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57068.51</v>
+        <v>57127.86</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57312.92</v>
+        <v>57372.53</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33091.55</v>
+        <v>33125.97</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32853.11</v>
+        <v>32887.28</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>32972.33</v>
+        <v>33006.62</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18805.59</v>
+        <v>18825.15</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18731.28</v>
+        <v>18750.76</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18768.44</v>
+        <v>18787.96</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.7606</v>
+        <v>13.7025</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7624.48</v>
+        <v>7632.41</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7383.22</v>
+        <v>7390.9</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7503.85</v>
+        <v>7511.66</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>399798.6</v>
+        <v>400218.85</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>394852.1</v>
+        <v>395267.15</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>397325.35</v>
+        <v>397743</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300140.6</v>
+        <v>300456.1</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301114.02</v>
+        <v>301430.54</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>300627.31</v>
+        <v>300943.32</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210009.3</v>
+        <v>210230.06</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>209882.61</v>
+        <v>210103.23</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>209945.96</v>
+        <v>210166.64</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127673.43</v>
+        <v>127807.64</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>127954.84</v>
+        <v>128089.34</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>127814.14</v>
+        <v>127948.49</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>61884.96</v>
+        <v>61950.01</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61595.86</v>
+        <v>61660.6</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61740.41</v>
+        <v>61805.31</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6882</v>
+        <v>13.6572</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31605.67</v>
+        <v>31638.89</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31629.54</v>
+        <v>31662.79</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31617.61</v>
+        <v>31650.84</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>403323.16</v>
+        <v>403736.39</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>403865.27</v>
+        <v>404279.06</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>403594.21</v>
+        <v>404007.73</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299382.49</v>
+        <v>299689.23</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>297513.17</v>
+        <v>297818</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>298447.83</v>
+        <v>298753.61</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203071.41</v>
+        <v>203279.47</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203140.88</v>
+        <v>203349.01</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203106.15</v>
+        <v>203314.24</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>122885.57</v>
+        <v>123011.47</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123397.93</v>
+        <v>123524.36</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123141.75</v>
+        <v>123267.92</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49075.02</v>
+        <v>49125.3</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49016.54</v>
+        <v>49066.76</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49045.78</v>
+        <v>49096.03</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5719</v>
+        <v>13.5643</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5398.09</v>
+        <v>5403.62</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5433.69</v>
+        <v>5439.26</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5415.89</v>
+        <v>5421.44</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168439.14</v>
+        <v>168609.37</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168466.08</v>
+        <v>168636.34</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168452.61</v>
+        <v>168622.85</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110692.48</v>
+        <v>110804.35</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110307.41</v>
+        <v>110418.89</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110499.95</v>
+        <v>110611.62</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>61992.68</v>
+        <v>62055.33</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62344.3</v>
+        <v>62407.31</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62168.49</v>
+        <v>62231.32</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26539.67</v>
+        <v>26566.49</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26737.39</v>
+        <v>26764.41</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26638.53</v>
+        <v>26665.45</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6247.16</v>
+        <v>6253.47</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6397.33</v>
+        <v>6403.79</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6322.24</v>
+        <v>6328.63</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5308</v>
+        <v>13.5297</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3699.89</v>
+        <v>3703.63</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3693.47</v>
+        <v>3697.21</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3696.68</v>
+        <v>3700.42</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188388.51</v>
+        <v>188574.05</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189308.39</v>
+        <v>189494.83</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>188848.45</v>
+        <v>189034.44</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136585.66</v>
+        <v>136720.17</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137538.8</v>
+        <v>137674.25</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137062.23</v>
+        <v>137197.21</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86335.82000000001</v>
+        <v>86420.85000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87034.5</v>
+        <v>87120.22</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86685.16</v>
+        <v>86770.53</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41239.37</v>
+        <v>41279.99</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41173.24</v>
+        <v>41213.79</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41206.31</v>
+        <v>41246.89</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12859.83</v>
+        <v>12872.49</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12718.18</v>
+        <v>12730.71</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12789</v>
+        <v>12801.6</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5117</v>
+        <v>13.5181</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4463.16</v>
+        <v>4467.56</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4354.21</v>
+        <v>4358.5</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4408.69</v>
+        <v>4413.03</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-26
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148600.27</v>
+        <v>148697.99</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150473.7</v>
+        <v>150572.64</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149536.99</v>
+        <v>149635.31</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113743.84</v>
+        <v>113818.64</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114517.19</v>
+        <v>114592.49</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114130.52</v>
+        <v>114205.57</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81102.02</v>
+        <v>81155.35000000001</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81607.39</v>
+        <v>81661.05</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81354.71000000001</v>
+        <v>81408.2</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57468.87</v>
+        <v>57506.66</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57033.33</v>
+        <v>57070.83</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57251.1</v>
+        <v>57288.74</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37122.61</v>
+        <v>37147.02</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37426.29</v>
+        <v>37450.9</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37274.45</v>
+        <v>37298.96</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.5071</v>
+        <v>13.4693</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16884.06</v>
+        <v>16895.16</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16773.18</v>
+        <v>16784.21</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16828.62</v>
+        <v>16839.69</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161417.96</v>
+        <v>161534.32</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160551.82</v>
+        <v>160667.55</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>160984.89</v>
+        <v>161100.93</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121225.38</v>
+        <v>121312.76</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119513.25</v>
+        <v>119599.4</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120369.31</v>
+        <v>120456.08</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86608</v>
+        <v>86670.42999999999</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85535.53</v>
+        <v>85597.19</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86071.77</v>
+        <v>86133.81</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>65973.59</v>
+        <v>66021.14</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65509.8</v>
+        <v>65557.03</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65741.7</v>
+        <v>65789.08</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51539.64</v>
+        <v>51576.79</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49687.35</v>
+        <v>49723.17</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50613.49</v>
+        <v>50649.98</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.5208</v>
+        <v>13.4755</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39069.84</v>
+        <v>39098</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40035.27</v>
+        <v>40064.13</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39552.55</v>
+        <v>39581.07</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166150.61</v>
+        <v>166279.48</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167681.13</v>
+        <v>167811.19</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>166915.87</v>
+        <v>167045.34</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119771.44</v>
+        <v>119864.35</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118339.92</v>
+        <v>118431.71</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119055.68</v>
+        <v>119148.03</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82045.33</v>
+        <v>82108.97</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81735.44</v>
+        <v>81798.84</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81890.39</v>
+        <v>81953.91</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54662.54</v>
+        <v>54704.94</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>54964.15</v>
+        <v>55006.78</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54813.34</v>
+        <v>54855.86</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>32991.63</v>
+        <v>33017.22</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32605.47</v>
+        <v>32630.77</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32798.55</v>
+        <v>32823.99</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5533</v>
+        <v>13.5046</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17127.85</v>
+        <v>17141.14</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17806.89</v>
+        <v>17820.7</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17467.37</v>
+        <v>17480.92</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128367.3</v>
+        <v>128474.58</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128461.36</v>
+        <v>128568.71</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128414.33</v>
+        <v>128521.65</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>88901.08</v>
+        <v>88975.38</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87521.59</v>
+        <v>87594.73</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88211.34</v>
+        <v>88285.06</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55879.32</v>
+        <v>55926.02</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56164.5</v>
+        <v>56211.43</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56021.91</v>
+        <v>56068.73</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29582.55</v>
+        <v>29607.28</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29781.68</v>
+        <v>29806.56</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29682.11</v>
+        <v>29706.92</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6785</v>
+        <v>6790.67</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6783.71</v>
+        <v>6789.38</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6784.35</v>
+        <v>6790.02</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.5859</v>
+        <v>13.5337</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3770.05</v>
+        <v>3773.2</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3681.12</v>
+        <v>3684.2</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3725.59</v>
+        <v>3728.7</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108347.23</v>
+        <v>108444.5</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108822.55</v>
+        <v>108920.25</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108584.89</v>
+        <v>108682.38</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>75982.47</v>
+        <v>76050.69</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75441.89</v>
+        <v>75509.62</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75712.17999999999</v>
+        <v>75780.14999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>45977.09</v>
+        <v>46018.37</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47076.34</v>
+        <v>47118.61</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46526.72</v>
+        <v>46568.49</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28563.68</v>
+        <v>28589.32</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28457.23</v>
+        <v>28482.78</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28510.45</v>
+        <v>28536.05</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14012.08</v>
+        <v>14024.66</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14133.56</v>
+        <v>14146.25</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14072.82</v>
+        <v>14085.46</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.6169</v>
+        <v>13.5615</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6496.01</v>
+        <v>6501.84</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6335.53</v>
+        <v>6341.21</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6415.77</v>
+        <v>6421.53</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49296.94</v>
+        <v>49344.65</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>48966.9</v>
+        <v>49014.3</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49131.92</v>
+        <v>49179.48</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43368.14</v>
+        <v>43410.12</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43560.68</v>
+        <v>43602.84</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43464.41</v>
+        <v>43506.48</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31738.96</v>
+        <v>31769.68</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32076.96</v>
+        <v>32108.01</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31907.96</v>
+        <v>31938.85</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22316.57</v>
+        <v>22338.17</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22469.83</v>
+        <v>22491.58</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22393.2</v>
+        <v>22414.87</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14343.57</v>
+        <v>14357.45</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14547.68</v>
+        <v>14561.76</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14445.63</v>
+        <v>14459.61</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.6494</v>
+        <v>13.5906</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8243.26</v>
+        <v>8251.24</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8297.870000000001</v>
+        <v>8305.91</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8270.57</v>
+        <v>8278.57</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48481.29</v>
+        <v>48532.04</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47767.77</v>
+        <v>47817.78</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48124.53</v>
+        <v>48174.91</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43415.68</v>
+        <v>43461.13</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43082.16</v>
+        <v>43127.26</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43248.92</v>
+        <v>43294.19</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31354.82</v>
+        <v>31387.64</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30791.16</v>
+        <v>30823.4</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31072.99</v>
+        <v>31105.52</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23369.74</v>
+        <v>23394.21</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23265.55</v>
+        <v>23289.9</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23317.64</v>
+        <v>23342.05</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18333.26</v>
+        <v>18352.45</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18149.02</v>
+        <v>18168.02</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18241.14</v>
+        <v>18260.24</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.6834</v>
+        <v>13.6211</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15419.53</v>
+        <v>15435.67</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15364.47</v>
+        <v>15380.56</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15392</v>
+        <v>15408.11</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>122996.72</v>
+        <v>123058.7</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123619.6</v>
+        <v>123681.9</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123308.16</v>
+        <v>123370.3</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88201.81</v>
+        <v>88246.25</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88558.36</v>
+        <v>88602.99000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88380.09</v>
+        <v>88424.62</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57617.19</v>
+        <v>57646.23</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57127.86</v>
+        <v>57156.64</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57372.53</v>
+        <v>57401.44</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33125.97</v>
+        <v>33142.66</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32887.28</v>
+        <v>32903.85</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33006.62</v>
+        <v>33023.25</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18825.15</v>
+        <v>18834.64</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18750.76</v>
+        <v>18760.21</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18787.96</v>
+        <v>18797.42</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.7025</v>
+        <v>13.7263</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7632.41</v>
+        <v>7636.26</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7390.9</v>
+        <v>7394.62</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7511.66</v>
+        <v>7515.44</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>400218.85</v>
+        <v>400413.98</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>395267.15</v>
+        <v>395459.87</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>397743</v>
+        <v>397936.93</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300456.1</v>
+        <v>300602.59</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301430.54</v>
+        <v>301577.51</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>300943.32</v>
+        <v>301090.05</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210230.06</v>
+        <v>210332.56</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210103.23</v>
+        <v>210205.67</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210166.64</v>
+        <v>210269.11</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127807.64</v>
+        <v>127869.95</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128089.34</v>
+        <v>128151.79</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>127948.49</v>
+        <v>128010.87</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>61950.01</v>
+        <v>61980.22</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61660.6</v>
+        <v>61690.67</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61805.31</v>
+        <v>61835.44</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6572</v>
+        <v>13.6775</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31638.89</v>
+        <v>31654.32</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31662.79</v>
+        <v>31678.23</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31650.84</v>
+        <v>31666.27</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>403736.39</v>
+        <v>403942.7</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>404279.06</v>
+        <v>404485.64</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>404007.73</v>
+        <v>404214.17</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299689.23</v>
+        <v>299842.36</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>297818</v>
+        <v>297970.18</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>298753.61</v>
+        <v>298906.27</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203279.47</v>
+        <v>203383.35</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203349.01</v>
+        <v>203452.92</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203314.24</v>
+        <v>203418.13</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123011.47</v>
+        <v>123074.33</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123524.36</v>
+        <v>123587.48</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123267.92</v>
+        <v>123330.9</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49125.3</v>
+        <v>49150.4</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49066.76</v>
+        <v>49091.83</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49096.03</v>
+        <v>49121.12</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5643</v>
+        <v>13.561</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5403.62</v>
+        <v>5406.38</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5439.26</v>
+        <v>5442.04</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5421.44</v>
+        <v>5424.21</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168609.37</v>
+        <v>168702.02</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168636.34</v>
+        <v>168729.01</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168622.85</v>
+        <v>168715.52</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110804.35</v>
+        <v>110865.24</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110418.89</v>
+        <v>110479.57</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110611.62</v>
+        <v>110672.41</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62055.33</v>
+        <v>62089.43</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62407.31</v>
+        <v>62441.6</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62231.32</v>
+        <v>62265.52</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26566.49</v>
+        <v>26581.09</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26764.41</v>
+        <v>26779.12</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26665.45</v>
+        <v>26680.1</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6253.47</v>
+        <v>6256.91</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6403.79</v>
+        <v>6407.31</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6328.63</v>
+        <v>6332.11</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5297</v>
+        <v>13.5115</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3703.63</v>
+        <v>3705.67</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3697.21</v>
+        <v>3699.24</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3700.42</v>
+        <v>3702.45</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188574.05</v>
+        <v>188686.63</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189494.83</v>
+        <v>189607.96</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189034.44</v>
+        <v>189147.3</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136720.17</v>
+        <v>136801.8</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137674.25</v>
+        <v>137756.45</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137197.21</v>
+        <v>137279.12</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86420.85000000001</v>
+        <v>86472.44</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87120.22</v>
+        <v>87172.23</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86770.53</v>
+        <v>86822.34</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41279.99</v>
+        <v>41304.63</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41213.79</v>
+        <v>41238.39</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41246.89</v>
+        <v>41271.51</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12872.49</v>
+        <v>12880.18</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12730.71</v>
+        <v>12738.31</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12801.6</v>
+        <v>12809.24</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.5181</v>
+        <v>13.4899</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4467.56</v>
+        <v>4470.23</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4358.5</v>
+        <v>4361.1</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4413.03</v>
+        <v>4415.67</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-27
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148697.99</v>
+        <v>148774.8</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150572.64</v>
+        <v>150650.43</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149635.31</v>
+        <v>149712.62</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113818.64</v>
+        <v>113877.44</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114592.49</v>
+        <v>114651.69</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114205.57</v>
+        <v>114264.56</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81155.35000000001</v>
+        <v>81197.28</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81661.05</v>
+        <v>81703.24000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81408.2</v>
+        <v>81450.25999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57506.66</v>
+        <v>57536.37</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57070.83</v>
+        <v>57100.31</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57288.74</v>
+        <v>57318.34</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37147.02</v>
+        <v>37166.21</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37450.9</v>
+        <v>37470.24</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37298.96</v>
+        <v>37318.23</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4693</v>
+        <v>13.4656</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16895.16</v>
+        <v>16903.89</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16784.21</v>
+        <v>16792.88</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16839.69</v>
+        <v>16848.39</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161534.32</v>
+        <v>161617.69</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160667.55</v>
+        <v>160750.47</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161100.93</v>
+        <v>161184.08</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121312.76</v>
+        <v>121375.37</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119599.4</v>
+        <v>119661.12</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120456.08</v>
+        <v>120518.25</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86670.42999999999</v>
+        <v>86715.16</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85597.19</v>
+        <v>85641.37</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86133.81</v>
+        <v>86178.25999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66021.14</v>
+        <v>66055.22</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65557.03</v>
+        <v>65590.86</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65789.08</v>
+        <v>65823.03999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51576.79</v>
+        <v>51603.41</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49723.17</v>
+        <v>49748.83</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50649.98</v>
+        <v>50676.12</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.4755</v>
+        <v>13.4725</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39098</v>
+        <v>39118.18</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40064.13</v>
+        <v>40084.81</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39581.07</v>
+        <v>39601.49</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166279.48</v>
+        <v>166363</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167811.19</v>
+        <v>167895.48</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167045.34</v>
+        <v>167129.24</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119864.35</v>
+        <v>119924.55</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118431.71</v>
+        <v>118491.19</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119148.03</v>
+        <v>119207.87</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82108.97</v>
+        <v>82150.21000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81798.84</v>
+        <v>81839.92999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81953.91</v>
+        <v>81995.07000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54704.94</v>
+        <v>54732.41</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55006.78</v>
+        <v>55034.41</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54855.86</v>
+        <v>54883.41</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33017.22</v>
+        <v>33033.8</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32630.77</v>
+        <v>32647.15</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32823.99</v>
+        <v>32840.48</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5046</v>
+        <v>13.5047</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17141.14</v>
+        <v>17149.75</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17820.7</v>
+        <v>17829.65</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17480.92</v>
+        <v>17489.7</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128474.58</v>
+        <v>128536.71</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128568.71</v>
+        <v>128630.9</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128521.65</v>
+        <v>128583.81</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>88975.38</v>
+        <v>89018.41</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87594.73</v>
+        <v>87637.10000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88285.06</v>
+        <v>88327.75</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55926.02</v>
+        <v>55953.07</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56211.43</v>
+        <v>56238.62</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56068.73</v>
+        <v>56095.84</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29607.28</v>
+        <v>29621.6</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29806.56</v>
+        <v>29820.98</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29706.92</v>
+        <v>29721.29</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6790.67</v>
+        <v>6793.96</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6789.38</v>
+        <v>6792.66</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6790.02</v>
+        <v>6793.31</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.5337</v>
+        <v>13.5369</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3773.2</v>
+        <v>3775.02</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3684.2</v>
+        <v>3685.98</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3728.7</v>
+        <v>3730.5</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108444.5</v>
+        <v>108494.54</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108920.25</v>
+        <v>108970.51</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108682.38</v>
+        <v>108732.53</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76050.69</v>
+        <v>76085.78</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75509.62</v>
+        <v>75544.46000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75780.14999999999</v>
+        <v>75815.12</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46018.37</v>
+        <v>46039.6</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47118.61</v>
+        <v>47140.35</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46568.49</v>
+        <v>46589.97</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28589.32</v>
+        <v>28602.51</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28482.78</v>
+        <v>28495.92</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28536.05</v>
+        <v>28549.22</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14024.66</v>
+        <v>14031.13</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14146.25</v>
+        <v>14152.78</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14085.46</v>
+        <v>14091.96</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.5615</v>
+        <v>13.5677</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6501.84</v>
+        <v>6504.84</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6341.21</v>
+        <v>6344.14</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6421.53</v>
+        <v>6424.49</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49344.65</v>
+        <v>49366.04</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49014.3</v>
+        <v>49035.55</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49179.48</v>
+        <v>49200.8</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43410.12</v>
+        <v>43428.94</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43602.84</v>
+        <v>43621.74</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43506.48</v>
+        <v>43525.34</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31769.68</v>
+        <v>31783.45</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32108.01</v>
+        <v>32121.93</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31938.85</v>
+        <v>31952.69</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22338.17</v>
+        <v>22347.85</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22491.58</v>
+        <v>22501.33</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22414.87</v>
+        <v>22424.59</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14357.45</v>
+        <v>14363.68</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14561.76</v>
+        <v>14568.08</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14459.61</v>
+        <v>14465.88</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.5906</v>
+        <v>13.5999</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8251.24</v>
+        <v>8254.82</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8305.91</v>
+        <v>8309.51</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8278.57</v>
+        <v>8282.16</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48532.04</v>
+        <v>48551.41</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47817.78</v>
+        <v>47836.86</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48174.91</v>
+        <v>48194.14</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43461.13</v>
+        <v>43478.48</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43127.26</v>
+        <v>43144.48</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43294.19</v>
+        <v>43311.48</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31387.64</v>
+        <v>31400.17</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30823.4</v>
+        <v>30835.7</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31105.52</v>
+        <v>31117.94</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23394.21</v>
+        <v>23403.54</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23289.9</v>
+        <v>23299.2</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23342.05</v>
+        <v>23351.37</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18352.45</v>
+        <v>18359.78</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18168.02</v>
+        <v>18175.28</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18260.24</v>
+        <v>18267.53</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.6211</v>
+        <v>13.6336</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15435.67</v>
+        <v>15441.83</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15380.56</v>
+        <v>15386.7</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15408.11</v>
+        <v>15414.26</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123058.7</v>
+        <v>123122.07</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123681.9</v>
+        <v>123745.58</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123370.3</v>
+        <v>123433.82</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88246.25</v>
+        <v>88291.69</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88602.99000000001</v>
+        <v>88648.61</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88424.62</v>
+        <v>88470.14999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57646.23</v>
+        <v>57675.91</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57156.64</v>
+        <v>57186.07</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57401.44</v>
+        <v>57430.99</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33142.66</v>
+        <v>33159.72</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32903.85</v>
+        <v>32920.79</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33023.25</v>
+        <v>33040.26</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18834.64</v>
+        <v>18844.34</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18760.21</v>
+        <v>18769.87</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18797.42</v>
+        <v>18807.1</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.7263</v>
+        <v>13.7055</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7636.26</v>
+        <v>7640.19</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7394.62</v>
+        <v>7398.43</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7515.44</v>
+        <v>7519.31</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>400413.98</v>
+        <v>400622.9</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>395459.87</v>
+        <v>395666.21</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>397936.93</v>
+        <v>398144.55</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300602.59</v>
+        <v>300759.43</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301577.51</v>
+        <v>301734.86</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301090.05</v>
+        <v>301247.15</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210332.56</v>
+        <v>210442.3</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210205.67</v>
+        <v>210315.35</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210269.11</v>
+        <v>210378.82</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127869.95</v>
+        <v>127936.67</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128151.79</v>
+        <v>128218.66</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128010.87</v>
+        <v>128077.66</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>61980.22</v>
+        <v>62012.56</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61690.67</v>
+        <v>61722.86</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61835.44</v>
+        <v>61867.71</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6775</v>
+        <v>13.6643</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31654.32</v>
+        <v>31670.84</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31678.23</v>
+        <v>31694.76</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31666.27</v>
+        <v>31682.8</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>403942.7</v>
+        <v>404154.56</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>404485.64</v>
+        <v>404697.8</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>404214.17</v>
+        <v>404426.18</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299842.36</v>
+        <v>299999.63</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>297970.18</v>
+        <v>298126.47</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>298906.27</v>
+        <v>299063.05</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203383.35</v>
+        <v>203490.02</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203452.92</v>
+        <v>203559.63</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203418.13</v>
+        <v>203524.83</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123074.33</v>
+        <v>123138.88</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123587.48</v>
+        <v>123652.3</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123330.9</v>
+        <v>123395.59</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49150.4</v>
+        <v>49176.18</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49091.83</v>
+        <v>49117.58</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49121.12</v>
+        <v>49146.88</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.561</v>
+        <v>13.5499</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5406.38</v>
+        <v>5409.22</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5442.04</v>
+        <v>5444.89</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5424.21</v>
+        <v>5427.06</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168702.02</v>
+        <v>168791.34</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168729.01</v>
+        <v>168818.34</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168715.52</v>
+        <v>168804.84</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110865.24</v>
+        <v>110923.94</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110479.57</v>
+        <v>110538.06</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110672.41</v>
+        <v>110731</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62089.43</v>
+        <v>62122.3</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62441.6</v>
+        <v>62474.66</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62265.52</v>
+        <v>62298.48</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26581.09</v>
+        <v>26595.16</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26779.12</v>
+        <v>26793.29</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26680.1</v>
+        <v>26694.23</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6256.91</v>
+        <v>6260.22</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6407.31</v>
+        <v>6410.71</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6332.11</v>
+        <v>6335.46</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5115</v>
+        <v>13.5008</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3705.67</v>
+        <v>3707.63</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3699.24</v>
+        <v>3701.2</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3702.45</v>
+        <v>3704.41</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188686.63</v>
+        <v>188785.81</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189607.96</v>
+        <v>189707.62</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189147.3</v>
+        <v>189246.71</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136801.8</v>
+        <v>136873.7</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137756.45</v>
+        <v>137828.85</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137279.12</v>
+        <v>137351.28</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86472.44</v>
+        <v>86517.89</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87172.23</v>
+        <v>87218.05</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86822.34</v>
+        <v>86867.97</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41304.63</v>
+        <v>41326.34</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41238.39</v>
+        <v>41260.07</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41271.51</v>
+        <v>41293.21</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12880.18</v>
+        <v>12886.95</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12738.31</v>
+        <v>12745</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12809.24</v>
+        <v>12815.98</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4899</v>
+        <v>13.4828</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4470.23</v>
+        <v>4472.58</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4361.1</v>
+        <v>4363.4</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4415.67</v>
+        <v>4417.99</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-28
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148774.8</v>
+        <v>148869.54</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150650.43</v>
+        <v>150746.36</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149712.62</v>
+        <v>149807.95</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113877.44</v>
+        <v>113949.95</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114651.69</v>
+        <v>114724.7</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114264.56</v>
+        <v>114337.33</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81197.28</v>
+        <v>81248.98</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81703.24000000001</v>
+        <v>81755.25999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81450.25999999999</v>
+        <v>81502.12</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57536.37</v>
+        <v>57573.01</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57100.31</v>
+        <v>57136.67</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57318.34</v>
+        <v>57354.84</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37166.21</v>
+        <v>37189.88</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37470.24</v>
+        <v>37494.1</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37318.23</v>
+        <v>37341.99</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4656</v>
+        <v>13.432</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16903.89</v>
+        <v>16914.65</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16792.88</v>
+        <v>16803.58</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16848.39</v>
+        <v>16859.11</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161617.69</v>
+        <v>161728.73</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160750.47</v>
+        <v>160860.92</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161184.08</v>
+        <v>161294.83</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121375.37</v>
+        <v>121458.77</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119661.12</v>
+        <v>119743.34</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120518.25</v>
+        <v>120601.05</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86715.16</v>
+        <v>86774.74000000001</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85641.37</v>
+        <v>85700.21000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86178.25999999999</v>
+        <v>86237.48</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66055.22</v>
+        <v>66100.60000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65590.86</v>
+        <v>65635.92999999999</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65823.03999999999</v>
+        <v>65868.25999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51603.41</v>
+        <v>51638.86</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49748.83</v>
+        <v>49783.01</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50676.12</v>
+        <v>50710.94</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.4725</v>
+        <v>13.4332</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39118.18</v>
+        <v>39145.06</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40084.81</v>
+        <v>40112.35</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39601.49</v>
+        <v>39628.7</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166363</v>
+        <v>166486.48</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>167895.48</v>
+        <v>168020.1</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167129.24</v>
+        <v>167253.29</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>119924.55</v>
+        <v>120013.57</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118491.19</v>
+        <v>118579.15</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119207.87</v>
+        <v>119296.36</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82150.21000000001</v>
+        <v>82211.19</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81839.92999999999</v>
+        <v>81900.67</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>81995.07000000001</v>
+        <v>82055.92999999999</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54732.41</v>
+        <v>54773.04</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55034.41</v>
+        <v>55075.26</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54883.41</v>
+        <v>54924.15</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33033.8</v>
+        <v>33058.32</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32647.15</v>
+        <v>32671.39</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32840.48</v>
+        <v>32864.85</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.5047</v>
+        <v>13.4611</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17149.75</v>
+        <v>17162.48</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17829.65</v>
+        <v>17842.88</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17489.7</v>
+        <v>17502.68</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128536.71</v>
+        <v>128640.07</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128630.9</v>
+        <v>128734.33</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128583.81</v>
+        <v>128687.2</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89018.41</v>
+        <v>89089.99000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87637.10000000001</v>
+        <v>87707.57000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88327.75</v>
+        <v>88398.78</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55953.07</v>
+        <v>55998.06</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56238.62</v>
+        <v>56283.84</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56095.84</v>
+        <v>56140.95</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29621.6</v>
+        <v>29645.41</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29820.98</v>
+        <v>29844.96</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29721.29</v>
+        <v>29745.19</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6793.96</v>
+        <v>6799.42</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6792.66</v>
+        <v>6798.12</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6793.31</v>
+        <v>6798.77</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.5369</v>
+        <v>13.489</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3775.02</v>
+        <v>3778.06</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3685.98</v>
+        <v>3688.95</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3730.5</v>
+        <v>3733.5</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108494.54</v>
+        <v>108588.86</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>108970.51</v>
+        <v>109065.25</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108732.53</v>
+        <v>108827.05</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76085.78</v>
+        <v>76151.92</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75544.46000000001</v>
+        <v>75610.14</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75815.12</v>
+        <v>75881.03</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46039.6</v>
+        <v>46079.63</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47140.35</v>
+        <v>47181.33</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46589.97</v>
+        <v>46630.48</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28602.51</v>
+        <v>28627.38</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28495.92</v>
+        <v>28520.69</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28549.22</v>
+        <v>28574.04</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14031.13</v>
+        <v>14043.33</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14152.78</v>
+        <v>14165.09</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14091.96</v>
+        <v>14104.21</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.5677</v>
+        <v>13.5156</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6504.84</v>
+        <v>6510.5</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6344.14</v>
+        <v>6349.66</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6424.49</v>
+        <v>6430.08</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49366.04</v>
+        <v>49412.66</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49035.55</v>
+        <v>49081.85</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49200.8</v>
+        <v>49247.25</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43428.94</v>
+        <v>43469.94</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43621.74</v>
+        <v>43662.93</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43525.34</v>
+        <v>43566.44</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31783.45</v>
+        <v>31813.46</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32121.93</v>
+        <v>32152.26</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31952.69</v>
+        <v>31982.86</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22347.85</v>
+        <v>22368.95</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22501.33</v>
+        <v>22522.58</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22424.59</v>
+        <v>22445.76</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14363.68</v>
+        <v>14377.24</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14568.08</v>
+        <v>14581.83</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14465.88</v>
+        <v>14479.54</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.5999</v>
+        <v>13.5435</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8254.82</v>
+        <v>8262.610000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8309.51</v>
+        <v>8317.35</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8282.16</v>
+        <v>8289.98</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48551.41</v>
+        <v>48601.4</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47836.86</v>
+        <v>47886.12</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48194.14</v>
+        <v>48243.76</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43478.48</v>
+        <v>43523.24</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43144.48</v>
+        <v>43188.9</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43311.48</v>
+        <v>43356.07</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31400.17</v>
+        <v>31432.5</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30835.7</v>
+        <v>30867.45</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31117.94</v>
+        <v>31149.98</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23403.54</v>
+        <v>23427.64</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23299.2</v>
+        <v>23323.19</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23351.37</v>
+        <v>23375.41</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18359.78</v>
+        <v>18378.68</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18175.28</v>
+        <v>18193.99</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18267.53</v>
+        <v>18286.34</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.6336</v>
+        <v>13.5726</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15441.83</v>
+        <v>15457.73</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15386.7</v>
+        <v>15402.54</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15414.26</v>
+        <v>15430.13</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123122.07</v>
+        <v>123185.75</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123745.58</v>
+        <v>123809.58</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123433.82</v>
+        <v>123497.67</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88291.69</v>
+        <v>88337.36</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88648.61</v>
+        <v>88694.46000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88470.14999999999</v>
+        <v>88515.91</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57675.91</v>
+        <v>57705.74</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57186.07</v>
+        <v>57215.65</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57430.99</v>
+        <v>57460.7</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33159.72</v>
+        <v>33176.87</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32920.79</v>
+        <v>32937.82</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33040.26</v>
+        <v>33057.35</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18844.34</v>
+        <v>18854.08</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18769.87</v>
+        <v>18779.58</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18807.1</v>
+        <v>18816.83</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.7055</v>
+        <v>13.6631</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7640.19</v>
+        <v>7644.14</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7398.43</v>
+        <v>7402.26</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7519.31</v>
+        <v>7523.2</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>400622.9</v>
+        <v>400839.12</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>395666.21</v>
+        <v>395879.75</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>398144.55</v>
+        <v>398359.43</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300759.43</v>
+        <v>300921.75</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301734.86</v>
+        <v>301897.71</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301247.15</v>
+        <v>301409.73</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210442.3</v>
+        <v>210555.88</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210315.35</v>
+        <v>210428.85</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210378.82</v>
+        <v>210492.37</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>127936.67</v>
+        <v>128005.72</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128218.66</v>
+        <v>128287.86</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128077.66</v>
+        <v>128146.79</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62012.56</v>
+        <v>62046.03</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61722.86</v>
+        <v>61756.17</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61867.71</v>
+        <v>61901.1</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6643</v>
+        <v>13.6311</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31670.84</v>
+        <v>31687.93</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31694.76</v>
+        <v>31711.86</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31682.8</v>
+        <v>31699.9</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>404154.56</v>
+        <v>404376.61</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>404697.8</v>
+        <v>404920.14</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>404426.18</v>
+        <v>404648.37</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>299999.63</v>
+        <v>300164.45</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298126.47</v>
+        <v>298290.26</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299063.05</v>
+        <v>299227.35</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203490.02</v>
+        <v>203601.82</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203559.63</v>
+        <v>203671.47</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203524.83</v>
+        <v>203636.64</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123138.88</v>
+        <v>123206.53</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123652.3</v>
+        <v>123720.24</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123395.59</v>
+        <v>123463.39</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49176.18</v>
+        <v>49203.2</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49117.58</v>
+        <v>49144.57</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49146.88</v>
+        <v>49173.88</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5499</v>
+        <v>13.5242</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5409.22</v>
+        <v>5412.19</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5444.89</v>
+        <v>5447.88</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5427.06</v>
+        <v>5430.04</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168791.34</v>
+        <v>168887.4</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168818.34</v>
+        <v>168914.41</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168804.84</v>
+        <v>168900.91</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110923.94</v>
+        <v>110987.07</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110538.06</v>
+        <v>110600.97</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110731</v>
+        <v>110794.02</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62122.3</v>
+        <v>62157.66</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62474.66</v>
+        <v>62510.22</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62298.48</v>
+        <v>62333.94</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26595.16</v>
+        <v>26610.29</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26793.29</v>
+        <v>26808.54</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26694.23</v>
+        <v>26709.42</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6260.22</v>
+        <v>6263.78</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6410.71</v>
+        <v>6414.35</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6335.46</v>
+        <v>6339.07</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.5008</v>
+        <v>13.4737</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3707.63</v>
+        <v>3709.74</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3701.2</v>
+        <v>3703.3</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3704.41</v>
+        <v>3706.52</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188785.81</v>
+        <v>188899.29</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189707.62</v>
+        <v>189821.66</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189246.71</v>
+        <v>189360.48</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136873.7</v>
+        <v>136955.98</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137828.85</v>
+        <v>137911.71</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137351.28</v>
+        <v>137433.84</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86517.89</v>
+        <v>86569.89999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87218.05</v>
+        <v>87270.48</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86867.97</v>
+        <v>86920.19</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41326.34</v>
+        <v>41351.19</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41260.07</v>
+        <v>41284.87</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41293.21</v>
+        <v>41318.03</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12886.95</v>
+        <v>12894.69</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12745</v>
+        <v>12752.66</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12815.98</v>
+        <v>12823.68</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4828</v>
+        <v>13.4524</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4472.58</v>
+        <v>4475.27</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4363.4</v>
+        <v>4366.02</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4417.99</v>
+        <v>4420.64</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-08-29
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148869.54</v>
+        <v>148892.04</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150746.36</v>
+        <v>150769.14</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149807.95</v>
+        <v>149830.59</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113949.95</v>
+        <v>113967.17</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114724.7</v>
+        <v>114742.04</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114337.33</v>
+        <v>114354.6</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81248.98</v>
+        <v>81261.25999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81755.25999999999</v>
+        <v>81767.62</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81502.12</v>
+        <v>81514.44</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57573.01</v>
+        <v>57581.71</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57136.67</v>
+        <v>57145.31</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57354.84</v>
+        <v>57363.51</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37189.88</v>
+        <v>37195.5</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37494.1</v>
+        <v>37499.77</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37341.99</v>
+        <v>37347.63</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.432</v>
+        <v>13.3944</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16914.65</v>
+        <v>16917.21</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16803.58</v>
+        <v>16806.12</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16859.11</v>
+        <v>16861.66</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161728.73</v>
+        <v>161758.34</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160860.92</v>
+        <v>160890.37</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161294.83</v>
+        <v>161324.35</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121458.77</v>
+        <v>121481</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119743.34</v>
+        <v>119765.26</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120601.05</v>
+        <v>120623.13</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86774.74000000001</v>
+        <v>86790.63</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85700.21000000001</v>
+        <v>85715.89999999999</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86237.48</v>
+        <v>86253.25999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66100.60000000001</v>
+        <v>66112.7</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65635.92999999999</v>
+        <v>65647.94</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65868.25999999999</v>
+        <v>65880.32000000001</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51638.86</v>
+        <v>51648.32</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49783.01</v>
+        <v>49792.12</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50710.94</v>
+        <v>50720.22</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.4332</v>
+        <v>13.3945</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39145.06</v>
+        <v>39152.22</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40112.35</v>
+        <v>40119.69</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39628.7</v>
+        <v>39635.96</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166486.48</v>
+        <v>166517.33</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168020.1</v>
+        <v>168051.24</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167253.29</v>
+        <v>167284.28</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120013.57</v>
+        <v>120035.8</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118579.15</v>
+        <v>118601.12</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119296.36</v>
+        <v>119318.46</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82211.19</v>
+        <v>82226.42</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81900.67</v>
+        <v>81915.85000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82055.92999999999</v>
+        <v>82071.14</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54773.04</v>
+        <v>54783.19</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55075.26</v>
+        <v>55085.46</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54924.15</v>
+        <v>54934.33</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33058.32</v>
+        <v>33064.45</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32671.39</v>
+        <v>32677.44</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32864.85</v>
+        <v>32870.94</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.4611</v>
+        <v>13.4274</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17162.48</v>
+        <v>17165.66</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17842.88</v>
+        <v>17846.19</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17502.68</v>
+        <v>17505.92</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128640.07</v>
+        <v>128663.21</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128734.33</v>
+        <v>128757.48</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128687.2</v>
+        <v>128710.34</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89089.99000000001</v>
+        <v>89106.00999999999</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87707.57000000001</v>
+        <v>87723.34</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88398.78</v>
+        <v>88414.67999999999</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>55998.06</v>
+        <v>56008.13</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56283.84</v>
+        <v>56293.96</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56140.95</v>
+        <v>56151.05</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29645.41</v>
+        <v>29650.75</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29844.96</v>
+        <v>29850.33</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29745.19</v>
+        <v>29750.54</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6799.42</v>
+        <v>6800.64</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6798.12</v>
+        <v>6799.34</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6798.77</v>
+        <v>6799.99</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.489</v>
+        <v>13.4602</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3778.06</v>
+        <v>3778.74</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3688.95</v>
+        <v>3689.61</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3733.5</v>
+        <v>3734.17</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108588.86</v>
+        <v>108607.04</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109065.25</v>
+        <v>109083.51</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108827.05</v>
+        <v>108845.28</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76151.92</v>
+        <v>76164.67999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75610.14</v>
+        <v>75622.8</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75881.03</v>
+        <v>75893.74000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46079.63</v>
+        <v>46087.34</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47181.33</v>
+        <v>47189.23</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46630.48</v>
+        <v>46638.29</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28627.38</v>
+        <v>28632.17</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28520.69</v>
+        <v>28525.47</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28574.04</v>
+        <v>28578.82</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14043.33</v>
+        <v>14045.68</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14165.09</v>
+        <v>14167.46</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14104.21</v>
+        <v>14106.57</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.5156</v>
+        <v>13.4916</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6510.5</v>
+        <v>6511.59</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6349.66</v>
+        <v>6350.72</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6430.08</v>
+        <v>6431.15</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49412.66</v>
+        <v>49419.92</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49081.85</v>
+        <v>49089.06</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49247.25</v>
+        <v>49254.49</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43469.94</v>
+        <v>43476.33</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43662.93</v>
+        <v>43669.34</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43566.44</v>
+        <v>43572.84</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31813.46</v>
+        <v>31818.13</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32152.26</v>
+        <v>32156.99</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31982.86</v>
+        <v>31987.56</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22368.95</v>
+        <v>22372.24</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22522.58</v>
+        <v>22525.88</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22445.76</v>
+        <v>22449.06</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14377.24</v>
+        <v>14379.35</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14581.83</v>
+        <v>14583.97</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14479.54</v>
+        <v>14481.66</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.5435</v>
+        <v>13.5245</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8262.610000000001</v>
+        <v>8263.82</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8317.35</v>
+        <v>8318.57</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8289.98</v>
+        <v>8291.200000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48601.4</v>
+        <v>48607.1</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47886.12</v>
+        <v>47891.73</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48243.76</v>
+        <v>48249.42</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43523.24</v>
+        <v>43528.34</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43188.9</v>
+        <v>43193.96</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43356.07</v>
+        <v>43361.15</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31432.5</v>
+        <v>31436.19</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30867.45</v>
+        <v>30871.07</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31149.98</v>
+        <v>31153.63</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23427.64</v>
+        <v>23430.39</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23323.19</v>
+        <v>23325.92</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23375.41</v>
+        <v>23378.15</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18378.68</v>
+        <v>18380.84</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18193.99</v>
+        <v>18196.12</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18286.34</v>
+        <v>18288.48</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5726</v>
+        <v>13.5589</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15457.73</v>
+        <v>15459.54</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15402.54</v>
+        <v>15404.34</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15430.13</v>
+        <v>15431.94</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123185.75</v>
+        <v>123185.39</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123809.58</v>
+        <v>123809.22</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123497.67</v>
+        <v>123497.31</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88337.36</v>
+        <v>88337.10000000001</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88694.46000000001</v>
+        <v>88694.2</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88515.91</v>
+        <v>88515.64999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57705.74</v>
+        <v>57705.57</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57215.65</v>
+        <v>57215.48</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57460.7</v>
+        <v>57460.53</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33176.87</v>
+        <v>33176.78</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32937.82</v>
+        <v>32937.72</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33057.35</v>
+        <v>33057.25</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18854.08</v>
+        <v>18854.03</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18779.58</v>
+        <v>18779.52</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18816.83</v>
+        <v>18816.78</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6631</v>
+        <v>13.6798</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7644.14</v>
+        <v>7644.12</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7402.26</v>
+        <v>7402.23</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7523.2</v>
+        <v>7523.18</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>400839.12</v>
+        <v>400835.28</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>395879.75</v>
+        <v>395875.96</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>398359.43</v>
+        <v>398355.62</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300921.75</v>
+        <v>300918.87</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301897.71</v>
+        <v>301894.82</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301409.73</v>
+        <v>301406.84</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210555.88</v>
+        <v>210553.86</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210428.85</v>
+        <v>210426.84</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210492.37</v>
+        <v>210490.35</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128005.72</v>
+        <v>128004.49</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128287.86</v>
+        <v>128286.63</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128146.79</v>
+        <v>128145.56</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62046.03</v>
+        <v>62045.43</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61756.17</v>
+        <v>61755.58</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61901.1</v>
+        <v>61900.5</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6311</v>
+        <v>13.6413</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31687.93</v>
+        <v>31687.63</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31711.86</v>
+        <v>31711.56</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31699.9</v>
+        <v>31699.59</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>404376.61</v>
+        <v>404385.3</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>404920.14</v>
+        <v>404928.84</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>404648.37</v>
+        <v>404657.07</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300164.45</v>
+        <v>300170.9</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298290.26</v>
+        <v>298296.67</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299227.35</v>
+        <v>299233.79</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203601.82</v>
+        <v>203606.19</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203671.47</v>
+        <v>203675.85</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203636.64</v>
+        <v>203641.02</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123206.53</v>
+        <v>123209.18</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123720.24</v>
+        <v>123722.9</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123463.39</v>
+        <v>123466.04</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49203.2</v>
+        <v>49204.26</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49144.57</v>
+        <v>49145.62</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49173.88</v>
+        <v>49174.94</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5242</v>
+        <v>13.5119</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5412.19</v>
+        <v>5412.31</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5447.88</v>
+        <v>5448</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5430.04</v>
+        <v>5430.15</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168887.4</v>
+        <v>168897.44</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168914.41</v>
+        <v>168924.45</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168900.91</v>
+        <v>168910.94</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110987.07</v>
+        <v>110993.66</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110600.97</v>
+        <v>110607.54</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110794.02</v>
+        <v>110800.6</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62157.66</v>
+        <v>62161.35</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62510.22</v>
+        <v>62513.93</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62333.94</v>
+        <v>62337.64</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26610.29</v>
+        <v>26611.88</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26808.54</v>
+        <v>26810.13</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26709.42</v>
+        <v>26711</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6263.78</v>
+        <v>6264.15</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6414.35</v>
+        <v>6414.73</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6339.07</v>
+        <v>6339.44</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4737</v>
+        <v>13.4494</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3709.74</v>
+        <v>3709.96</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3703.3</v>
+        <v>3703.52</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3706.52</v>
+        <v>3706.74</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188899.29</v>
+        <v>188918.38</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189821.66</v>
+        <v>189840.84</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189360.48</v>
+        <v>189379.61</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136955.98</v>
+        <v>136969.82</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137911.71</v>
+        <v>137925.64</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137433.84</v>
+        <v>137447.73</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86569.89999999999</v>
+        <v>86578.64999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87270.48</v>
+        <v>87279.3</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86920.19</v>
+        <v>86928.97</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41351.19</v>
+        <v>41355.36</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41284.87</v>
+        <v>41289.04</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41318.03</v>
+        <v>41322.2</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12894.69</v>
+        <v>12896</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12752.66</v>
+        <v>12753.95</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12823.68</v>
+        <v>12824.98</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4524</v>
+        <v>13.4213</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4475.27</v>
+        <v>4475.72</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4366.02</v>
+        <v>4366.46</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4420.64</v>
+        <v>4421.09</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-01
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>148892.04</v>
+        <v>149034.63</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150769.14</v>
+        <v>150913.53</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149830.59</v>
+        <v>149974.08</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>113967.17</v>
+        <v>114076.31</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114742.04</v>
+        <v>114851.92</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114354.6</v>
+        <v>114464.12</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81261.25999999999</v>
+        <v>81339.08</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81767.62</v>
+        <v>81845.92999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81514.44</v>
+        <v>81592.5</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57581.71</v>
+        <v>57636.85</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57145.31</v>
+        <v>57200.03</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57363.51</v>
+        <v>57418.44</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37195.5</v>
+        <v>37231.12</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37499.77</v>
+        <v>37535.68</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37347.63</v>
+        <v>37383.4</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3944</v>
+        <v>13.4047</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16917.21</v>
+        <v>16933.41</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16806.12</v>
+        <v>16822.21</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16861.66</v>
+        <v>16877.81</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161758.34</v>
+        <v>161912.32</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>160890.37</v>
+        <v>161043.53</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161324.35</v>
+        <v>161477.93</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121481</v>
+        <v>121596.65</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119765.26</v>
+        <v>119879.27</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120623.13</v>
+        <v>120737.96</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86790.63</v>
+        <v>86873.25</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85715.89999999999</v>
+        <v>85797.49000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86253.25999999999</v>
+        <v>86335.37</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66112.7</v>
+        <v>66175.64</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65647.94</v>
+        <v>65710.44</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65880.32000000001</v>
+        <v>65943.03999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51648.32</v>
+        <v>51697.48</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49792.12</v>
+        <v>49839.52</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50720.22</v>
+        <v>50768.5</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3945</v>
+        <v>13.4044</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39152.22</v>
+        <v>39189.49</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40119.69</v>
+        <v>40157.88</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39635.96</v>
+        <v>39673.69</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166517.33</v>
+        <v>166671.82</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168051.24</v>
+        <v>168207.15</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167284.28</v>
+        <v>167439.49</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120035.8</v>
+        <v>120147.17</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118601.12</v>
+        <v>118711.15</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119318.46</v>
+        <v>119429.16</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82226.42</v>
+        <v>82302.71000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81915.85000000001</v>
+        <v>81991.85000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82071.14</v>
+        <v>82147.28</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54783.19</v>
+        <v>54834.01</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55085.46</v>
+        <v>55136.57</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54934.33</v>
+        <v>54985.29</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33064.45</v>
+        <v>33095.12</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32677.44</v>
+        <v>32707.76</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32870.94</v>
+        <v>32901.44</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.4274</v>
+        <v>13.4407</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17165.66</v>
+        <v>17181.58</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17846.19</v>
+        <v>17862.75</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17505.92</v>
+        <v>17522.16</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128663.21</v>
+        <v>128778.78</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128757.48</v>
+        <v>128873.14</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128710.34</v>
+        <v>128825.96</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89106.00999999999</v>
+        <v>89186.05</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87723.34</v>
+        <v>87802.14</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88414.67999999999</v>
+        <v>88494.10000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56008.13</v>
+        <v>56058.44</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56293.96</v>
+        <v>56344.53</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56151.05</v>
+        <v>56201.48</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29650.75</v>
+        <v>29677.38</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29850.33</v>
+        <v>29877.14</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29750.54</v>
+        <v>29777.26</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6800.64</v>
+        <v>6806.75</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6799.34</v>
+        <v>6805.45</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6799.99</v>
+        <v>6806.1</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4602</v>
+        <v>13.4771</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3778.74</v>
+        <v>3782.13</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3689.61</v>
+        <v>3692.92</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3734.17</v>
+        <v>3737.53</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108607.04</v>
+        <v>108701</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109083.51</v>
+        <v>109177.88</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108845.28</v>
+        <v>108939.44</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76164.67999999999</v>
+        <v>76230.57000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75622.8</v>
+        <v>75688.22</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75893.74000000001</v>
+        <v>75959.39</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46087.34</v>
+        <v>46127.21</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47189.23</v>
+        <v>47230.05</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46638.29</v>
+        <v>46678.63</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28632.17</v>
+        <v>28656.94</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28525.47</v>
+        <v>28550.14</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28578.82</v>
+        <v>28603.54</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14045.68</v>
+        <v>14057.84</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14167.46</v>
+        <v>14179.71</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14106.57</v>
+        <v>14118.77</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4916</v>
+        <v>13.5118</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6511.59</v>
+        <v>6517.22</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6350.72</v>
+        <v>6356.21</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6431.15</v>
+        <v>6436.72</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49419.92</v>
+        <v>49460.7</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49089.06</v>
+        <v>49129.57</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49254.49</v>
+        <v>49295.13</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43476.33</v>
+        <v>43512.2</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43669.34</v>
+        <v>43705.38</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43572.84</v>
+        <v>43608.79</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31818.13</v>
+        <v>31844.39</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32156.99</v>
+        <v>32183.52</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>31987.56</v>
+        <v>32013.96</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22372.24</v>
+        <v>22390.7</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22525.88</v>
+        <v>22544.47</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22449.06</v>
+        <v>22467.59</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14379.35</v>
+        <v>14391.22</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14583.97</v>
+        <v>14596.01</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14481.66</v>
+        <v>14493.61</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.5245</v>
+        <v>13.5482</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8263.82</v>
+        <v>8270.639999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8318.57</v>
+        <v>8325.440000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8291.200000000001</v>
+        <v>8298.040000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48607.1</v>
+        <v>48644.91</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47891.73</v>
+        <v>47928.98</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48249.42</v>
+        <v>48286.94</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43528.34</v>
+        <v>43562.2</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43193.96</v>
+        <v>43227.56</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43361.15</v>
+        <v>43394.88</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31436.19</v>
+        <v>31460.64</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30871.07</v>
+        <v>30895.08</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31153.63</v>
+        <v>31177.86</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23430.39</v>
+        <v>23448.61</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23325.92</v>
+        <v>23344.06</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23378.15</v>
+        <v>23396.34</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18380.84</v>
+        <v>18395.13</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18196.12</v>
+        <v>18210.27</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18288.48</v>
+        <v>18302.7</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5589</v>
+        <v>13.5862</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15459.54</v>
+        <v>15471.56</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15404.34</v>
+        <v>15416.32</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15431.94</v>
+        <v>15443.94</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123185.39</v>
+        <v>123311.13</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123809.22</v>
+        <v>123935.6</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123497.31</v>
+        <v>123623.37</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88337.10000000001</v>
+        <v>88427.27</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88694.2</v>
+        <v>88784.74000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88515.64999999999</v>
+        <v>88606.00999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57705.57</v>
+        <v>57764.48</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57215.48</v>
+        <v>57273.89</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57460.53</v>
+        <v>57519.18</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33176.78</v>
+        <v>33210.64</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32937.72</v>
+        <v>32971.35</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33057.25</v>
+        <v>33091</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18854.03</v>
+        <v>18873.27</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18779.52</v>
+        <v>18798.69</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18816.78</v>
+        <v>18835.98</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6798</v>
+        <v>13.6544</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7644.12</v>
+        <v>7651.92</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7402.23</v>
+        <v>7409.79</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7523.18</v>
+        <v>7530.86</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>400835.28</v>
+        <v>401246.07</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>395875.96</v>
+        <v>396281.66</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>398355.62</v>
+        <v>398763.86</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>300918.87</v>
+        <v>301227.26</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>301894.82</v>
+        <v>302204.2</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301406.84</v>
+        <v>301715.73</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210553.86</v>
+        <v>210769.64</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210426.84</v>
+        <v>210642.49</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210490.35</v>
+        <v>210706.07</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128004.49</v>
+        <v>128135.67</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128286.63</v>
+        <v>128418.1</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128145.56</v>
+        <v>128276.89</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62045.43</v>
+        <v>62109.02</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61755.58</v>
+        <v>61818.86</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61900.5</v>
+        <v>61963.94</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6413</v>
+        <v>13.6305</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31687.63</v>
+        <v>31720.1</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31711.56</v>
+        <v>31744.06</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31699.59</v>
+        <v>31732.08</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>404385.3</v>
+        <v>404795.88</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>404928.84</v>
+        <v>405339.98</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>404657.07</v>
+        <v>405067.93</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300170.9</v>
+        <v>300475.68</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298296.67</v>
+        <v>298599.54</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299233.79</v>
+        <v>299537.61</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203606.19</v>
+        <v>203812.92</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203675.85</v>
+        <v>203882.64</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203641.02</v>
+        <v>203847.78</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123209.18</v>
+        <v>123334.28</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123722.9</v>
+        <v>123848.52</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123466.04</v>
+        <v>123591.4</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49204.26</v>
+        <v>49254.22</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49145.62</v>
+        <v>49195.52</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49174.94</v>
+        <v>49224.87</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5119</v>
+        <v>13.5065</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5412.31</v>
+        <v>5417.8</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5448</v>
+        <v>5453.53</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5430.15</v>
+        <v>5435.67</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>168897.44</v>
+        <v>169068.16</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>168924.45</v>
+        <v>169095.2</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>168910.94</v>
+        <v>169081.68</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>110993.66</v>
+        <v>111105.85</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110607.54</v>
+        <v>110719.34</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110800.6</v>
+        <v>110912.6</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62161.35</v>
+        <v>62224.18</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62513.93</v>
+        <v>62577.12</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62337.64</v>
+        <v>62400.65</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26611.88</v>
+        <v>26638.78</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26810.13</v>
+        <v>26837.23</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26711</v>
+        <v>26738</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6264.15</v>
+        <v>6270.49</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6414.73</v>
+        <v>6421.22</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6339.44</v>
+        <v>6345.85</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4494</v>
+        <v>13.4457</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3709.96</v>
+        <v>3713.71</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3703.52</v>
+        <v>3707.27</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3706.74</v>
+        <v>3710.49</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>188918.38</v>
+        <v>189105.25</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>189840.84</v>
+        <v>190028.62</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189379.61</v>
+        <v>189566.93</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>136969.82</v>
+        <v>137105.3</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>137925.64</v>
+        <v>138062.07</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137447.73</v>
+        <v>137583.69</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86578.64999999999</v>
+        <v>86664.28999999999</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87279.3</v>
+        <v>87365.63</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>86928.97</v>
+        <v>87014.96000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41355.36</v>
+        <v>41396.27</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41289.04</v>
+        <v>41329.88</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41322.2</v>
+        <v>41363.08</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12896</v>
+        <v>12908.75</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12753.95</v>
+        <v>12766.57</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12824.98</v>
+        <v>12837.66</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4213</v>
+        <v>13.4247</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4475.72</v>
+        <v>4480.15</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4366.46</v>
+        <v>4370.78</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4421.09</v>
+        <v>4425.46</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-02
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149034.63</v>
+        <v>149120.83</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>150913.53</v>
+        <v>151000.81</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>149974.08</v>
+        <v>150060.82</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114076.31</v>
+        <v>114142.29</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114851.92</v>
+        <v>114918.35</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114464.12</v>
+        <v>114530.32</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81339.08</v>
+        <v>81386.13</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81845.92999999999</v>
+        <v>81893.25999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81592.5</v>
+        <v>81639.7</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57636.85</v>
+        <v>57670.19</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57200.03</v>
+        <v>57233.12</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57418.44</v>
+        <v>57451.65</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37231.12</v>
+        <v>37252.65</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37535.68</v>
+        <v>37557.39</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37383.4</v>
+        <v>37405.02</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.4047</v>
+        <v>13.3845</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16933.41</v>
+        <v>16943.2</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16822.21</v>
+        <v>16831.94</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16877.81</v>
+        <v>16887.57</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>161912.32</v>
+        <v>162013.28</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161043.53</v>
+        <v>161143.95</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161477.93</v>
+        <v>161578.61</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121596.65</v>
+        <v>121672.47</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119879.27</v>
+        <v>119954.02</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120737.96</v>
+        <v>120813.24</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86873.25</v>
+        <v>86927.41</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85797.49000000001</v>
+        <v>85850.99000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86335.37</v>
+        <v>86389.2</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66175.64</v>
+        <v>66216.89999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65710.44</v>
+        <v>65751.41</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65943.03999999999</v>
+        <v>65984.14999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51697.48</v>
+        <v>51729.72</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49839.52</v>
+        <v>49870.6</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50768.5</v>
+        <v>50800.16</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.4044</v>
+        <v>13.3775</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39189.49</v>
+        <v>39213.93</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40157.88</v>
+        <v>40182.92</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39673.69</v>
+        <v>39698.43</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166671.82</v>
+        <v>166783.12</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168207.15</v>
+        <v>168319.47</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167439.49</v>
+        <v>167551.3</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120147.17</v>
+        <v>120227.4</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118711.15</v>
+        <v>118790.43</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119429.16</v>
+        <v>119508.92</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82302.71000000001</v>
+        <v>82357.67</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>81991.85000000001</v>
+        <v>82046.60000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82147.28</v>
+        <v>82202.14</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54834.01</v>
+        <v>54870.63</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55136.57</v>
+        <v>55173.39</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>54985.29</v>
+        <v>55022.01</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33095.12</v>
+        <v>33117.22</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32707.76</v>
+        <v>32729.6</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32901.44</v>
+        <v>32923.41</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.4407</v>
+        <v>13.4097</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17181.58</v>
+        <v>17193.06</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17862.75</v>
+        <v>17874.67</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17522.16</v>
+        <v>17533.87</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128778.78</v>
+        <v>128871.29</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128873.14</v>
+        <v>128965.72</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128825.96</v>
+        <v>128918.51</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89186.05</v>
+        <v>89250.12</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87802.14</v>
+        <v>87865.22</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88494.10000000001</v>
+        <v>88557.67</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56058.44</v>
+        <v>56098.71</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56344.53</v>
+        <v>56385.01</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56201.48</v>
+        <v>56241.86</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29677.38</v>
+        <v>29698.7</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29877.14</v>
+        <v>29898.6</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29777.26</v>
+        <v>29798.65</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6806.75</v>
+        <v>6811.64</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6805.45</v>
+        <v>6810.34</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6806.1</v>
+        <v>6810.99</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4771</v>
+        <v>13.442</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3782.13</v>
+        <v>3784.85</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3692.92</v>
+        <v>3695.58</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3737.53</v>
+        <v>3740.21</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108701</v>
+        <v>108784.98</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109177.88</v>
+        <v>109262.23</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>108939.44</v>
+        <v>109023.61</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76230.57000000001</v>
+        <v>76289.46000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75688.22</v>
+        <v>75746.69</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>75959.39</v>
+        <v>76018.08</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46127.21</v>
+        <v>46162.85</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47230.05</v>
+        <v>47266.54</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46678.63</v>
+        <v>46714.7</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28656.94</v>
+        <v>28679.08</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28550.14</v>
+        <v>28572.2</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28603.54</v>
+        <v>28625.64</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14057.84</v>
+        <v>14068.7</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14179.71</v>
+        <v>14190.67</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14118.77</v>
+        <v>14129.68</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.5118</v>
+        <v>13.4727</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6517.22</v>
+        <v>6522.25</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6356.21</v>
+        <v>6361.12</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6436.72</v>
+        <v>6441.69</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49460.7</v>
+        <v>49502.03</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49129.57</v>
+        <v>49170.62</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49295.13</v>
+        <v>49336.32</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43512.2</v>
+        <v>43548.56</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43705.38</v>
+        <v>43741.9</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43608.79</v>
+        <v>43645.23</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31844.39</v>
+        <v>31871</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32183.52</v>
+        <v>32210.41</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32013.96</v>
+        <v>32040.71</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22390.7</v>
+        <v>22409.41</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22544.47</v>
+        <v>22563.31</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22467.59</v>
+        <v>22486.36</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14391.22</v>
+        <v>14403.24</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14596.01</v>
+        <v>14608.21</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14493.61</v>
+        <v>14505.72</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.5482</v>
+        <v>13.505</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8270.639999999999</v>
+        <v>8277.549999999999</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8325.440000000001</v>
+        <v>8332.4</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8298.040000000001</v>
+        <v>8304.969999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48644.91</v>
+        <v>48689.09</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47928.98</v>
+        <v>47972.51</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48286.94</v>
+        <v>48330.8</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43562.2</v>
+        <v>43601.76</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43227.56</v>
+        <v>43266.82</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43394.88</v>
+        <v>43434.29</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31460.64</v>
+        <v>31489.21</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30895.08</v>
+        <v>30923.14</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31177.86</v>
+        <v>31206.18</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23448.61</v>
+        <v>23469.91</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23344.06</v>
+        <v>23365.26</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23396.34</v>
+        <v>23417.59</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18395.13</v>
+        <v>18411.84</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18210.27</v>
+        <v>18226.81</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18302.7</v>
+        <v>18319.33</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5862</v>
+        <v>13.5386</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15471.56</v>
+        <v>15485.62</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15416.32</v>
+        <v>15430.33</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15443.94</v>
+        <v>15457.97</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123311.13</v>
+        <v>123373.81</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123935.6</v>
+        <v>123998.6</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123623.37</v>
+        <v>123686.2</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88427.27</v>
+        <v>88472.22</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88784.74000000001</v>
+        <v>88829.87</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88606.00999999999</v>
+        <v>88651.03999999999</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57764.48</v>
+        <v>57793.84</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57273.89</v>
+        <v>57303</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57519.18</v>
+        <v>57548.42</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33210.64</v>
+        <v>33227.52</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32971.35</v>
+        <v>32988.11</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33091</v>
+        <v>33107.81</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18873.27</v>
+        <v>18882.87</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18798.69</v>
+        <v>18808.25</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18835.98</v>
+        <v>18845.56</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6544</v>
+        <v>13.6507</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7651.92</v>
+        <v>7655.81</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7409.79</v>
+        <v>7413.56</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7530.86</v>
+        <v>7534.68</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>401246.07</v>
+        <v>401448.96</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>396281.66</v>
+        <v>396482.04</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>398763.86</v>
+        <v>398965.5</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301227.26</v>
+        <v>301379.58</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302204.2</v>
+        <v>302357.01</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301715.73</v>
+        <v>301868.3</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210769.64</v>
+        <v>210876.22</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210642.49</v>
+        <v>210749</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210706.07</v>
+        <v>210812.61</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128135.67</v>
+        <v>128200.47</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128418.1</v>
+        <v>128483.03</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128276.89</v>
+        <v>128341.75</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62109.02</v>
+        <v>62140.42</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61818.86</v>
+        <v>61850.12</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61963.94</v>
+        <v>61995.27</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6305</v>
+        <v>13.6324</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31720.1</v>
+        <v>31736.14</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31744.06</v>
+        <v>31760.11</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31732.08</v>
+        <v>31748.12</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>404795.88</v>
+        <v>405002.01</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>405339.98</v>
+        <v>405546.38</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405067.93</v>
+        <v>405274.19</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300475.68</v>
+        <v>300628.68</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298599.54</v>
+        <v>298751.59</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299537.61</v>
+        <v>299690.13</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203812.92</v>
+        <v>203916.7</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203882.64</v>
+        <v>203986.46</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203847.78</v>
+        <v>203951.58</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123334.28</v>
+        <v>123397.08</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123848.52</v>
+        <v>123911.58</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123591.4</v>
+        <v>123654.33</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49254.22</v>
+        <v>49279.3</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49195.52</v>
+        <v>49220.57</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49224.87</v>
+        <v>49249.93</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5065</v>
+        <v>13.5027</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5417.8</v>
+        <v>5420.56</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5453.53</v>
+        <v>5456.31</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5435.67</v>
+        <v>5438.44</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169068.16</v>
+        <v>169156.96</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169095.2</v>
+        <v>169184.02</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169081.68</v>
+        <v>169170.49</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111105.85</v>
+        <v>111164.21</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110719.34</v>
+        <v>110777.5</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110912.6</v>
+        <v>110970.85</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62224.18</v>
+        <v>62256.87</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62577.12</v>
+        <v>62609.99</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62400.65</v>
+        <v>62433.43</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26638.78</v>
+        <v>26652.77</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26837.23</v>
+        <v>26851.33</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26738</v>
+        <v>26752.05</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6270.49</v>
+        <v>6273.78</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6421.22</v>
+        <v>6424.59</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6345.85</v>
+        <v>6349.18</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4457</v>
+        <v>13.4353</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3713.71</v>
+        <v>3715.66</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3707.27</v>
+        <v>3709.21</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3710.49</v>
+        <v>3712.44</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189105.25</v>
+        <v>189208.98</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190028.62</v>
+        <v>190132.87</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189566.93</v>
+        <v>189670.92</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137105.3</v>
+        <v>137180.51</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138062.07</v>
+        <v>138137.81</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137583.69</v>
+        <v>137659.16</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86664.28999999999</v>
+        <v>86711.83</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87365.63</v>
+        <v>87413.56</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87014.96000000001</v>
+        <v>87062.69</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41396.27</v>
+        <v>41418.98</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41329.88</v>
+        <v>41352.55</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41363.08</v>
+        <v>41385.77</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12908.75</v>
+        <v>12915.84</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12766.57</v>
+        <v>12773.57</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12837.66</v>
+        <v>12844.7</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4247</v>
+        <v>13.4093</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4480.15</v>
+        <v>4482.6</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4370.78</v>
+        <v>4373.18</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4425.46</v>
+        <v>4427.89</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-03
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149120.83</v>
+        <v>149203.92</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151000.81</v>
+        <v>151084.95</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150060.82</v>
+        <v>150144.43</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114142.29</v>
+        <v>114205.89</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114918.35</v>
+        <v>114982.38</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114530.32</v>
+        <v>114594.14</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81386.13</v>
+        <v>81431.48</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81893.25999999999</v>
+        <v>81938.89999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81639.7</v>
+        <v>81685.19</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57670.19</v>
+        <v>57702.32</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57233.12</v>
+        <v>57265.01</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57451.65</v>
+        <v>57483.66</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37252.65</v>
+        <v>37273.41</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37557.39</v>
+        <v>37578.32</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37405.02</v>
+        <v>37425.87</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3845</v>
+        <v>13.3694</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16943.2</v>
+        <v>16952.64</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16831.94</v>
+        <v>16841.32</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16887.57</v>
+        <v>16896.98</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162013.28</v>
+        <v>162111.65</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161143.95</v>
+        <v>161241.78</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161578.61</v>
+        <v>161676.72</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121672.47</v>
+        <v>121746.34</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>119954.02</v>
+        <v>120026.85</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120813.24</v>
+        <v>120886.59</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86927.41</v>
+        <v>86980.19</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85850.99000000001</v>
+        <v>85903.12</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86389.2</v>
+        <v>86441.64999999999</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66216.89999999999</v>
+        <v>66257.10000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65751.41</v>
+        <v>65791.33</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>65984.14999999999</v>
+        <v>66024.22</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51729.72</v>
+        <v>51761.13</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49870.6</v>
+        <v>49900.88</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50800.16</v>
+        <v>50831</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3775</v>
+        <v>13.3538</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39213.93</v>
+        <v>39237.74</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40182.92</v>
+        <v>40207.32</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39698.43</v>
+        <v>39722.53</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166783.12</v>
+        <v>166895.28</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168319.47</v>
+        <v>168432.66</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167551.3</v>
+        <v>167663.97</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120227.4</v>
+        <v>120308.25</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118790.43</v>
+        <v>118870.31</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119508.92</v>
+        <v>119589.28</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82357.67</v>
+        <v>82413.05</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82046.60000000001</v>
+        <v>82101.77</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82202.14</v>
+        <v>82257.41</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54870.63</v>
+        <v>54907.53</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55173.39</v>
+        <v>55210.49</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55022.01</v>
+        <v>55059.01</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33117.22</v>
+        <v>33139.49</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32729.6</v>
+        <v>32751.61</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32923.41</v>
+        <v>32945.55</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.4097</v>
+        <v>13.3774</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17193.06</v>
+        <v>17204.62</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17874.67</v>
+        <v>17886.69</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17533.87</v>
+        <v>17545.66</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128871.29</v>
+        <v>128968.07</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>128965.72</v>
+        <v>129062.56</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>128918.51</v>
+        <v>129015.31</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89250.12</v>
+        <v>89317.14</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87865.22</v>
+        <v>87931.2</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88557.67</v>
+        <v>88624.17</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56098.71</v>
+        <v>56140.84</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56385.01</v>
+        <v>56427.35</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56241.86</v>
+        <v>56284.09</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29698.7</v>
+        <v>29721</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29898.6</v>
+        <v>29921.05</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29798.65</v>
+        <v>29821.03</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6811.64</v>
+        <v>6816.75</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6810.34</v>
+        <v>6815.45</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6810.99</v>
+        <v>6816.1</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.442</v>
+        <v>13.4011</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3784.85</v>
+        <v>3787.69</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3695.58</v>
+        <v>3698.35</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3740.21</v>
+        <v>3743.02</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108784.98</v>
+        <v>108876.16</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109262.23</v>
+        <v>109353.8</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109023.61</v>
+        <v>109114.98</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76289.46000000001</v>
+        <v>76353.39999999999</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75746.69</v>
+        <v>75810.17999999999</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76018.08</v>
+        <v>76081.78999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46162.85</v>
+        <v>46201.54</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47266.54</v>
+        <v>47306.16</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46714.7</v>
+        <v>46753.85</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28679.08</v>
+        <v>28703.12</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28572.2</v>
+        <v>28596.15</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28625.64</v>
+        <v>28649.63</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14068.7</v>
+        <v>14080.49</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14190.67</v>
+        <v>14202.56</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14129.68</v>
+        <v>14141.52</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4727</v>
+        <v>13.4237</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6522.25</v>
+        <v>6527.72</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6361.12</v>
+        <v>6366.46</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6441.69</v>
+        <v>6447.09</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49502.03</v>
+        <v>49548.67</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49170.62</v>
+        <v>49216.95</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49336.32</v>
+        <v>49382.81</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43548.56</v>
+        <v>43589.6</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43741.9</v>
+        <v>43783.12</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43645.23</v>
+        <v>43686.36</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31871</v>
+        <v>31901.03</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32210.41</v>
+        <v>32240.77</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32040.71</v>
+        <v>32070.9</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22409.41</v>
+        <v>22430.53</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22563.31</v>
+        <v>22584.57</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22486.36</v>
+        <v>22507.55</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14403.24</v>
+        <v>14416.81</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14608.21</v>
+        <v>14621.97</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14505.72</v>
+        <v>14519.39</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.505</v>
+        <v>13.4473</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8277.549999999999</v>
+        <v>8285.35</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8332.4</v>
+        <v>8340.25</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8304.969999999999</v>
+        <v>8312.799999999999</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48689.09</v>
+        <v>48740.96</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>47972.51</v>
+        <v>48023.62</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48330.8</v>
+        <v>48382.29</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43601.76</v>
+        <v>43648.22</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43266.82</v>
+        <v>43312.91</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43434.29</v>
+        <v>43480.56</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31489.21</v>
+        <v>31522.76</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30923.14</v>
+        <v>30956.08</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31206.18</v>
+        <v>31239.42</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23469.91</v>
+        <v>23494.91</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23365.26</v>
+        <v>23390.16</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23417.59</v>
+        <v>23442.53</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18411.84</v>
+        <v>18431.46</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18226.81</v>
+        <v>18246.23</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18319.33</v>
+        <v>18338.84</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.5386</v>
+        <v>13.4721</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15485.62</v>
+        <v>15502.11</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15430.33</v>
+        <v>15446.76</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15457.97</v>
+        <v>15474.44</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123373.81</v>
+        <v>123436.52</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>123998.6</v>
+        <v>124061.62</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123686.2</v>
+        <v>123749.07</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88472.22</v>
+        <v>88517.19</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88829.87</v>
+        <v>88875.02</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88651.03999999999</v>
+        <v>88696.10000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57793.84</v>
+        <v>57823.21</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57303</v>
+        <v>57332.13</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57548.42</v>
+        <v>57577.67</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33227.52</v>
+        <v>33244.41</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>32988.11</v>
+        <v>33004.87</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33107.81</v>
+        <v>33124.64</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18882.87</v>
+        <v>18892.46</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18808.25</v>
+        <v>18817.81</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18845.56</v>
+        <v>18855.14</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6507</v>
+        <v>13.6405</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7655.81</v>
+        <v>7659.7</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7413.56</v>
+        <v>7417.33</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7534.68</v>
+        <v>7538.51</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>401448.96</v>
+        <v>401653.71</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>396482.04</v>
+        <v>396684.26</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>398965.5</v>
+        <v>399168.99</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301379.58</v>
+        <v>301533.29</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302357.01</v>
+        <v>302511.23</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>301868.3</v>
+        <v>302022.26</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210876.22</v>
+        <v>210983.77</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210749</v>
+        <v>210856.49</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210812.61</v>
+        <v>210920.13</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128200.47</v>
+        <v>128265.85</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128483.03</v>
+        <v>128548.56</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128341.75</v>
+        <v>128407.21</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62140.42</v>
+        <v>62172.12</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61850.12</v>
+        <v>61881.67</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>61995.27</v>
+        <v>62026.89</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6324</v>
+        <v>13.6289</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31736.14</v>
+        <v>31752.33</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31760.11</v>
+        <v>31776.31</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31748.12</v>
+        <v>31764.32</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405002.01</v>
+        <v>405205.28</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>405546.38</v>
+        <v>405749.93</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405274.19</v>
+        <v>405477.61</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300628.68</v>
+        <v>300779.57</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298751.59</v>
+        <v>298901.53</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299690.13</v>
+        <v>299840.55</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>203916.7</v>
+        <v>204019.05</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>203986.46</v>
+        <v>204088.85</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>203951.58</v>
+        <v>204053.95</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123397.08</v>
+        <v>123459.02</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123911.58</v>
+        <v>123973.77</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123654.33</v>
+        <v>123716.4</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49279.3</v>
+        <v>49304.03</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49220.57</v>
+        <v>49245.28</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49249.93</v>
+        <v>49274.65</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5027</v>
+        <v>13.5032</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5420.56</v>
+        <v>5423.28</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5456.31</v>
+        <v>5459.05</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5438.44</v>
+        <v>5441.17</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169156.96</v>
+        <v>169242.69</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169184.02</v>
+        <v>169269.76</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169170.49</v>
+        <v>169256.23</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111164.21</v>
+        <v>111220.55</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110777.5</v>
+        <v>110833.64</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>110970.85</v>
+        <v>111027.1</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62256.87</v>
+        <v>62288.42</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62609.99</v>
+        <v>62641.72</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62433.43</v>
+        <v>62465.07</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26652.77</v>
+        <v>26666.28</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26851.33</v>
+        <v>26864.94</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26752.05</v>
+        <v>26765.61</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6273.78</v>
+        <v>6276.96</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6424.59</v>
+        <v>6427.85</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6349.18</v>
+        <v>6352.4</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4353</v>
+        <v>13.4325</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3715.66</v>
+        <v>3717.54</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3709.21</v>
+        <v>3711.09</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3712.44</v>
+        <v>3714.32</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189208.98</v>
+        <v>189308.83</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190132.87</v>
+        <v>190233.2</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189670.92</v>
+        <v>189771.02</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137180.51</v>
+        <v>137252.91</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138137.81</v>
+        <v>138210.71</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137659.16</v>
+        <v>137731.81</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86711.83</v>
+        <v>86757.59</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87413.56</v>
+        <v>87459.69</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87062.69</v>
+        <v>87108.64</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41418.98</v>
+        <v>41440.84</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41352.55</v>
+        <v>41374.38</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41385.77</v>
+        <v>41407.61</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12915.84</v>
+        <v>12922.65</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12773.57</v>
+        <v>12780.31</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12844.7</v>
+        <v>12851.48</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4093</v>
+        <v>13.4003</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4482.6</v>
+        <v>4484.97</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4373.18</v>
+        <v>4375.48</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4427.89</v>
+        <v>4430.23</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-04
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149203.92</v>
+        <v>149286.83</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151084.95</v>
+        <v>151168.91</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150144.43</v>
+        <v>150227.87</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114205.89</v>
+        <v>114269.36</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>114982.38</v>
+        <v>115046.28</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114594.14</v>
+        <v>114657.82</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81431.48</v>
+        <v>81476.73</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81938.89999999999</v>
+        <v>81984.42999999999</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81685.19</v>
+        <v>81730.58</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57702.32</v>
+        <v>57734.39</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57265.01</v>
+        <v>57296.83</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57483.66</v>
+        <v>57515.61</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37273.41</v>
+        <v>37294.12</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37578.32</v>
+        <v>37599.2</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37425.87</v>
+        <v>37446.66</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3694</v>
+        <v>13.3545</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16952.64</v>
+        <v>16962.06</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16841.32</v>
+        <v>16850.68</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16896.98</v>
+        <v>16906.37</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162111.65</v>
+        <v>162210.02</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161241.78</v>
+        <v>161339.63</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161676.72</v>
+        <v>161774.82</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121746.34</v>
+        <v>121820.22</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120026.85</v>
+        <v>120099.68</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120886.59</v>
+        <v>120959.95</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>86980.19</v>
+        <v>87032.97</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85903.12</v>
+        <v>85955.24000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86441.64999999999</v>
+        <v>86494.11</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66257.10000000001</v>
+        <v>66297.31</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65791.33</v>
+        <v>65831.25</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66024.22</v>
+        <v>66064.28</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51761.13</v>
+        <v>51792.54</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49900.88</v>
+        <v>49931.16</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50831</v>
+        <v>50861.85</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3538</v>
+        <v>13.3298</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39237.74</v>
+        <v>39261.55</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40207.32</v>
+        <v>40231.72</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39722.53</v>
+        <v>39746.63</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>166895.28</v>
+        <v>167004.29</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168432.66</v>
+        <v>168542.68</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167663.97</v>
+        <v>167773.48</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120308.25</v>
+        <v>120386.83</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118870.31</v>
+        <v>118947.95</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119589.28</v>
+        <v>119667.39</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82413.05</v>
+        <v>82466.88</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82101.77</v>
+        <v>82155.39999999999</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82257.41</v>
+        <v>82311.14</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54907.53</v>
+        <v>54943.39</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55210.49</v>
+        <v>55246.55</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55059.01</v>
+        <v>55094.97</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33139.49</v>
+        <v>33161.14</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32751.61</v>
+        <v>32773</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32945.55</v>
+        <v>32967.07</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3774</v>
+        <v>13.3484</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17204.62</v>
+        <v>17215.85</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17886.69</v>
+        <v>17898.38</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17545.66</v>
+        <v>17557.12</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>128968.07</v>
+        <v>129059.29</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129062.56</v>
+        <v>129153.85</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129015.31</v>
+        <v>129106.57</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89317.14</v>
+        <v>89380.32000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87931.2</v>
+        <v>87993.39</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88624.17</v>
+        <v>88686.86</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56140.84</v>
+        <v>56180.55</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56427.35</v>
+        <v>56467.26</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56284.09</v>
+        <v>56323.9</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29721</v>
+        <v>29742.02</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29921.05</v>
+        <v>29942.22</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29821.03</v>
+        <v>29842.12</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6816.75</v>
+        <v>6821.58</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6815.45</v>
+        <v>6820.28</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6816.1</v>
+        <v>6820.93</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4011</v>
+        <v>13.3669</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3787.69</v>
+        <v>3790.37</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3698.35</v>
+        <v>3700.97</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3743.02</v>
+        <v>3745.67</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108876.16</v>
+        <v>108959.6</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109353.8</v>
+        <v>109437.61</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109114.98</v>
+        <v>109198.6</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76353.39999999999</v>
+        <v>76411.91</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75810.17999999999</v>
+        <v>75868.28</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76081.78999999999</v>
+        <v>76140.10000000001</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46201.54</v>
+        <v>46236.95</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47306.16</v>
+        <v>47342.41</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46753.85</v>
+        <v>46789.68</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28703.12</v>
+        <v>28725.12</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28596.15</v>
+        <v>28618.06</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28649.63</v>
+        <v>28671.59</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14080.49</v>
+        <v>14091.28</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14202.56</v>
+        <v>14213.45</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14141.52</v>
+        <v>14152.36</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4237</v>
+        <v>13.3847</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6527.72</v>
+        <v>6532.72</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6366.46</v>
+        <v>6371.33</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6447.09</v>
+        <v>6452.03</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49548.67</v>
+        <v>49590.09</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49216.95</v>
+        <v>49258.09</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49382.81</v>
+        <v>49424.09</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43589.6</v>
+        <v>43626.03</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43783.12</v>
+        <v>43819.71</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43686.36</v>
+        <v>43722.87</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31901.03</v>
+        <v>31927.69</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32240.77</v>
+        <v>32267.71</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32070.9</v>
+        <v>32097.7</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22430.53</v>
+        <v>22449.27</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22584.57</v>
+        <v>22603.45</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22507.55</v>
+        <v>22526.36</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14416.81</v>
+        <v>14428.86</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14621.97</v>
+        <v>14634.19</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14519.39</v>
+        <v>14531.53</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4473</v>
+        <v>13.4032</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8285.35</v>
+        <v>8292.280000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8340.25</v>
+        <v>8347.219999999999</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8312.799999999999</v>
+        <v>8319.75</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48740.96</v>
+        <v>48785.64</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48023.62</v>
+        <v>48067.64</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48382.29</v>
+        <v>48426.64</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43648.22</v>
+        <v>43688.23</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43312.91</v>
+        <v>43352.62</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43480.56</v>
+        <v>43520.42</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31522.76</v>
+        <v>31551.66</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30956.08</v>
+        <v>30984.46</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31239.42</v>
+        <v>31268.06</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23494.91</v>
+        <v>23516.45</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23390.16</v>
+        <v>23411.6</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23442.53</v>
+        <v>23464.02</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18431.46</v>
+        <v>18448.35</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18246.23</v>
+        <v>18262.96</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18338.84</v>
+        <v>18355.66</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4721</v>
+        <v>13.4227</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15502.11</v>
+        <v>15516.32</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15446.76</v>
+        <v>15460.92</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15474.44</v>
+        <v>15488.62</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123436.52</v>
+        <v>123499.17</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>124061.62</v>
+        <v>124124.59</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123749.07</v>
+        <v>123811.88</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88517.19</v>
+        <v>88562.11</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88875.02</v>
+        <v>88920.13</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88696.10000000001</v>
+        <v>88741.12</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57823.21</v>
+        <v>57852.56</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57332.13</v>
+        <v>57361.22</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57577.67</v>
+        <v>57606.89</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33244.41</v>
+        <v>33261.29</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>33004.87</v>
+        <v>33021.62</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33124.64</v>
+        <v>33141.45</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18892.46</v>
+        <v>18902.05</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18817.81</v>
+        <v>18827.36</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18855.14</v>
+        <v>18864.71</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6405</v>
+        <v>13.6634</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7659.7</v>
+        <v>7663.59</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7417.33</v>
+        <v>7421.09</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7538.51</v>
+        <v>7542.34</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>401653.71</v>
+        <v>401848.73</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>396684.26</v>
+        <v>396876.87</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399168.99</v>
+        <v>399362.8</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301533.29</v>
+        <v>301679.7</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302511.23</v>
+        <v>302658.11</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302022.26</v>
+        <v>302168.91</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>210983.77</v>
+        <v>211086.22</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210856.49</v>
+        <v>210958.87</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>210920.13</v>
+        <v>211022.54</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128265.85</v>
+        <v>128328.13</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128548.56</v>
+        <v>128610.98</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128407.21</v>
+        <v>128469.56</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62172.12</v>
+        <v>62202.31</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61881.67</v>
+        <v>61911.72</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62026.89</v>
+        <v>62057.01</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6289</v>
+        <v>13.657</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31752.33</v>
+        <v>31767.74</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31776.31</v>
+        <v>31791.74</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31764.32</v>
+        <v>31779.74</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405205.28</v>
+        <v>405400.86</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>405749.93</v>
+        <v>405945.77</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405477.61</v>
+        <v>405673.31</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300779.57</v>
+        <v>300924.74</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>298901.53</v>
+        <v>299045.8</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299840.55</v>
+        <v>299985.27</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204019.05</v>
+        <v>204117.52</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204088.85</v>
+        <v>204187.35</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204053.95</v>
+        <v>204152.44</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123459.02</v>
+        <v>123518.61</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>123973.77</v>
+        <v>124033.61</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123716.4</v>
+        <v>123776.11</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49304.03</v>
+        <v>49327.83</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49245.28</v>
+        <v>49269.05</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49274.65</v>
+        <v>49298.44</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5032</v>
+        <v>13.5159</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5423.28</v>
+        <v>5425.9</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5459.05</v>
+        <v>5461.68</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5441.17</v>
+        <v>5443.79</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169242.69</v>
+        <v>169327.02</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169269.76</v>
+        <v>169354.1</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169256.23</v>
+        <v>169340.56</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111220.55</v>
+        <v>111275.97</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110833.64</v>
+        <v>110888.86</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111027.1</v>
+        <v>111082.41</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62288.42</v>
+        <v>62319.45</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62641.72</v>
+        <v>62672.93</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62465.07</v>
+        <v>62496.19</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26666.28</v>
+        <v>26679.56</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26864.94</v>
+        <v>26878.32</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26765.61</v>
+        <v>26778.94</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6276.96</v>
+        <v>6280.09</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6427.85</v>
+        <v>6431.05</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6352.4</v>
+        <v>6355.57</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4325</v>
+        <v>13.4334</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3717.54</v>
+        <v>3719.4</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3711.09</v>
+        <v>3712.94</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3714.32</v>
+        <v>3716.17</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189308.83</v>
+        <v>189407.53</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190233.2</v>
+        <v>190332.38</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189771.02</v>
+        <v>189869.96</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137252.91</v>
+        <v>137324.47</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138210.71</v>
+        <v>138282.76</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137731.81</v>
+        <v>137803.61</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86757.59</v>
+        <v>86802.82000000001</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87459.69</v>
+        <v>87505.28</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87108.64</v>
+        <v>87154.05</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41440.84</v>
+        <v>41462.44</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41374.38</v>
+        <v>41395.95</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41407.61</v>
+        <v>41429.2</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12922.65</v>
+        <v>12929.39</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12780.31</v>
+        <v>12786.98</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12851.48</v>
+        <v>12858.18</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4003</v>
+        <v>13.3931</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4484.97</v>
+        <v>4487.31</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4375.48</v>
+        <v>4377.77</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4430.23</v>
+        <v>4432.54</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-06
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149286.83</v>
+        <v>149285.32</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151168.91</v>
+        <v>151167.38</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150227.87</v>
+        <v>150226.35</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114269.36</v>
+        <v>114268.2</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115046.28</v>
+        <v>115045.12</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114657.82</v>
+        <v>114656.66</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81476.73</v>
+        <v>81475.89999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81984.42999999999</v>
+        <v>81983.60000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81730.58</v>
+        <v>81729.75</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57734.39</v>
+        <v>57733.8</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57296.83</v>
+        <v>57296.25</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57515.61</v>
+        <v>57515.03</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37294.12</v>
+        <v>37293.75</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37599.2</v>
+        <v>37598.82</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37446.66</v>
+        <v>37446.29</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3545</v>
+        <v>13.3571</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16962.06</v>
+        <v>16961.89</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16850.68</v>
+        <v>16850.51</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16906.37</v>
+        <v>16906.2</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162210.02</v>
+        <v>162209.14</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161339.63</v>
+        <v>161338.75</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161774.82</v>
+        <v>161773.94</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121820.22</v>
+        <v>121819.56</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120099.68</v>
+        <v>120099.03</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120959.95</v>
+        <v>120959.29</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87032.97</v>
+        <v>87032.5</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85955.24000000001</v>
+        <v>85954.78</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86494.11</v>
+        <v>86493.64</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66297.31</v>
+        <v>66296.95</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65831.25</v>
+        <v>65830.89</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66064.28</v>
+        <v>66063.92</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51792.54</v>
+        <v>51792.25</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49931.16</v>
+        <v>49930.89</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50861.85</v>
+        <v>50861.57</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3298</v>
+        <v>13.331</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39261.55</v>
+        <v>39261.33</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40231.72</v>
+        <v>40231.5</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39746.63</v>
+        <v>39746.42</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167004.29</v>
+        <v>167003.76</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168542.68</v>
+        <v>168542.14</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167773.48</v>
+        <v>167772.95</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120386.83</v>
+        <v>120386.45</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118947.95</v>
+        <v>118947.57</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119667.39</v>
+        <v>119667.01</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82466.88</v>
+        <v>82466.62</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82155.39999999999</v>
+        <v>82155.14</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82311.14</v>
+        <v>82310.88</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54943.39</v>
+        <v>54943.22</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55246.55</v>
+        <v>55246.38</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55094.97</v>
+        <v>55094.8</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33161.14</v>
+        <v>33161.03</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32773</v>
+        <v>32772.9</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32967.07</v>
+        <v>32966.97</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3484</v>
+        <v>13.349</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17215.85</v>
+        <v>17215.8</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17898.38</v>
+        <v>17898.32</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17557.12</v>
+        <v>17557.06</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4027,7 +4027,7 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129059.29</v>
+        <v>129059.28</v>
       </c>
       <c r="L22" s="57" t="n">
         <v>129153.85</v>
@@ -4086,7 +4086,7 @@
         <v>87993.39</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88686.86</v>
+        <v>88686.85000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108959.6</v>
+        <v>108960.01</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109437.61</v>
+        <v>109438.02</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109198.6</v>
+        <v>109199.02</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76411.91</v>
+        <v>76412.21000000001</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75868.28</v>
+        <v>75868.57000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76140.10000000001</v>
+        <v>76140.39</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46236.95</v>
+        <v>46237.12</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47342.41</v>
+        <v>47342.59</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46789.68</v>
+        <v>46789.86</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28725.12</v>
+        <v>28725.23</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28618.06</v>
+        <v>28618.17</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28671.59</v>
+        <v>28671.7</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14091.28</v>
+        <v>14091.33</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14213.45</v>
+        <v>14213.5</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14152.36</v>
+        <v>14152.42</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3847</v>
+        <v>13.3841</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6532.72</v>
+        <v>6532.75</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6371.33</v>
+        <v>6371.36</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6452.03</v>
+        <v>6452.05</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49590.09</v>
+        <v>49590.52</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49258.09</v>
+        <v>49258.52</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49424.09</v>
+        <v>49424.52</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43626.03</v>
+        <v>43626.42</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43819.71</v>
+        <v>43820.1</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43722.87</v>
+        <v>43723.26</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31927.69</v>
+        <v>31927.97</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32267.71</v>
+        <v>32268</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32097.7</v>
+        <v>32097.99</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22449.27</v>
+        <v>22449.47</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22603.45</v>
+        <v>22603.65</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22526.36</v>
+        <v>22526.56</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14428.86</v>
+        <v>14428.99</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14634.19</v>
+        <v>14634.32</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14531.53</v>
+        <v>14531.66</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4032</v>
+        <v>13.4021</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8292.280000000001</v>
+        <v>8292.35</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8347.219999999999</v>
+        <v>8347.290000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8319.75</v>
+        <v>8319.82</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48785.64</v>
+        <v>48786.37</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48067.64</v>
+        <v>48068.36</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48426.64</v>
+        <v>48427.36</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43688.23</v>
+        <v>43688.88</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43352.62</v>
+        <v>43353.26</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43520.42</v>
+        <v>43521.07</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31551.66</v>
+        <v>31552.13</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30984.46</v>
+        <v>30984.92</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31268.06</v>
+        <v>31268.53</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23516.45</v>
+        <v>23516.8</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23411.6</v>
+        <v>23411.95</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23464.02</v>
+        <v>23464.37</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18448.35</v>
+        <v>18448.63</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18262.96</v>
+        <v>18263.23</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18355.66</v>
+        <v>18355.93</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4227</v>
+        <v>13.4209</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15516.32</v>
+        <v>15516.56</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15460.92</v>
+        <v>15461.16</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15488.62</v>
+        <v>15488.86</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5269,11 +5269,11 @@
       </c>
       <c r="B46" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>123499.17</v>
+        <v>108374.67</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>124124.59</v>
+        <v>108923.5</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>123811.88</v>
+        <v>108649.09</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5322,11 +5322,11 @@
       </c>
       <c r="B47" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>88562.11</v>
+        <v>77716.23</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>88920.13</v>
+        <v>78030.39999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>88741.12</v>
+        <v>77873.32000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5375,11 +5375,11 @@
       </c>
       <c r="B48" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>57852.56</v>
+        <v>50767.57</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>57361.22</v>
+        <v>50336.4</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>57606.89</v>
+        <v>50551.99</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5428,11 +5428,11 @@
       </c>
       <c r="B49" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>33261.29</v>
+        <v>29187.9</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>33021.62</v>
+        <v>28977.59</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>33141.45</v>
+        <v>29082.74</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5481,11 +5481,11 @@
       </c>
       <c r="B50" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>18902.05</v>
+        <v>16587.19</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>18827.36</v>
+        <v>16521.64</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>18864.71</v>
+        <v>16554.41</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5534,11 +5534,11 @@
       </c>
       <c r="B51" s="54" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2027-09-06</t>
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.6634</v>
+        <v>13.4436</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>7663.59</v>
+        <v>6725.06</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>7421.09</v>
+        <v>6512.26</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>7542.34</v>
+        <v>6618.66</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>401848.73</v>
+        <v>401842.21</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>396876.87</v>
+        <v>396870.43</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399362.8</v>
+        <v>399356.32</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301679.7</v>
+        <v>301674.8</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302658.11</v>
+        <v>302653.2</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302168.91</v>
+        <v>302164</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211086.22</v>
+        <v>211082.79</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210958.87</v>
+        <v>210955.45</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211022.54</v>
+        <v>211019.12</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128328.13</v>
+        <v>128326.05</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128610.98</v>
+        <v>128608.89</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128469.56</v>
+        <v>128467.47</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62202.31</v>
+        <v>62201.3</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61911.72</v>
+        <v>61910.71</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62057.01</v>
+        <v>62056</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.657</v>
+        <v>13.6781</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31767.74</v>
+        <v>31767.23</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31791.74</v>
+        <v>31791.22</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31779.74</v>
+        <v>31779.22</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405400.86</v>
+        <v>405393.71</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>405945.77</v>
+        <v>405938.6</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405673.31</v>
+        <v>405666.16</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300924.74</v>
+        <v>300919.44</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299045.8</v>
+        <v>299040.52</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299985.27</v>
+        <v>299979.98</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204117.52</v>
+        <v>204113.92</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204187.35</v>
+        <v>204183.75</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204152.44</v>
+        <v>204148.84</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123518.61</v>
+        <v>123516.43</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124033.61</v>
+        <v>124031.42</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123776.11</v>
+        <v>123773.92</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49327.83</v>
+        <v>49326.96</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49269.05</v>
+        <v>49268.18</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49298.44</v>
+        <v>49297.57</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5159</v>
+        <v>13.5271</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5425.9</v>
+        <v>5425.81</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5461.68</v>
+        <v>5461.59</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5443.79</v>
+        <v>5443.7</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169327.02</v>
+        <v>169324.58</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169354.1</v>
+        <v>169351.66</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169340.56</v>
+        <v>169338.12</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111275.97</v>
+        <v>111274.36</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110888.86</v>
+        <v>110887.27</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111082.41</v>
+        <v>111080.81</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62319.45</v>
+        <v>62318.56</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62672.93</v>
+        <v>62672.03</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62496.19</v>
+        <v>62495.29</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26679.56</v>
+        <v>26679.18</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26878.32</v>
+        <v>26877.94</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26778.94</v>
+        <v>26778.56</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6280.09</v>
+        <v>6280</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6431.05</v>
+        <v>6430.96</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6355.57</v>
+        <v>6355.48</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4334</v>
+        <v>13.4397</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3719.4</v>
+        <v>3719.34</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3712.94</v>
+        <v>3712.89</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3716.17</v>
+        <v>3716.12</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189407.53</v>
+        <v>189404.94</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190332.38</v>
+        <v>190329.78</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189869.96</v>
+        <v>189867.36</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137324.47</v>
+        <v>137322.59</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138282.76</v>
+        <v>138280.87</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137803.61</v>
+        <v>137801.73</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86802.82000000001</v>
+        <v>86801.64</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87505.28</v>
+        <v>87504.09</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87154.05</v>
+        <v>87152.86</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41462.44</v>
+        <v>41461.88</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41395.95</v>
+        <v>41395.38</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41429.2</v>
+        <v>41428.63</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12929.39</v>
+        <v>12929.21</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12786.98</v>
+        <v>12786.8</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12858.18</v>
+        <v>12858.01</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3931</v>
+        <v>13.3975</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4487.31</v>
+        <v>4487.25</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4377.77</v>
+        <v>4377.71</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4432.54</v>
+        <v>4432.48</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-07
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149285.32</v>
+        <v>149358.56</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151167.38</v>
+        <v>151241.55</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150226.35</v>
+        <v>150300.06</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114268.2</v>
+        <v>114324.27</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115045.12</v>
+        <v>115101.56</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114656.66</v>
+        <v>114712.91</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81475.89999999999</v>
+        <v>81515.88</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>81983.60000000001</v>
+        <v>82023.82000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81729.75</v>
+        <v>81769.85000000001</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57733.8</v>
+        <v>57762.13</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57296.25</v>
+        <v>57324.36</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57515.03</v>
+        <v>57543.25</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37293.75</v>
+        <v>37312.05</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37598.82</v>
+        <v>37617.27</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37446.29</v>
+        <v>37464.66</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3571</v>
+        <v>13.3589</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16961.89</v>
+        <v>16970.21</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16850.51</v>
+        <v>16858.78</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16906.2</v>
+        <v>16914.5</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162209.14</v>
+        <v>162290.31</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161338.75</v>
+        <v>161419.49</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161773.94</v>
+        <v>161854.9</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121819.56</v>
+        <v>121880.52</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120099.03</v>
+        <v>120159.13</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>120959.29</v>
+        <v>121019.82</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87032.5</v>
+        <v>87076.05</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85954.78</v>
+        <v>85997.78999999999</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86493.64</v>
+        <v>86536.92</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66296.95</v>
+        <v>66330.13</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65830.89</v>
+        <v>65863.84</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66063.92</v>
+        <v>66096.98</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51792.25</v>
+        <v>51818.17</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49930.89</v>
+        <v>49955.87</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50861.57</v>
+        <v>50887.02</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.331</v>
+        <v>13.3302</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39261.33</v>
+        <v>39280.98</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40231.5</v>
+        <v>40251.63</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39746.42</v>
+        <v>39766.31</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167003.76</v>
+        <v>167087.54</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168542.14</v>
+        <v>168626.69</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167772.95</v>
+        <v>167857.11</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120386.45</v>
+        <v>120446.84</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>118947.57</v>
+        <v>119007.24</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119667.01</v>
+        <v>119727.04</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82466.62</v>
+        <v>82507.99000000001</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82155.14</v>
+        <v>82196.35000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82310.88</v>
+        <v>82352.17</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54943.22</v>
+        <v>54970.78</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55246.38</v>
+        <v>55274.09</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55094.8</v>
+        <v>55122.44</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33161.03</v>
+        <v>33177.67</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32772.9</v>
+        <v>32789.34</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32966.97</v>
+        <v>32983.5</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.349</v>
+        <v>13.3481</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17215.8</v>
+        <v>17224.44</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17898.32</v>
+        <v>17907.3</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17557.06</v>
+        <v>17565.87</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129059.28</v>
+        <v>129124.19</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129153.85</v>
+        <v>129218.81</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129106.57</v>
+        <v>129171.5</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89380.32000000001</v>
+        <v>89425.27</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>87993.39</v>
+        <v>88037.64</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88686.85000000001</v>
+        <v>88731.46000000001</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56180.55</v>
+        <v>56208.8</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56467.26</v>
+        <v>56495.66</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56323.9</v>
+        <v>56352.23</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29742.02</v>
+        <v>29756.98</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29942.22</v>
+        <v>29957.28</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29842.12</v>
+        <v>29857.13</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6821.58</v>
+        <v>6825.01</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6820.28</v>
+        <v>6823.71</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6820.93</v>
+        <v>6824.36</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3669</v>
+        <v>13.3661</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3790.37</v>
+        <v>3792.28</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3700.97</v>
+        <v>3702.83</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3745.67</v>
+        <v>3747.55</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>108960.01</v>
+        <v>109014.94</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109438.02</v>
+        <v>109493.2</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109199.02</v>
+        <v>109254.07</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76412.21000000001</v>
+        <v>76450.73</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75868.57000000001</v>
+        <v>75906.82000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76140.39</v>
+        <v>76178.77</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46237.12</v>
+        <v>46260.43</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47342.59</v>
+        <v>47366.46</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46789.86</v>
+        <v>46813.45</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28725.23</v>
+        <v>28739.71</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28618.17</v>
+        <v>28632.6</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28671.7</v>
+        <v>28686.15</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14091.33</v>
+        <v>14098.44</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14213.5</v>
+        <v>14220.67</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14152.42</v>
+        <v>14159.55</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3841</v>
+        <v>13.3833</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6532.75</v>
+        <v>6536.04</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6371.36</v>
+        <v>6374.57</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6452.05</v>
+        <v>6455.31</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49590.52</v>
+        <v>49615.58</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49258.52</v>
+        <v>49283.42</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49424.52</v>
+        <v>49449.5</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43626.42</v>
+        <v>43648.46</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43820.1</v>
+        <v>43842.24</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43723.26</v>
+        <v>43745.35</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31927.97</v>
+        <v>31944.11</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32268</v>
+        <v>32284.3</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32097.99</v>
+        <v>32114.21</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22449.47</v>
+        <v>22460.82</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22603.65</v>
+        <v>22615.07</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22526.56</v>
+        <v>22537.94</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14428.99</v>
+        <v>14436.28</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14634.32</v>
+        <v>14641.72</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14531.66</v>
+        <v>14539</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4021</v>
+        <v>13.4013</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8292.35</v>
+        <v>8296.540000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8347.290000000001</v>
+        <v>8351.51</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8319.82</v>
+        <v>8324.030000000001</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48786.37</v>
+        <v>48811.09</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48068.36</v>
+        <v>48092.71</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48427.36</v>
+        <v>48451.9</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43688.88</v>
+        <v>43711.02</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43353.26</v>
+        <v>43375.23</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43521.07</v>
+        <v>43543.12</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31552.13</v>
+        <v>31568.11</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>30984.92</v>
+        <v>31000.62</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31268.53</v>
+        <v>31284.37</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23516.8</v>
+        <v>23528.72</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23411.95</v>
+        <v>23423.81</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23464.37</v>
+        <v>23476.26</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18448.63</v>
+        <v>18457.98</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18263.23</v>
+        <v>18272.48</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18355.93</v>
+        <v>18365.23</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4209</v>
+        <v>13.4201</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15516.56</v>
+        <v>15524.42</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15461.16</v>
+        <v>15468.99</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15488.86</v>
+        <v>15496.7</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108374.67</v>
+        <v>108430.34</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>108923.5</v>
+        <v>108979.45</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108649.09</v>
+        <v>108704.89</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77716.23</v>
+        <v>77756.14999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78030.39999999999</v>
+        <v>78070.48</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>77873.32000000001</v>
+        <v>77913.32000000001</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50767.57</v>
+        <v>50793.64</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50336.4</v>
+        <v>50362.26</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50551.99</v>
+        <v>50577.95</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29187.9</v>
+        <v>29202.89</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>28977.59</v>
+        <v>28992.47</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29082.74</v>
+        <v>29097.68</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16587.19</v>
+        <v>16595.71</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16521.64</v>
+        <v>16530.13</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16554.41</v>
+        <v>16562.92</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4436</v>
+        <v>13.4421</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6725.06</v>
+        <v>6728.51</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6512.26</v>
+        <v>6515.6</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6618.66</v>
+        <v>6622.06</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>401842.21</v>
+        <v>402044.67</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>396870.43</v>
+        <v>397070.38</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399356.32</v>
+        <v>399557.53</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301674.8</v>
+        <v>301826.8</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302653.2</v>
+        <v>302805.69</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302164</v>
+        <v>302316.24</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211082.79</v>
+        <v>211189.14</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>210955.45</v>
+        <v>211061.73</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211019.12</v>
+        <v>211125.44</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128326.05</v>
+        <v>128390.7</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128608.89</v>
+        <v>128673.69</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128467.47</v>
+        <v>128532.2</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62201.3</v>
+        <v>62232.63</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61910.71</v>
+        <v>61941.9</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62056</v>
+        <v>62087.27</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6781</v>
+        <v>13.685</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31767.23</v>
+        <v>31783.23</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31791.22</v>
+        <v>31807.24</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31779.22</v>
+        <v>31795.23</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405393.71</v>
+        <v>405594.96</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>405938.6</v>
+        <v>406140.12</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405666.16</v>
+        <v>405867.54</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>300919.44</v>
+        <v>301068.82</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299040.52</v>
+        <v>299188.98</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>299979.98</v>
+        <v>300128.9</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204113.92</v>
+        <v>204215.25</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204183.75</v>
+        <v>204285.11</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204148.84</v>
+        <v>204250.18</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123516.43</v>
+        <v>123577.74</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124031.42</v>
+        <v>124092.99</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123773.92</v>
+        <v>123835.37</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49326.96</v>
+        <v>49351.44</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49268.18</v>
+        <v>49292.64</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49297.57</v>
+        <v>49322.04</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5271</v>
+        <v>13.5318</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5425.81</v>
+        <v>5428.5</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5461.59</v>
+        <v>5464.3</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5443.7</v>
+        <v>5446.4</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169324.58</v>
+        <v>169408.63</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169351.66</v>
+        <v>169435.73</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169338.12</v>
+        <v>169422.18</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111274.36</v>
+        <v>111329.6</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110887.27</v>
+        <v>110942.31</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111080.81</v>
+        <v>111135.96</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62318.56</v>
+        <v>62349.49</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62672.03</v>
+        <v>62703.14</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62495.29</v>
+        <v>62526.32</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26679.18</v>
+        <v>26692.42</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26877.94</v>
+        <v>26891.28</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26778.56</v>
+        <v>26791.85</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6280</v>
+        <v>6283.11</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6430.96</v>
+        <v>6434.15</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6355.48</v>
+        <v>6358.63</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4397</v>
+        <v>13.4416</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3719.34</v>
+        <v>3721.19</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3712.89</v>
+        <v>3714.73</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3716.12</v>
+        <v>3717.96</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189404.94</v>
+        <v>189498.41</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190329.78</v>
+        <v>190423.7</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189867.36</v>
+        <v>189961.05</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137322.59</v>
+        <v>137390.35</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138280.87</v>
+        <v>138349.11</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137801.73</v>
+        <v>137869.73</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86801.64</v>
+        <v>86844.47</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87504.09</v>
+        <v>87547.27</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87152.86</v>
+        <v>87195.87</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41461.88</v>
+        <v>41482.34</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41395.38</v>
+        <v>41415.81</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41428.63</v>
+        <v>41449.07</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12929.21</v>
+        <v>12935.59</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12786.8</v>
+        <v>12793.11</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12858.01</v>
+        <v>12864.35</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3975</v>
+        <v>13.3993</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4487.25</v>
+        <v>4489.46</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4377.71</v>
+        <v>4379.87</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4432.48</v>
+        <v>4434.66</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-08
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149358.56</v>
+        <v>149431.86</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151241.55</v>
+        <v>151315.77</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150300.06</v>
+        <v>150373.82</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114324.27</v>
+        <v>114380.37</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115101.56</v>
+        <v>115158.05</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114712.91</v>
+        <v>114769.21</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81515.88</v>
+        <v>81555.88</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82023.82000000001</v>
+        <v>82064.08</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81769.85000000001</v>
+        <v>81809.98</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57762.13</v>
+        <v>57790.48</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57324.36</v>
+        <v>57352.49</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57543.25</v>
+        <v>57571.48</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37312.05</v>
+        <v>37330.36</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37617.27</v>
+        <v>37635.73</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37464.66</v>
+        <v>37483.04</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3589</v>
+        <v>13.3608</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16970.21</v>
+        <v>16978.54</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16858.78</v>
+        <v>16867.05</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16914.5</v>
+        <v>16922.8</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162290.31</v>
+        <v>162371.51</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161419.49</v>
+        <v>161500.26</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161854.9</v>
+        <v>161935.88</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121880.52</v>
+        <v>121941.5</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120159.13</v>
+        <v>120219.25</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121019.82</v>
+        <v>121080.38</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87076.05</v>
+        <v>87119.62</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>85997.78999999999</v>
+        <v>86040.82000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86536.92</v>
+        <v>86580.22</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66330.13</v>
+        <v>66363.32000000001</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65863.84</v>
+        <v>65896.78999999999</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66096.98</v>
+        <v>66130.05</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51818.17</v>
+        <v>51844.1</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49955.87</v>
+        <v>49980.87</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50887.02</v>
+        <v>50912.48</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3302</v>
+        <v>13.3293</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39280.98</v>
+        <v>39300.64</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40251.63</v>
+        <v>40271.77</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39766.31</v>
+        <v>39786.2</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167087.54</v>
+        <v>167171.35</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168626.69</v>
+        <v>168711.28</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167857.11</v>
+        <v>167941.31</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120446.84</v>
+        <v>120507.26</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119007.24</v>
+        <v>119066.94</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119727.04</v>
+        <v>119787.1</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82507.99000000001</v>
+        <v>82549.38</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82196.35000000001</v>
+        <v>82237.58</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82352.17</v>
+        <v>82393.48</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54970.78</v>
+        <v>54998.36</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55274.09</v>
+        <v>55301.82</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55122.44</v>
+        <v>55150.09</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33177.67</v>
+        <v>33194.31</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32789.34</v>
+        <v>32805.79</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>32983.5</v>
+        <v>33000.05</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3481</v>
+        <v>13.3473</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17224.44</v>
+        <v>17233.08</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17907.3</v>
+        <v>17916.28</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17565.87</v>
+        <v>17574.68</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129124.19</v>
+        <v>129189.13</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129218.81</v>
+        <v>129283.79</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129171.5</v>
+        <v>129236.46</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89425.27</v>
+        <v>89470.24000000001</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88037.64</v>
+        <v>88081.92</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88731.46000000001</v>
+        <v>88776.08</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56208.8</v>
+        <v>56237.07</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56495.66</v>
+        <v>56524.07</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56352.23</v>
+        <v>56380.57</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29756.98</v>
+        <v>29771.95</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29957.28</v>
+        <v>29972.34</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29857.13</v>
+        <v>29872.14</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6825.01</v>
+        <v>6828.44</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6823.71</v>
+        <v>6827.14</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6824.36</v>
+        <v>6827.79</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3661</v>
+        <v>13.3653</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3792.28</v>
+        <v>3794.18</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3702.83</v>
+        <v>3704.69</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3747.55</v>
+        <v>3749.44</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109014.94</v>
+        <v>109069.9</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109493.2</v>
+        <v>109548.39</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109254.07</v>
+        <v>109309.14</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76450.73</v>
+        <v>76489.27</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75906.82000000001</v>
+        <v>75945.08</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76178.77</v>
+        <v>76217.17</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46260.43</v>
+        <v>46283.75</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47366.46</v>
+        <v>47390.34</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46813.45</v>
+        <v>46837.04</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28739.71</v>
+        <v>28754.19</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28632.6</v>
+        <v>28647.03</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28686.15</v>
+        <v>28700.61</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14098.44</v>
+        <v>14105.54</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14220.67</v>
+        <v>14227.83</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14159.55</v>
+        <v>14166.69</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3833</v>
+        <v>13.3825</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6536.04</v>
+        <v>6539.34</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6374.57</v>
+        <v>6377.78</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6455.31</v>
+        <v>6458.56</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49615.58</v>
+        <v>49640.66</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49283.42</v>
+        <v>49308.32</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49449.5</v>
+        <v>49474.49</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43648.46</v>
+        <v>43670.52</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43842.24</v>
+        <v>43864.4</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43745.35</v>
+        <v>43767.46</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31944.11</v>
+        <v>31960.25</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32284.3</v>
+        <v>32300.62</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32114.21</v>
+        <v>32130.44</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22460.82</v>
+        <v>22472.17</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22615.07</v>
+        <v>22626.5</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22537.94</v>
+        <v>22549.33</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14436.28</v>
+        <v>14443.58</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14641.72</v>
+        <v>14649.12</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14539</v>
+        <v>14546.35</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4013</v>
+        <v>13.4005</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8296.540000000001</v>
+        <v>8300.74</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8351.51</v>
+        <v>8355.73</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8324.030000000001</v>
+        <v>8328.23</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48811.09</v>
+        <v>48835.82</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48092.71</v>
+        <v>48117.08</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48451.9</v>
+        <v>48476.45</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43711.02</v>
+        <v>43733.16</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43375.23</v>
+        <v>43397.21</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43543.12</v>
+        <v>43565.18</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31568.11</v>
+        <v>31584.11</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31000.62</v>
+        <v>31016.33</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31284.37</v>
+        <v>31300.22</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23528.72</v>
+        <v>23540.64</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23423.81</v>
+        <v>23435.68</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23476.26</v>
+        <v>23488.16</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18457.98</v>
+        <v>18467.33</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18272.48</v>
+        <v>18281.74</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18365.23</v>
+        <v>18374.53</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4201</v>
+        <v>13.4193</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15524.42</v>
+        <v>15532.28</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15468.99</v>
+        <v>15476.83</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15496.7</v>
+        <v>15504.56</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108430.34</v>
+        <v>108486.02</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>108979.45</v>
+        <v>109035.42</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108704.89</v>
+        <v>108760.72</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77756.14999999999</v>
+        <v>77796.08</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78070.48</v>
+        <v>78110.57000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>77913.32000000001</v>
+        <v>77953.33</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50793.64</v>
+        <v>50819.73</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50362.26</v>
+        <v>50388.12</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50577.95</v>
+        <v>50603.93</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29202.89</v>
+        <v>29217.89</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>28992.47</v>
+        <v>29007.36</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29097.68</v>
+        <v>29112.62</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16595.71</v>
+        <v>16604.23</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16530.13</v>
+        <v>16538.62</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16562.92</v>
+        <v>16571.42</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4421</v>
+        <v>13.4407</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6728.51</v>
+        <v>6731.97</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6515.6</v>
+        <v>6518.95</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6622.06</v>
+        <v>6625.46</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402044.67</v>
+        <v>402249.35</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397070.38</v>
+        <v>397272.53</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399557.53</v>
+        <v>399760.94</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301826.8</v>
+        <v>301980.46</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302805.69</v>
+        <v>302959.84</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302316.24</v>
+        <v>302470.15</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211189.14</v>
+        <v>211296.66</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211061.73</v>
+        <v>211169.19</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211125.44</v>
+        <v>211232.92</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128390.7</v>
+        <v>128456.07</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128673.69</v>
+        <v>128739.2</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128532.2</v>
+        <v>128597.63</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62232.63</v>
+        <v>62264.32</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61941.9</v>
+        <v>61973.44</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62087.27</v>
+        <v>62118.88</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31783.23</v>
+        <v>31799.41</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31807.24</v>
+        <v>31823.43</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31795.23</v>
+        <v>31811.42</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405594.96</v>
+        <v>405796.44</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406140.12</v>
+        <v>406341.87</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>405867.54</v>
+        <v>406069.16</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301068.82</v>
+        <v>301218.38</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299188.98</v>
+        <v>299337.6</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300128.9</v>
+        <v>300277.99</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204215.25</v>
+        <v>204316.7</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204285.11</v>
+        <v>204386.59</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204250.18</v>
+        <v>204351.64</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123577.74</v>
+        <v>123639.13</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124092.99</v>
+        <v>124154.64</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123835.37</v>
+        <v>123896.88</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49351.44</v>
+        <v>49375.96</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49292.64</v>
+        <v>49317.12</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49322.04</v>
+        <v>49346.54</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5318</v>
+        <v>13.5364</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5428.5</v>
+        <v>5431.2</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5464.3</v>
+        <v>5467.01</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5446.4</v>
+        <v>5449.1</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169408.63</v>
+        <v>169492.75</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169435.73</v>
+        <v>169519.86</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169422.18</v>
+        <v>169506.31</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111329.6</v>
+        <v>111384.88</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110942.31</v>
+        <v>110997.4</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111135.96</v>
+        <v>111191.14</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62349.49</v>
+        <v>62380.45</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62703.14</v>
+        <v>62734.28</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62526.32</v>
+        <v>62557.36</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26692.42</v>
+        <v>26705.68</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26891.28</v>
+        <v>26904.63</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26791.85</v>
+        <v>26805.15</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6283.11</v>
+        <v>6286.23</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6434.15</v>
+        <v>6437.34</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6358.63</v>
+        <v>6361.79</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4416</v>
+        <v>13.4434</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3721.19</v>
+        <v>3723.04</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3714.73</v>
+        <v>3716.58</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3717.96</v>
+        <v>3719.81</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189498.41</v>
+        <v>189591.94</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190423.7</v>
+        <v>190517.69</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>189961.05</v>
+        <v>190054.82</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137390.35</v>
+        <v>137458.17</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138349.11</v>
+        <v>138417.4</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137869.73</v>
+        <v>137937.78</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86844.47</v>
+        <v>86887.33</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87547.27</v>
+        <v>87590.48</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87195.87</v>
+        <v>87238.91</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41482.34</v>
+        <v>41502.81</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41415.81</v>
+        <v>41436.25</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41449.07</v>
+        <v>41469.53</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12935.59</v>
+        <v>12941.98</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12793.11</v>
+        <v>12799.42</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12864.35</v>
+        <v>12870.7</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.3993</v>
+        <v>13.4012</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4489.46</v>
+        <v>4491.68</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4379.87</v>
+        <v>4382.03</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4434.66</v>
+        <v>4436.85</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-09
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149431.86</v>
+        <v>149509.86</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151315.77</v>
+        <v>151394.75</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150373.82</v>
+        <v>150452.3</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114380.37</v>
+        <v>114440.07</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115158.05</v>
+        <v>115218.15</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114769.21</v>
+        <v>114829.11</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81555.88</v>
+        <v>81598.45</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82064.08</v>
+        <v>82106.91</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81809.98</v>
+        <v>81852.67999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57790.48</v>
+        <v>57820.64</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57352.49</v>
+        <v>57382.43</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57571.48</v>
+        <v>57601.53</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37330.36</v>
+        <v>37349.84</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37635.73</v>
+        <v>37655.37</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37483.04</v>
+        <v>37502.61</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3608</v>
+        <v>13.3543</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16978.54</v>
+        <v>16987.4</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16867.05</v>
+        <v>16875.85</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16922.8</v>
+        <v>16931.63</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162371.51</v>
+        <v>162459.04</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161500.26</v>
+        <v>161587.31</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>161935.88</v>
+        <v>162023.17</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>121941.5</v>
+        <v>122007.23</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120219.25</v>
+        <v>120284.05</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121080.38</v>
+        <v>121145.64</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87119.62</v>
+        <v>87166.58</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86040.82000000001</v>
+        <v>86087.2</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86580.22</v>
+        <v>86626.89</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66363.32000000001</v>
+        <v>66399.09</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65896.78999999999</v>
+        <v>65932.31</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66130.05</v>
+        <v>66165.7</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51844.1</v>
+        <v>51872.05</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>49980.87</v>
+        <v>50007.81</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50912.48</v>
+        <v>50939.93</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3293</v>
+        <v>13.3198</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39300.64</v>
+        <v>39321.82</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40271.77</v>
+        <v>40293.48</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39786.2</v>
+        <v>39807.65</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167171.35</v>
+        <v>167266.72</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168711.28</v>
+        <v>168807.53</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>167941.31</v>
+        <v>168037.13</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120507.26</v>
+        <v>120576.01</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119066.94</v>
+        <v>119134.87</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119787.1</v>
+        <v>119855.44</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82549.38</v>
+        <v>82596.47</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82237.58</v>
+        <v>82284.5</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82393.48</v>
+        <v>82440.49000000001</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>54998.36</v>
+        <v>55029.73</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55301.82</v>
+        <v>55333.37</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55150.09</v>
+        <v>55181.55</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33194.31</v>
+        <v>33213.25</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32805.79</v>
+        <v>32824.5</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33000.05</v>
+        <v>33018.88</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3473</v>
+        <v>13.3333</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17233.08</v>
+        <v>17242.91</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17916.28</v>
+        <v>17926.5</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17574.68</v>
+        <v>17584.71</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129189.13</v>
+        <v>129267.79</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129283.79</v>
+        <v>129362.51</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129236.46</v>
+        <v>129315.15</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89470.24000000001</v>
+        <v>89524.72</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88081.92</v>
+        <v>88135.55</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88776.08</v>
+        <v>88830.13</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56237.07</v>
+        <v>56271.31</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56524.07</v>
+        <v>56558.49</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56380.57</v>
+        <v>56414.9</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29771.95</v>
+        <v>29790.07</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29972.34</v>
+        <v>29990.59</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29872.14</v>
+        <v>29890.33</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6828.44</v>
+        <v>6832.6</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6827.14</v>
+        <v>6831.29</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6827.79</v>
+        <v>6831.95</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3653</v>
+        <v>13.3468</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3794.18</v>
+        <v>3796.49</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3704.69</v>
+        <v>3706.95</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3749.44</v>
+        <v>3751.72</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109069.9</v>
+        <v>109141.01</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109548.39</v>
+        <v>109619.82</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109309.14</v>
+        <v>109380.42</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76489.27</v>
+        <v>76539.14</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75945.08</v>
+        <v>75994.60000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76217.17</v>
+        <v>76266.87</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46283.75</v>
+        <v>46313.93</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47390.34</v>
+        <v>47421.24</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46837.04</v>
+        <v>46867.58</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28754.19</v>
+        <v>28772.94</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28647.03</v>
+        <v>28665.71</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28700.61</v>
+        <v>28719.33</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14105.54</v>
+        <v>14114.74</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14227.83</v>
+        <v>14237.11</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14166.69</v>
+        <v>14175.93</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3825</v>
+        <v>13.3596</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6539.34</v>
+        <v>6543.6</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6377.78</v>
+        <v>6381.94</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6458.56</v>
+        <v>6462.77</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49640.66</v>
+        <v>49675.6</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49308.32</v>
+        <v>49343.03</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49474.49</v>
+        <v>49509.32</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43670.52</v>
+        <v>43701.27</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43864.4</v>
+        <v>43895.28</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43767.46</v>
+        <v>43798.27</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31960.25</v>
+        <v>31982.75</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32300.62</v>
+        <v>32323.36</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32130.44</v>
+        <v>32153.06</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22472.17</v>
+        <v>22487.99</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22626.5</v>
+        <v>22642.43</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22549.33</v>
+        <v>22565.21</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14443.58</v>
+        <v>14453.75</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14649.12</v>
+        <v>14659.43</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14546.35</v>
+        <v>14556.59</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4005</v>
+        <v>13.3731</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8300.74</v>
+        <v>8306.58</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8355.73</v>
+        <v>8361.610000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8328.23</v>
+        <v>8334.1</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48835.82</v>
+        <v>48873.21</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48117.08</v>
+        <v>48153.93</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48476.45</v>
+        <v>48513.57</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43733.16</v>
+        <v>43766.65</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43397.21</v>
+        <v>43430.44</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43565.18</v>
+        <v>43598.54</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31584.11</v>
+        <v>31608.29</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31016.33</v>
+        <v>31040.08</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31300.22</v>
+        <v>31324.19</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23540.64</v>
+        <v>23558.66</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23435.68</v>
+        <v>23453.62</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23488.16</v>
+        <v>23506.14</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18467.33</v>
+        <v>18481.47</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18281.74</v>
+        <v>18295.74</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18374.53</v>
+        <v>18388.61</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4193</v>
+        <v>13.3872</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15532.28</v>
+        <v>15544.18</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15476.83</v>
+        <v>15488.68</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15504.56</v>
+        <v>15516.43</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108486.02</v>
+        <v>108577.45</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109035.42</v>
+        <v>109127.3</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108760.72</v>
+        <v>108852.38</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77796.08</v>
+        <v>77861.64</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78110.57000000001</v>
+        <v>78176.39999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>77953.33</v>
+        <v>78019.02</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50819.73</v>
+        <v>50862.56</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50388.12</v>
+        <v>50430.59</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50603.93</v>
+        <v>50646.57</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29217.89</v>
+        <v>29242.51</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29007.36</v>
+        <v>29031.8</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29112.62</v>
+        <v>29137.16</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16604.23</v>
+        <v>16618.22</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16538.62</v>
+        <v>16552.55</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16571.42</v>
+        <v>16585.39</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4407</v>
+        <v>13.4028</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6731.97</v>
+        <v>6737.64</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6518.95</v>
+        <v>6524.44</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6625.46</v>
+        <v>6631.04</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402249.35</v>
+        <v>402451.52</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397272.53</v>
+        <v>397472.2</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399760.94</v>
+        <v>399961.86</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>301980.46</v>
+        <v>302132.23</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>302959.84</v>
+        <v>303112.11</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302470.15</v>
+        <v>302622.17</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211296.66</v>
+        <v>211402.85</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211169.19</v>
+        <v>211275.32</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211232.92</v>
+        <v>211339.09</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128456.07</v>
+        <v>128520.63</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128739.2</v>
+        <v>128803.9</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128597.63</v>
+        <v>128662.27</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62264.32</v>
+        <v>62295.61</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>61973.44</v>
+        <v>62004.59</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62118.88</v>
+        <v>62150.1</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.685</v>
+        <v>13.6948</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31799.41</v>
+        <v>31815.4</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31823.43</v>
+        <v>31839.42</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31811.42</v>
+        <v>31827.41</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>405796.44</v>
+        <v>406000</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406341.87</v>
+        <v>406545.71</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>406069.16</v>
+        <v>406272.85</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301218.38</v>
+        <v>301369.48</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299337.6</v>
+        <v>299487.76</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300277.99</v>
+        <v>300428.62</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204316.7</v>
+        <v>204419.19</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204386.59</v>
+        <v>204489.12</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204351.64</v>
+        <v>204454.15</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123639.13</v>
+        <v>123701.15</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124154.64</v>
+        <v>124216.92</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123896.88</v>
+        <v>123959.04</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49375.96</v>
+        <v>49400.73</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49317.12</v>
+        <v>49341.86</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49346.54</v>
+        <v>49371.29</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5364</v>
+        <v>13.538</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5431.2</v>
+        <v>5433.92</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5467.01</v>
+        <v>5469.75</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5449.1</v>
+        <v>5451.84</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169492.75</v>
+        <v>169578.68</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169519.86</v>
+        <v>169605.81</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169506.31</v>
+        <v>169592.25</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111384.88</v>
+        <v>111441.35</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>110997.4</v>
+        <v>111053.67</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111191.14</v>
+        <v>111247.51</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62380.45</v>
+        <v>62412.08</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62734.28</v>
+        <v>62766.08</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62557.36</v>
+        <v>62589.08</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26705.68</v>
+        <v>26719.21</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26904.63</v>
+        <v>26918.27</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26805.15</v>
+        <v>26818.74</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6286.23</v>
+        <v>6289.42</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6437.34</v>
+        <v>6440.61</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6361.79</v>
+        <v>6365.01</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4434</v>
+        <v>13.4405</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3723.04</v>
+        <v>3724.92</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3716.58</v>
+        <v>3718.46</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3719.81</v>
+        <v>3721.69</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189591.94</v>
+        <v>189690.08</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190517.69</v>
+        <v>190616.31</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190054.82</v>
+        <v>190153.2</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137458.17</v>
+        <v>137529.32</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138417.4</v>
+        <v>138489.05</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>137937.78</v>
+        <v>138009.18</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86887.33</v>
+        <v>86932.31</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87590.48</v>
+        <v>87635.82000000001</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87238.91</v>
+        <v>87284.07000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41502.81</v>
+        <v>41524.29</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41436.25</v>
+        <v>41457.7</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41469.53</v>
+        <v>41491</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12941.98</v>
+        <v>12948.68</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12799.42</v>
+        <v>12806.05</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12870.7</v>
+        <v>12877.36</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4012</v>
+        <v>13.395</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4491.68</v>
+        <v>4494</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4382.03</v>
+        <v>4384.3</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4436.85</v>
+        <v>4439.15</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-10
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149509.86</v>
+        <v>149575.11</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151394.75</v>
+        <v>151460.82</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150452.3</v>
+        <v>150517.97</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114440.07</v>
+        <v>114490.02</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115218.15</v>
+        <v>115268.44</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114829.11</v>
+        <v>114879.23</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81598.45</v>
+        <v>81634.06</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82106.91</v>
+        <v>82142.74000000001</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81852.67999999999</v>
+        <v>81888.39999999999</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57820.64</v>
+        <v>57845.87</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57382.43</v>
+        <v>57407.47</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57601.53</v>
+        <v>57626.67</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37349.84</v>
+        <v>37366.14</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37655.37</v>
+        <v>37671.81</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37502.61</v>
+        <v>37518.97</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3543</v>
+        <v>13.3708</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16987.4</v>
+        <v>16994.82</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16875.85</v>
+        <v>16883.22</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16931.63</v>
+        <v>16939.02</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162459.04</v>
+        <v>162522.76</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161587.31</v>
+        <v>161650.69</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162023.17</v>
+        <v>162086.72</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122007.23</v>
+        <v>122055.08</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120284.05</v>
+        <v>120331.23</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121145.64</v>
+        <v>121193.16</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87166.58</v>
+        <v>87200.77</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86087.2</v>
+        <v>86120.96000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86626.89</v>
+        <v>86660.87</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66399.09</v>
+        <v>66425.13</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65932.31</v>
+        <v>65958.17</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66165.7</v>
+        <v>66191.64999999999</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51872.05</v>
+        <v>51892.39</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50007.81</v>
+        <v>50027.42</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50939.93</v>
+        <v>50959.91</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3198</v>
+        <v>13.3434</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39321.82</v>
+        <v>39337.24</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40293.48</v>
+        <v>40309.29</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39807.65</v>
+        <v>39823.26</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167266.72</v>
+        <v>167320.52</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168807.53</v>
+        <v>168861.82</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168037.13</v>
+        <v>168091.17</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120576.01</v>
+        <v>120614.79</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119134.87</v>
+        <v>119173.18</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119855.44</v>
+        <v>119893.98</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82596.47</v>
+        <v>82623.03</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82284.5</v>
+        <v>82310.96000000001</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82440.49000000001</v>
+        <v>82467</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55029.73</v>
+        <v>55047.43</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55333.37</v>
+        <v>55351.16</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55181.55</v>
+        <v>55199.3</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33213.25</v>
+        <v>33223.93</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32824.5</v>
+        <v>32835.06</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33018.88</v>
+        <v>33029.49</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3333</v>
+        <v>13.3671</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17242.91</v>
+        <v>17248.45</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17926.5</v>
+        <v>17932.27</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17584.71</v>
+        <v>17590.36</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129267.79</v>
+        <v>129298.2</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129362.51</v>
+        <v>129392.94</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129315.15</v>
+        <v>129345.57</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89524.72</v>
+        <v>89545.78</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88135.55</v>
+        <v>88156.28999999999</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88830.13</v>
+        <v>88851.03</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56271.31</v>
+        <v>56284.55</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56558.49</v>
+        <v>56571.79</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56414.9</v>
+        <v>56428.17</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29790.07</v>
+        <v>29797.08</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29990.59</v>
+        <v>29997.65</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29890.33</v>
+        <v>29897.36</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6832.6</v>
+        <v>6834.2</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6831.29</v>
+        <v>6832.9</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6831.95</v>
+        <v>6833.55</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3468</v>
+        <v>13.3908</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3796.49</v>
+        <v>3797.39</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3706.95</v>
+        <v>3707.82</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3751.72</v>
+        <v>3752.6</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109141.01</v>
+        <v>109156.1</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109619.82</v>
+        <v>109634.97</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109380.42</v>
+        <v>109395.54</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76539.14</v>
+        <v>76549.72</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>75994.60000000001</v>
+        <v>76005.10000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76266.87</v>
+        <v>76277.41</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46313.93</v>
+        <v>46320.33</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47421.24</v>
+        <v>47427.79</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46867.58</v>
+        <v>46874.06</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28772.94</v>
+        <v>28776.92</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28665.71</v>
+        <v>28669.67</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28719.33</v>
+        <v>28723.3</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14114.74</v>
+        <v>14116.69</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14237.11</v>
+        <v>14239.08</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14175.93</v>
+        <v>14177.89</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.3596</v>
+        <v>13.4134</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6543.6</v>
+        <v>6544.5</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6381.94</v>
+        <v>6382.82</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6462.77</v>
+        <v>6463.66</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49675.6</v>
+        <v>49676.66</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49343.03</v>
+        <v>49344.08</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49509.32</v>
+        <v>49510.37</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43701.27</v>
+        <v>43702.19</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43895.28</v>
+        <v>43896.21</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43798.27</v>
+        <v>43799.2</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31982.75</v>
+        <v>31983.43</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32323.36</v>
+        <v>32324.04</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32153.06</v>
+        <v>32153.74</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22487.99</v>
+        <v>22488.47</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22642.43</v>
+        <v>22642.91</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22565.21</v>
+        <v>22565.69</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14453.75</v>
+        <v>14454.05</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14659.43</v>
+        <v>14659.74</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14556.59</v>
+        <v>14556.9</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.3731</v>
+        <v>13.4371</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8306.58</v>
+        <v>8306.76</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8361.610000000001</v>
+        <v>8361.790000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8334.1</v>
+        <v>8334.27</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48873.21</v>
+        <v>48867.45</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48153.93</v>
+        <v>48148.25</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48513.57</v>
+        <v>48507.85</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43766.65</v>
+        <v>43761.49</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43430.44</v>
+        <v>43425.32</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43598.54</v>
+        <v>43593.41</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31608.29</v>
+        <v>31604.57</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31040.08</v>
+        <v>31036.42</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31324.19</v>
+        <v>31320.5</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23558.66</v>
+        <v>23555.89</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23453.62</v>
+        <v>23450.86</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23506.14</v>
+        <v>23503.37</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18481.47</v>
+        <v>18479.29</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18295.74</v>
+        <v>18293.59</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18388.61</v>
+        <v>18386.44</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.3872</v>
+        <v>13.4619</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15544.18</v>
+        <v>15542.35</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15488.68</v>
+        <v>15486.85</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15516.43</v>
+        <v>15514.6</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108577.45</v>
+        <v>108550.75</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109127.3</v>
+        <v>109100.47</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108852.38</v>
+        <v>108825.61</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77861.64</v>
+        <v>77842.5</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78176.39999999999</v>
+        <v>78157.17999999999</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78019.02</v>
+        <v>77999.84</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50862.56</v>
+        <v>50850.05</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50430.59</v>
+        <v>50418.18</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50646.57</v>
+        <v>50634.12</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29242.51</v>
+        <v>29235.32</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29031.8</v>
+        <v>29024.67</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29137.16</v>
+        <v>29129.99</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16618.22</v>
+        <v>16614.14</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16552.55</v>
+        <v>16548.48</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16585.39</v>
+        <v>16581.31</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4028</v>
+        <v>13.4857</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6737.64</v>
+        <v>6735.99</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6524.44</v>
+        <v>6522.84</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6631.04</v>
+        <v>6629.41</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402451.52</v>
+        <v>402659.74</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397472.2</v>
+        <v>397677.84</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>399961.86</v>
+        <v>400168.79</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302132.23</v>
+        <v>302288.55</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303112.11</v>
+        <v>303268.93</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302622.17</v>
+        <v>302778.74</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211402.85</v>
+        <v>211512.23</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211275.32</v>
+        <v>211384.63</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211339.09</v>
+        <v>211448.43</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128520.63</v>
+        <v>128587.12</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128803.9</v>
+        <v>128870.54</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128662.27</v>
+        <v>128728.83</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62295.61</v>
+        <v>62327.84</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62004.59</v>
+        <v>62036.67</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62150.1</v>
+        <v>62182.25</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6948</v>
+        <v>13.6822</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31815.4</v>
+        <v>31831.86</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31839.42</v>
+        <v>31855.9</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31827.41</v>
+        <v>31843.88</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>406000</v>
+        <v>406207.15</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406545.71</v>
+        <v>406753.14</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>406272.85</v>
+        <v>406480.15</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301369.48</v>
+        <v>301523.25</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299487.76</v>
+        <v>299640.57</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300428.62</v>
+        <v>300581.91</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204419.19</v>
+        <v>204523.49</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204489.12</v>
+        <v>204593.46</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204454.15</v>
+        <v>204558.47</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123701.15</v>
+        <v>123764.27</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124216.92</v>
+        <v>124280.3</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>123959.04</v>
+        <v>124022.28</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49400.73</v>
+        <v>49425.93</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49341.86</v>
+        <v>49367.04</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49371.29</v>
+        <v>49396.48</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.538</v>
+        <v>13.5336</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5433.92</v>
+        <v>5436.69</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5469.75</v>
+        <v>5472.55</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5451.84</v>
+        <v>5454.62</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169578.68</v>
+        <v>169664.17</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169605.81</v>
+        <v>169691.31</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169592.25</v>
+        <v>169677.74</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111441.35</v>
+        <v>111497.53</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111053.67</v>
+        <v>111109.66</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111247.51</v>
+        <v>111303.6</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62412.08</v>
+        <v>62443.54</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62766.08</v>
+        <v>62797.72</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62589.08</v>
+        <v>62620.63</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26719.21</v>
+        <v>26732.68</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26918.27</v>
+        <v>26931.84</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26818.74</v>
+        <v>26832.26</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6289.42</v>
+        <v>6292.59</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6440.61</v>
+        <v>6443.86</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6365.01</v>
+        <v>6368.22</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4405</v>
+        <v>13.4388</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3724.92</v>
+        <v>3726.8</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3718.46</v>
+        <v>3720.34</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3721.69</v>
+        <v>3723.57</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189690.08</v>
+        <v>189781.43</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190616.31</v>
+        <v>190708.11</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190153.2</v>
+        <v>190244.77</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137529.32</v>
+        <v>137595.55</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138489.05</v>
+        <v>138555.74</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138009.18</v>
+        <v>138075.65</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86932.31</v>
+        <v>86974.17</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87635.82000000001</v>
+        <v>87678.02</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87284.07000000001</v>
+        <v>87326.10000000001</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41524.29</v>
+        <v>41544.29</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41457.7</v>
+        <v>41477.67</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41491</v>
+        <v>41510.98</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12948.68</v>
+        <v>12954.91</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12806.05</v>
+        <v>12812.22</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12877.36</v>
+        <v>12883.56</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.395</v>
+        <v>13.4009</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4494</v>
+        <v>4496.16</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4384.3</v>
+        <v>4386.41</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4439.15</v>
+        <v>4441.29</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-11
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149575.11</v>
+        <v>149645.84</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151460.82</v>
+        <v>151532.44</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150517.97</v>
+        <v>150589.14</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114490.02</v>
+        <v>114544.16</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115268.44</v>
+        <v>115322.94</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114879.23</v>
+        <v>114933.55</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81634.06</v>
+        <v>81672.66</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82142.74000000001</v>
+        <v>82181.59</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81888.39999999999</v>
+        <v>81927.13</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57845.87</v>
+        <v>57873.23</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57407.47</v>
+        <v>57434.62</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57626.67</v>
+        <v>57653.92</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37366.14</v>
+        <v>37383.81</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37671.81</v>
+        <v>37689.62</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37518.97</v>
+        <v>37536.72</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3708</v>
+        <v>13.3776</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>16994.82</v>
+        <v>17002.85</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16883.22</v>
+        <v>16891.2</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16939.02</v>
+        <v>16947.03</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162522.76</v>
+        <v>162594.94</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161650.69</v>
+        <v>161722.48</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162086.72</v>
+        <v>162158.71</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122055.08</v>
+        <v>122109.3</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120331.23</v>
+        <v>120384.68</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121193.16</v>
+        <v>121246.99</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87200.77</v>
+        <v>87239.5</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86120.96000000001</v>
+        <v>86159.21000000001</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86660.87</v>
+        <v>86699.36</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66425.13</v>
+        <v>66454.63</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65958.17</v>
+        <v>65987.47</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66191.64999999999</v>
+        <v>66221.05</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51892.39</v>
+        <v>51915.44</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50027.42</v>
+        <v>50049.64</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50959.91</v>
+        <v>50982.54</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3434</v>
+        <v>13.3555</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39337.24</v>
+        <v>39354.71</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40309.29</v>
+        <v>40327.19</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39823.26</v>
+        <v>39840.95</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167320.52</v>
+        <v>167394.67</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168861.82</v>
+        <v>168936.66</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168091.17</v>
+        <v>168165.67</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120614.79</v>
+        <v>120668.25</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119173.18</v>
+        <v>119226</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119893.98</v>
+        <v>119947.12</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82623.03</v>
+        <v>82659.64999999999</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82310.96000000001</v>
+        <v>82347.45</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82467</v>
+        <v>82503.55</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55047.43</v>
+        <v>55071.83</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55351.16</v>
+        <v>55375.7</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55199.3</v>
+        <v>55223.76</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33223.93</v>
+        <v>33238.66</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32835.06</v>
+        <v>32849.61</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33029.49</v>
+        <v>33044.13</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3671</v>
+        <v>13.3777</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17248.45</v>
+        <v>17256.1</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17932.27</v>
+        <v>17940.22</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17590.36</v>
+        <v>17598.16</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129298.2</v>
+        <v>129353.99</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129392.94</v>
+        <v>129448.77</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129345.57</v>
+        <v>129401.38</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89545.78</v>
+        <v>89584.41</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88156.28999999999</v>
+        <v>88194.32000000001</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88851.03</v>
+        <v>88889.37</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56284.55</v>
+        <v>56308.83</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56571.79</v>
+        <v>56596.2</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56428.17</v>
+        <v>56452.52</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29797.08</v>
+        <v>29809.94</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>29997.65</v>
+        <v>30010.59</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29897.36</v>
+        <v>29910.26</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6834.2</v>
+        <v>6837.15</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6832.9</v>
+        <v>6835.85</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6833.55</v>
+        <v>6836.5</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.3908</v>
+        <v>13.4022</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3797.39</v>
+        <v>3799.02</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3707.82</v>
+        <v>3709.42</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3752.6</v>
+        <v>3754.22</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109156.1</v>
+        <v>109201.84</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109634.97</v>
+        <v>109680.92</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109395.54</v>
+        <v>109441.38</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76549.72</v>
+        <v>76581.8</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76005.10000000001</v>
+        <v>76036.95</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76277.41</v>
+        <v>76309.38</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46320.33</v>
+        <v>46339.74</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47427.79</v>
+        <v>47447.67</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46874.06</v>
+        <v>46893.71</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28776.92</v>
+        <v>28788.98</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28669.67</v>
+        <v>28681.69</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28723.3</v>
+        <v>28735.34</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14116.69</v>
+        <v>14122.61</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14239.08</v>
+        <v>14245.05</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14177.89</v>
+        <v>14183.83</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4134</v>
+        <v>13.4255</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6544.5</v>
+        <v>6547.25</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6382.82</v>
+        <v>6385.5</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6463.66</v>
+        <v>6466.37</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49676.66</v>
+        <v>49696.78</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49344.08</v>
+        <v>49364.07</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49510.37</v>
+        <v>49530.42</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43702.19</v>
+        <v>43719.89</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43896.21</v>
+        <v>43913.99</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43799.2</v>
+        <v>43816.94</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31983.43</v>
+        <v>31996.39</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32324.04</v>
+        <v>32337.14</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32153.74</v>
+        <v>32166.76</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22488.47</v>
+        <v>22497.57</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22642.91</v>
+        <v>22652.08</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22565.69</v>
+        <v>22574.83</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14454.05</v>
+        <v>14459.91</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14659.74</v>
+        <v>14665.68</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14556.9</v>
+        <v>14562.79</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.4371</v>
+        <v>13.45</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8306.76</v>
+        <v>8310.120000000001</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8361.790000000001</v>
+        <v>8365.18</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8334.27</v>
+        <v>8337.65</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48867.45</v>
+        <v>48886.47</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48148.25</v>
+        <v>48166.99</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48507.85</v>
+        <v>48526.73</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43761.49</v>
+        <v>43778.52</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43425.32</v>
+        <v>43442.22</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43593.41</v>
+        <v>43610.37</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31604.57</v>
+        <v>31616.87</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31036.42</v>
+        <v>31048.5</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31320.5</v>
+        <v>31332.68</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23555.89</v>
+        <v>23565.05</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23450.86</v>
+        <v>23459.99</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23503.37</v>
+        <v>23512.52</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18479.29</v>
+        <v>18486.48</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18293.59</v>
+        <v>18300.7</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18386.44</v>
+        <v>18393.59</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4619</v>
+        <v>13.4755</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15542.35</v>
+        <v>15548.39</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15486.85</v>
+        <v>15492.88</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15514.6</v>
+        <v>15520.64</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108550.75</v>
+        <v>108592.22</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109100.47</v>
+        <v>109142.15</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108825.61</v>
+        <v>108867.18</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77842.5</v>
+        <v>77872.24000000001</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78157.17999999999</v>
+        <v>78187.03</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>77999.84</v>
+        <v>78029.64</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50850.05</v>
+        <v>50869.48</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50418.18</v>
+        <v>50437.45</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50634.12</v>
+        <v>50653.46</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29235.32</v>
+        <v>29246.49</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29024.67</v>
+        <v>29035.75</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29129.99</v>
+        <v>29141.12</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16614.14</v>
+        <v>16620.48</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16548.48</v>
+        <v>16554.81</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16581.31</v>
+        <v>16587.64</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4857</v>
+        <v>13.4991</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6735.99</v>
+        <v>6738.56</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6522.84</v>
+        <v>6525.33</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6629.41</v>
+        <v>6631.94</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402659.74</v>
+        <v>402862.69</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397677.84</v>
+        <v>397878.28</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>400168.79</v>
+        <v>400370.48</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302288.55</v>
+        <v>302440.9</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303268.93</v>
+        <v>303421.79</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302778.74</v>
+        <v>302931.34</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211512.23</v>
+        <v>211618.83</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211384.63</v>
+        <v>211491.17</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211448.43</v>
+        <v>211555</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128587.12</v>
+        <v>128651.93</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128870.54</v>
+        <v>128935.5</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128728.83</v>
+        <v>128793.71</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62327.84</v>
+        <v>62359.26</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62036.67</v>
+        <v>62067.93</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62182.25</v>
+        <v>62213.59</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6822</v>
+        <v>13.6906</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31831.86</v>
+        <v>31847.9</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31855.9</v>
+        <v>31871.95</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31843.88</v>
+        <v>31859.93</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>406207.15</v>
+        <v>406409.7</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406753.14</v>
+        <v>406955.96</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>406480.15</v>
+        <v>406682.83</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301523.25</v>
+        <v>301673.59</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299640.57</v>
+        <v>299789.98</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300581.91</v>
+        <v>300731.79</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204523.49</v>
+        <v>204625.47</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204593.46</v>
+        <v>204695.47</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204558.47</v>
+        <v>204660.47</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123764.27</v>
+        <v>123825.98</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124280.3</v>
+        <v>124342.27</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124022.28</v>
+        <v>124084.12</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49425.93</v>
+        <v>49450.58</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49367.04</v>
+        <v>49391.65</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49396.48</v>
+        <v>49421.12</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5336</v>
+        <v>13.5373</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5436.69</v>
+        <v>5439.4</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5472.55</v>
+        <v>5475.27</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5454.62</v>
+        <v>5457.34</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169664.17</v>
+        <v>169749.39</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169691.31</v>
+        <v>169776.54</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169677.74</v>
+        <v>169762.96</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111497.53</v>
+        <v>111553.53</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111109.66</v>
+        <v>111165.46</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111303.6</v>
+        <v>111359.5</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62443.54</v>
+        <v>62474.9</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62797.72</v>
+        <v>62829.26</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62620.63</v>
+        <v>62652.08</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26732.68</v>
+        <v>26746.11</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26931.84</v>
+        <v>26945.37</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26832.26</v>
+        <v>26845.74</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6292.59</v>
+        <v>6295.75</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6443.86</v>
+        <v>6447.09</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6368.22</v>
+        <v>6371.42</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.4388</v>
+        <v>13.438</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3726.8</v>
+        <v>3728.67</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3720.34</v>
+        <v>3722.2</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3723.57</v>
+        <v>3725.44</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189781.43</v>
+        <v>189875.55</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190708.11</v>
+        <v>190802.69</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190244.77</v>
+        <v>190339.12</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137595.55</v>
+        <v>137663.79</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138555.74</v>
+        <v>138624.46</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138075.65</v>
+        <v>138144.12</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>86974.17</v>
+        <v>87017.31</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87678.02</v>
+        <v>87721.50999999999</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87326.10000000001</v>
+        <v>87369.41</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41544.29</v>
+        <v>41564.9</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41477.67</v>
+        <v>41498.24</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41510.98</v>
+        <v>41531.57</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12954.91</v>
+        <v>12961.34</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12812.22</v>
+        <v>12818.57</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12883.56</v>
+        <v>12889.95</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.4009</v>
+        <v>13.402</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4496.16</v>
+        <v>4498.39</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4386.41</v>
+        <v>4388.58</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4441.29</v>
+        <v>4443.49</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>

<commit_message>
Atualização automática - 2026-09-12
</commit_message>
<xml_diff>
--- a/temperatura-sp/Derivativo_Temperatura_SP.xlsx
+++ b/temperatura-sp/Derivativo_Temperatura_SP.xlsx
@@ -3047,7 +3047,7 @@
         </is>
       </c>
       <c r="C4" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D4" s="50" t="n">
         <v>137.2</v>
@@ -3073,13 +3073,13 @@
         <v>0.872</v>
       </c>
       <c r="K4" s="53" t="n">
-        <v>149645.84</v>
+        <v>149649.93</v>
       </c>
       <c r="L4" s="53" t="n">
-        <v>151532.44</v>
+        <v>151536.58</v>
       </c>
       <c r="M4" s="53" t="n">
-        <v>150589.14</v>
+        <v>150593.25</v>
       </c>
       <c r="N4" s="53" t="n">
         <v>684329.84</v>
@@ -3100,7 +3100,7 @@
         </is>
       </c>
       <c r="C5" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D5" s="50" t="n">
         <v>137.2</v>
@@ -3126,13 +3126,13 @@
         <v>0.739</v>
       </c>
       <c r="K5" s="53" t="n">
-        <v>114544.16</v>
+        <v>114547.28</v>
       </c>
       <c r="L5" s="53" t="n">
-        <v>115322.94</v>
+        <v>115326.1</v>
       </c>
       <c r="M5" s="53" t="n">
-        <v>114933.55</v>
+        <v>114936.69</v>
       </c>
       <c r="N5" s="53" t="n">
         <v>564111.6899999999</v>
@@ -3153,7 +3153,7 @@
         </is>
       </c>
       <c r="C6" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D6" s="50" t="n">
         <v>137.2</v>
@@ -3179,13 +3179,13 @@
         <v>0.611</v>
       </c>
       <c r="K6" s="53" t="n">
-        <v>81672.66</v>
+        <v>81674.89999999999</v>
       </c>
       <c r="L6" s="53" t="n">
-        <v>82181.59</v>
+        <v>82183.83</v>
       </c>
       <c r="M6" s="53" t="n">
-        <v>81927.13</v>
+        <v>81929.36</v>
       </c>
       <c r="N6" s="53" t="n">
         <v>443893.54</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="C7" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D7" s="50" t="n">
         <v>137.2</v>
@@ -3232,13 +3232,13 @@
         <v>0.259</v>
       </c>
       <c r="K7" s="53" t="n">
-        <v>57873.23</v>
+        <v>57874.81</v>
       </c>
       <c r="L7" s="53" t="n">
-        <v>57434.62</v>
+        <v>57436.19</v>
       </c>
       <c r="M7" s="53" t="n">
-        <v>57653.92</v>
+        <v>57655.5</v>
       </c>
       <c r="N7" s="53" t="n">
         <v>323675.4</v>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
       <c r="C8" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D8" s="50" t="n">
         <v>137.2</v>
@@ -3285,13 +3285,13 @@
         <v>0.263</v>
       </c>
       <c r="K8" s="53" t="n">
-        <v>37383.81</v>
+        <v>37384.83</v>
       </c>
       <c r="L8" s="53" t="n">
-        <v>37689.62</v>
+        <v>37690.65</v>
       </c>
       <c r="M8" s="53" t="n">
-        <v>37536.72</v>
+        <v>37537.74</v>
       </c>
       <c r="N8" s="53" t="n">
         <v>203457.25</v>
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="C9" s="51" t="n">
-        <v>13.3776</v>
+        <v>13.3702</v>
       </c>
       <c r="D9" s="50" t="n">
         <v>137.2</v>
@@ -3338,13 +3338,13 @@
         <v>0.215</v>
       </c>
       <c r="K9" s="53" t="n">
-        <v>17002.85</v>
+        <v>17003.32</v>
       </c>
       <c r="L9" s="53" t="n">
-        <v>16891.2</v>
+        <v>16891.66</v>
       </c>
       <c r="M9" s="53" t="n">
-        <v>16947.03</v>
+        <v>16947.49</v>
       </c>
       <c r="N9" s="53" t="n">
         <v>90883.74000000001</v>
@@ -3365,7 +3365,7 @@
         </is>
       </c>
       <c r="C10" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D10" s="54" t="n">
         <v>125.2</v>
@@ -3391,13 +3391,13 @@
         <v>0.913</v>
       </c>
       <c r="K10" s="57" t="n">
-        <v>162594.94</v>
+        <v>162600.21</v>
       </c>
       <c r="L10" s="57" t="n">
-        <v>161722.48</v>
+        <v>161727.72</v>
       </c>
       <c r="M10" s="57" t="n">
-        <v>162158.71</v>
+        <v>162163.96</v>
       </c>
       <c r="N10" s="57" t="n">
         <v>268304.58</v>
@@ -3418,7 +3418,7 @@
         </is>
       </c>
       <c r="C11" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D11" s="54" t="n">
         <v>125.2</v>
@@ -3444,13 +3444,13 @@
         <v>0.826</v>
       </c>
       <c r="K11" s="57" t="n">
-        <v>122109.3</v>
+        <v>122113.25</v>
       </c>
       <c r="L11" s="57" t="n">
-        <v>120384.68</v>
+        <v>120388.58</v>
       </c>
       <c r="M11" s="57" t="n">
-        <v>121246.99</v>
+        <v>121250.91</v>
       </c>
       <c r="N11" s="57" t="n">
         <v>152244.07</v>
@@ -3471,7 +3471,7 @@
         </is>
       </c>
       <c r="C12" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D12" s="54" t="n">
         <v>125.2</v>
@@ -3497,13 +3497,13 @@
         <v>0.652</v>
       </c>
       <c r="K12" s="57" t="n">
-        <v>87239.5</v>
+        <v>87242.33</v>
       </c>
       <c r="L12" s="57" t="n">
-        <v>86159.21000000001</v>
+        <v>86162</v>
       </c>
       <c r="M12" s="57" t="n">
-        <v>86699.36</v>
+        <v>86702.17</v>
       </c>
       <c r="N12" s="57" t="n">
         <v>104659.79</v>
@@ -3524,7 +3524,7 @@
         </is>
       </c>
       <c r="C13" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D13" s="54" t="n">
         <v>125.2</v>
@@ -3550,13 +3550,13 @@
         <v>0.351</v>
       </c>
       <c r="K13" s="57" t="n">
-        <v>66454.63</v>
+        <v>66456.78999999999</v>
       </c>
       <c r="L13" s="57" t="n">
-        <v>65987.47</v>
+        <v>65989.61</v>
       </c>
       <c r="M13" s="57" t="n">
-        <v>66221.05</v>
+        <v>66223.2</v>
       </c>
       <c r="N13" s="57" t="n">
         <v>80134.59</v>
@@ -3577,7 +3577,7 @@
         </is>
       </c>
       <c r="C14" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D14" s="54" t="n">
         <v>125.2</v>
@@ -3603,13 +3603,13 @@
         <v>0.173</v>
       </c>
       <c r="K14" s="57" t="n">
-        <v>51915.44</v>
+        <v>51917.12</v>
       </c>
       <c r="L14" s="57" t="n">
-        <v>50049.64</v>
+        <v>50051.27</v>
       </c>
       <c r="M14" s="57" t="n">
-        <v>50982.54</v>
+        <v>50984.19</v>
       </c>
       <c r="N14" s="57" t="n">
         <v>55609.39</v>
@@ -3630,7 +3630,7 @@
         </is>
       </c>
       <c r="C15" s="55" t="n">
-        <v>13.3555</v>
+        <v>13.3481</v>
       </c>
       <c r="D15" s="54" t="n">
         <v>125.2</v>
@@ -3656,13 +3656,13 @@
         <v>0.13</v>
       </c>
       <c r="K15" s="57" t="n">
-        <v>39354.71</v>
+        <v>39355.99</v>
       </c>
       <c r="L15" s="57" t="n">
-        <v>40327.19</v>
+        <v>40328.49</v>
       </c>
       <c r="M15" s="57" t="n">
-        <v>39840.95</v>
+        <v>39842.24</v>
       </c>
       <c r="N15" s="57" t="n">
         <v>31084.18</v>
@@ -3683,7 +3683,7 @@
         </is>
       </c>
       <c r="C16" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D16" s="50" t="n">
         <v>115.9</v>
@@ -3709,13 +3709,13 @@
         <v>0.957</v>
       </c>
       <c r="K16" s="53" t="n">
-        <v>167394.67</v>
+        <v>167400.72</v>
       </c>
       <c r="L16" s="53" t="n">
-        <v>168936.66</v>
+        <v>168942.76</v>
       </c>
       <c r="M16" s="53" t="n">
-        <v>168165.67</v>
+        <v>168171.74</v>
       </c>
       <c r="N16" s="53" t="n">
         <v>754714.99</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="C17" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D17" s="50" t="n">
         <v>115.9</v>
@@ -3762,13 +3762,13 @@
         <v>0.825</v>
       </c>
       <c r="K17" s="53" t="n">
-        <v>120668.25</v>
+        <v>120672.6</v>
       </c>
       <c r="L17" s="53" t="n">
-        <v>119226</v>
+        <v>119230.31</v>
       </c>
       <c r="M17" s="53" t="n">
-        <v>119947.12</v>
+        <v>119951.45</v>
       </c>
       <c r="N17" s="53" t="n">
         <v>660063.6899999999</v>
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="C18" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D18" s="50" t="n">
         <v>115.9</v>
@@ -3815,13 +3815,13 @@
         <v>0.612</v>
       </c>
       <c r="K18" s="53" t="n">
-        <v>82659.64999999999</v>
+        <v>82662.64</v>
       </c>
       <c r="L18" s="53" t="n">
-        <v>82347.45</v>
+        <v>82350.42</v>
       </c>
       <c r="M18" s="53" t="n">
-        <v>82503.55</v>
+        <v>82506.53</v>
       </c>
       <c r="N18" s="53" t="n">
         <v>565412.38</v>
@@ -3842,7 +3842,7 @@
         </is>
       </c>
       <c r="C19" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D19" s="50" t="n">
         <v>115.9</v>
@@ -3868,13 +3868,13 @@
         <v>0.349</v>
       </c>
       <c r="K19" s="53" t="n">
-        <v>55071.83</v>
+        <v>55073.82</v>
       </c>
       <c r="L19" s="53" t="n">
-        <v>55375.7</v>
+        <v>55377.69</v>
       </c>
       <c r="M19" s="53" t="n">
-        <v>55223.76</v>
+        <v>55225.76</v>
       </c>
       <c r="N19" s="53" t="n">
         <v>372763.86</v>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="C20" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D20" s="50" t="n">
         <v>115.9</v>
@@ -3921,13 +3921,13 @@
         <v>0.215</v>
       </c>
       <c r="K20" s="53" t="n">
-        <v>33238.66</v>
+        <v>33239.86</v>
       </c>
       <c r="L20" s="53" t="n">
-        <v>32849.61</v>
+        <v>32850.8</v>
       </c>
       <c r="M20" s="53" t="n">
-        <v>33044.13</v>
+        <v>33045.33</v>
       </c>
       <c r="N20" s="53" t="n">
         <v>130838.89</v>
@@ -3948,7 +3948,7 @@
         </is>
       </c>
       <c r="C21" s="51" t="n">
-        <v>13.3777</v>
+        <v>13.3707</v>
       </c>
       <c r="D21" s="50" t="n">
         <v>115.9</v>
@@ -3974,13 +3974,13 @@
         <v>0.177</v>
       </c>
       <c r="K21" s="53" t="n">
-        <v>17256.1</v>
+        <v>17256.72</v>
       </c>
       <c r="L21" s="53" t="n">
-        <v>17940.22</v>
+        <v>17940.86</v>
       </c>
       <c r="M21" s="53" t="n">
-        <v>17598.16</v>
+        <v>17598.79</v>
       </c>
       <c r="N21" s="53" t="n">
         <v>37203.15</v>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="C22" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D22" s="54" t="n">
         <v>69</v>
@@ -4027,13 +4027,13 @@
         <v>0.915</v>
       </c>
       <c r="K22" s="57" t="n">
-        <v>129353.99</v>
+        <v>129359.05</v>
       </c>
       <c r="L22" s="57" t="n">
-        <v>129448.77</v>
+        <v>129453.83</v>
       </c>
       <c r="M22" s="57" t="n">
-        <v>129401.38</v>
+        <v>129406.44</v>
       </c>
       <c r="N22" s="57" t="n">
         <v>263399.59</v>
@@ -4054,7 +4054,7 @@
         </is>
       </c>
       <c r="C23" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D23" s="54" t="n">
         <v>69</v>
@@ -4080,13 +4080,13 @@
         <v>0.737</v>
       </c>
       <c r="K23" s="57" t="n">
-        <v>89584.41</v>
+        <v>89587.92</v>
       </c>
       <c r="L23" s="57" t="n">
-        <v>88194.32000000001</v>
+        <v>88197.77</v>
       </c>
       <c r="M23" s="57" t="n">
-        <v>88889.37</v>
+        <v>88892.84</v>
       </c>
       <c r="N23" s="57" t="n">
         <v>179697.37</v>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="C24" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D24" s="54" t="n">
         <v>69</v>
@@ -4133,13 +4133,13 @@
         <v>0.524</v>
       </c>
       <c r="K24" s="57" t="n">
-        <v>56308.83</v>
+        <v>56311.04</v>
       </c>
       <c r="L24" s="57" t="n">
-        <v>56596.2</v>
+        <v>56598.41</v>
       </c>
       <c r="M24" s="57" t="n">
-        <v>56452.52</v>
+        <v>56454.72</v>
       </c>
       <c r="N24" s="57" t="n">
         <v>125239.21</v>
@@ -4160,7 +4160,7 @@
         </is>
       </c>
       <c r="C25" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D25" s="54" t="n">
         <v>69</v>
@@ -4186,13 +4186,13 @@
         <v>0.391</v>
       </c>
       <c r="K25" s="57" t="n">
-        <v>29809.94</v>
+        <v>29811.1</v>
       </c>
       <c r="L25" s="57" t="n">
-        <v>30010.59</v>
+        <v>30011.76</v>
       </c>
       <c r="M25" s="57" t="n">
-        <v>29910.26</v>
+        <v>29911.43</v>
       </c>
       <c r="N25" s="57" t="n">
         <v>102444.46</v>
@@ -4213,7 +4213,7 @@
         </is>
       </c>
       <c r="C26" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D26" s="54" t="n">
         <v>69</v>
@@ -4239,13 +4239,13 @@
         <v>0.263</v>
       </c>
       <c r="K26" s="57" t="n">
-        <v>6837.15</v>
+        <v>6837.42</v>
       </c>
       <c r="L26" s="57" t="n">
-        <v>6835.85</v>
+        <v>6836.12</v>
       </c>
       <c r="M26" s="57" t="n">
-        <v>6836.5</v>
+        <v>6836.77</v>
       </c>
       <c r="N26" s="57" t="n">
         <v>28785.13</v>
@@ -4266,7 +4266,7 @@
         </is>
       </c>
       <c r="C27" s="55" t="n">
-        <v>13.4022</v>
+        <v>13.3956</v>
       </c>
       <c r="D27" s="54" t="n">
         <v>69</v>
@@ -4292,13 +4292,13 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="K27" s="57" t="n">
-        <v>3799.02</v>
+        <v>3799.17</v>
       </c>
       <c r="L27" s="57" t="n">
-        <v>3709.42</v>
+        <v>3709.56</v>
       </c>
       <c r="M27" s="57" t="n">
-        <v>3754.22</v>
+        <v>3754.37</v>
       </c>
       <c r="N27" s="57" t="n">
         <v>12442.28</v>
@@ -4319,7 +4319,7 @@
         </is>
       </c>
       <c r="C28" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D28" s="50" t="n">
         <v>21.8</v>
@@ -4345,13 +4345,13 @@
         <v>1</v>
       </c>
       <c r="K28" s="53" t="n">
-        <v>109201.84</v>
+        <v>109206.37</v>
       </c>
       <c r="L28" s="53" t="n">
-        <v>109680.92</v>
+        <v>109685.46</v>
       </c>
       <c r="M28" s="53" t="n">
-        <v>109441.38</v>
+        <v>109445.91</v>
       </c>
       <c r="N28" s="53" t="n">
         <v>370727.33</v>
@@ -4372,7 +4372,7 @@
         </is>
       </c>
       <c r="C29" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D29" s="50" t="n">
         <v>21.8</v>
@@ -4398,13 +4398,13 @@
         <v>0.738</v>
       </c>
       <c r="K29" s="53" t="n">
-        <v>76581.8</v>
+        <v>76584.97</v>
       </c>
       <c r="L29" s="53" t="n">
-        <v>76036.95</v>
+        <v>76040.10000000001</v>
       </c>
       <c r="M29" s="53" t="n">
-        <v>76309.38</v>
+        <v>76312.53999999999</v>
       </c>
       <c r="N29" s="53" t="n">
         <v>303416.13</v>
@@ -4425,7 +4425,7 @@
         </is>
       </c>
       <c r="C30" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D30" s="50" t="n">
         <v>21.8</v>
@@ -4451,13 +4451,13 @@
         <v>0.307</v>
       </c>
       <c r="K30" s="53" t="n">
-        <v>46339.74</v>
+        <v>46341.66</v>
       </c>
       <c r="L30" s="53" t="n">
-        <v>47447.67</v>
+        <v>47449.63</v>
       </c>
       <c r="M30" s="53" t="n">
-        <v>46893.71</v>
+        <v>46895.65</v>
       </c>
       <c r="N30" s="53" t="n">
         <v>226061.25</v>
@@ -4478,7 +4478,7 @@
         </is>
       </c>
       <c r="C31" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D31" s="50" t="n">
         <v>21.8</v>
@@ -4504,13 +4504,13 @@
         <v>0.216</v>
       </c>
       <c r="K31" s="53" t="n">
-        <v>28788.98</v>
+        <v>28790.17</v>
       </c>
       <c r="L31" s="53" t="n">
-        <v>28681.69</v>
+        <v>28682.88</v>
       </c>
       <c r="M31" s="53" t="n">
-        <v>28735.34</v>
+        <v>28736.53</v>
       </c>
       <c r="N31" s="53" t="n">
         <v>147030.84</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C32" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D32" s="50" t="n">
         <v>21.8</v>
@@ -4557,13 +4557,13 @@
         <v>0.176</v>
       </c>
       <c r="K32" s="53" t="n">
-        <v>14122.61</v>
+        <v>14123.19</v>
       </c>
       <c r="L32" s="53" t="n">
-        <v>14245.05</v>
+        <v>14245.64</v>
       </c>
       <c r="M32" s="53" t="n">
-        <v>14183.83</v>
+        <v>14184.41</v>
       </c>
       <c r="N32" s="53" t="n">
         <v>95608.42</v>
@@ -4584,7 +4584,7 @@
         </is>
       </c>
       <c r="C33" s="51" t="n">
-        <v>13.4255</v>
+        <v>13.4193</v>
       </c>
       <c r="D33" s="50" t="n">
         <v>21.8</v>
@@ -4610,13 +4610,13 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="K33" s="53" t="n">
-        <v>6547.25</v>
+        <v>6547.52</v>
       </c>
       <c r="L33" s="53" t="n">
-        <v>6385.5</v>
+        <v>6385.76</v>
       </c>
       <c r="M33" s="53" t="n">
-        <v>6466.37</v>
+        <v>6466.64</v>
       </c>
       <c r="N33" s="53" t="n">
         <v>44185.99</v>
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="C34" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D34" s="54" t="n">
         <v>8</v>
@@ -4663,13 +4663,13 @@
         <v>0.957</v>
       </c>
       <c r="K34" s="57" t="n">
-        <v>49696.78</v>
+        <v>49698.93</v>
       </c>
       <c r="L34" s="57" t="n">
-        <v>49364.07</v>
+        <v>49366.2</v>
       </c>
       <c r="M34" s="57" t="n">
-        <v>49530.42</v>
+        <v>49532.56</v>
       </c>
       <c r="N34" s="57" t="n">
         <v>180244.15</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="C35" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D35" s="54" t="n">
         <v>8</v>
@@ -4716,13 +4716,13 @@
         <v>0.607</v>
       </c>
       <c r="K35" s="57" t="n">
-        <v>43719.89</v>
+        <v>43721.78</v>
       </c>
       <c r="L35" s="57" t="n">
-        <v>43913.99</v>
+        <v>43915.89</v>
       </c>
       <c r="M35" s="57" t="n">
-        <v>43816.94</v>
+        <v>43818.84</v>
       </c>
       <c r="N35" s="57" t="n">
         <v>163867.48</v>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="C36" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D36" s="54" t="n">
         <v>8</v>
@@ -4769,13 +4769,13 @@
         <v>0.48</v>
       </c>
       <c r="K36" s="57" t="n">
-        <v>31996.39</v>
+        <v>31997.77</v>
       </c>
       <c r="L36" s="57" t="n">
-        <v>32337.14</v>
+        <v>32338.53</v>
       </c>
       <c r="M36" s="57" t="n">
-        <v>32166.76</v>
+        <v>32168.15</v>
       </c>
       <c r="N36" s="57" t="n">
         <v>125305.23</v>
@@ -4796,7 +4796,7 @@
         </is>
       </c>
       <c r="C37" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D37" s="54" t="n">
         <v>8</v>
@@ -4822,13 +4822,13 @@
         <v>0.35</v>
       </c>
       <c r="K37" s="57" t="n">
-        <v>22497.57</v>
+        <v>22498.55</v>
       </c>
       <c r="L37" s="57" t="n">
-        <v>22652.08</v>
+        <v>22653.06</v>
       </c>
       <c r="M37" s="57" t="n">
-        <v>22574.83</v>
+        <v>22575.8</v>
       </c>
       <c r="N37" s="57" t="n">
         <v>86742.98</v>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="C38" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D38" s="54" t="n">
         <v>8</v>
@@ -4875,13 +4875,13 @@
         <v>0.218</v>
       </c>
       <c r="K38" s="57" t="n">
-        <v>14459.91</v>
+        <v>14460.53</v>
       </c>
       <c r="L38" s="57" t="n">
-        <v>14665.68</v>
+        <v>14666.31</v>
       </c>
       <c r="M38" s="57" t="n">
-        <v>14562.79</v>
+        <v>14563.42</v>
       </c>
       <c r="N38" s="57" t="n">
         <v>48180.73</v>
@@ -4902,7 +4902,7 @@
         </is>
       </c>
       <c r="C39" s="55" t="n">
-        <v>13.45</v>
+        <v>13.4441</v>
       </c>
       <c r="D39" s="54" t="n">
         <v>8</v>
@@ -4928,13 +4928,13 @@
         <v>0.129</v>
       </c>
       <c r="K39" s="57" t="n">
-        <v>8310.120000000001</v>
+        <v>8310.48</v>
       </c>
       <c r="L39" s="57" t="n">
-        <v>8365.18</v>
+        <v>8365.540000000001</v>
       </c>
       <c r="M39" s="57" t="n">
-        <v>8337.65</v>
+        <v>8338.01</v>
       </c>
       <c r="N39" s="57" t="n">
         <v>38148.18</v>
@@ -4955,7 +4955,7 @@
         </is>
       </c>
       <c r="C40" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D40" s="50" t="n">
         <v>7.2</v>
@@ -4981,13 +4981,13 @@
         <v>0.957</v>
       </c>
       <c r="K40" s="53" t="n">
-        <v>48886.47</v>
+        <v>48888.64</v>
       </c>
       <c r="L40" s="53" t="n">
-        <v>48166.99</v>
+        <v>48169.13</v>
       </c>
       <c r="M40" s="53" t="n">
-        <v>48526.73</v>
+        <v>48528.89</v>
       </c>
       <c r="N40" s="53" t="n">
         <v>176653.37</v>
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="C41" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D41" s="50" t="n">
         <v>7.2</v>
@@ -5034,13 +5034,13 @@
         <v>0.869</v>
       </c>
       <c r="K41" s="53" t="n">
-        <v>43778.52</v>
+        <v>43780.47</v>
       </c>
       <c r="L41" s="53" t="n">
-        <v>43442.22</v>
+        <v>43444.15</v>
       </c>
       <c r="M41" s="53" t="n">
-        <v>43610.37</v>
+        <v>43612.31</v>
       </c>
       <c r="N41" s="53" t="n">
         <v>156054.26</v>
@@ -5061,7 +5061,7 @@
         </is>
       </c>
       <c r="C42" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D42" s="50" t="n">
         <v>7.2</v>
@@ -5087,13 +5087,13 @@
         <v>0.478</v>
       </c>
       <c r="K42" s="53" t="n">
-        <v>31616.87</v>
+        <v>31618.27</v>
       </c>
       <c r="L42" s="53" t="n">
-        <v>31048.5</v>
+        <v>31049.88</v>
       </c>
       <c r="M42" s="53" t="n">
-        <v>31332.68</v>
+        <v>31334.08</v>
       </c>
       <c r="N42" s="53" t="n">
         <v>95240.89</v>
@@ -5114,7 +5114,7 @@
         </is>
       </c>
       <c r="C43" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D43" s="50" t="n">
         <v>7.2</v>
@@ -5140,13 +5140,13 @@
         <v>0.217</v>
       </c>
       <c r="K43" s="53" t="n">
-        <v>23565.05</v>
+        <v>23566.1</v>
       </c>
       <c r="L43" s="53" t="n">
-        <v>23459.99</v>
+        <v>23461.03</v>
       </c>
       <c r="M43" s="53" t="n">
-        <v>23512.52</v>
+        <v>23513.56</v>
       </c>
       <c r="N43" s="53" t="n">
         <v>40108.54</v>
@@ -5167,7 +5167,7 @@
         </is>
       </c>
       <c r="C44" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D44" s="50" t="n">
         <v>7.2</v>
@@ -5193,13 +5193,13 @@
         <v>0.131</v>
       </c>
       <c r="K44" s="53" t="n">
-        <v>18486.48</v>
+        <v>18487.3</v>
       </c>
       <c r="L44" s="53" t="n">
-        <v>18300.7</v>
+        <v>18301.52</v>
       </c>
       <c r="M44" s="53" t="n">
-        <v>18393.59</v>
+        <v>18394.41</v>
       </c>
       <c r="N44" s="53" t="n">
         <v>32942.36</v>
@@ -5220,7 +5220,7 @@
         </is>
       </c>
       <c r="C45" s="51" t="n">
-        <v>13.4755</v>
+        <v>13.4701</v>
       </c>
       <c r="D45" s="50" t="n">
         <v>7.2</v>
@@ -5246,13 +5246,13 @@
         <v>0.08799999999999999</v>
       </c>
       <c r="K45" s="53" t="n">
-        <v>15548.39</v>
+        <v>15549.08</v>
       </c>
       <c r="L45" s="53" t="n">
-        <v>15492.88</v>
+        <v>15493.57</v>
       </c>
       <c r="M45" s="53" t="n">
-        <v>15520.64</v>
+        <v>15521.33</v>
       </c>
       <c r="N45" s="53" t="n">
         <v>25776.17</v>
@@ -5273,7 +5273,7 @@
         </is>
       </c>
       <c r="C46" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D46" s="54" t="n">
         <v>27.4</v>
@@ -5299,13 +5299,13 @@
         <v>1</v>
       </c>
       <c r="K46" s="57" t="n">
-        <v>108592.22</v>
+        <v>108597.01</v>
       </c>
       <c r="L46" s="57" t="n">
-        <v>109142.15</v>
+        <v>109146.97</v>
       </c>
       <c r="M46" s="57" t="n">
-        <v>108867.18</v>
+        <v>108871.99</v>
       </c>
       <c r="N46" s="57" t="n">
         <v>416743.87</v>
@@ -5326,7 +5326,7 @@
         </is>
       </c>
       <c r="C47" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D47" s="54" t="n">
         <v>27.4</v>
@@ -5352,13 +5352,13 @@
         <v>0.697</v>
       </c>
       <c r="K47" s="57" t="n">
-        <v>77872.24000000001</v>
+        <v>77875.67999999999</v>
       </c>
       <c r="L47" s="57" t="n">
-        <v>78187.03</v>
+        <v>78190.49000000001</v>
       </c>
       <c r="M47" s="57" t="n">
-        <v>78029.64</v>
+        <v>78033.08</v>
       </c>
       <c r="N47" s="57" t="n">
         <v>284312.36</v>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="C48" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D48" s="54" t="n">
         <v>27.4</v>
@@ -5405,13 +5405,13 @@
         <v>0.609</v>
       </c>
       <c r="K48" s="57" t="n">
-        <v>50869.48</v>
+        <v>50871.72</v>
       </c>
       <c r="L48" s="57" t="n">
-        <v>50437.45</v>
+        <v>50439.67</v>
       </c>
       <c r="M48" s="57" t="n">
-        <v>50653.46</v>
+        <v>50655.7</v>
       </c>
       <c r="N48" s="57" t="n">
         <v>155579.65</v>
@@ -5432,7 +5432,7 @@
         </is>
       </c>
       <c r="C49" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D49" s="54" t="n">
         <v>27.4</v>
@@ -5458,13 +5458,13 @@
         <v>0.347</v>
       </c>
       <c r="K49" s="57" t="n">
-        <v>29246.49</v>
+        <v>29247.78</v>
       </c>
       <c r="L49" s="57" t="n">
-        <v>29035.75</v>
+        <v>29037.04</v>
       </c>
       <c r="M49" s="57" t="n">
-        <v>29141.12</v>
+        <v>29142.41</v>
       </c>
       <c r="N49" s="57" t="n">
         <v>129090.76</v>
@@ -5485,7 +5485,7 @@
         </is>
       </c>
       <c r="C50" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D50" s="54" t="n">
         <v>27.4</v>
@@ -5511,13 +5511,13 @@
         <v>0.307</v>
       </c>
       <c r="K50" s="57" t="n">
-        <v>16620.48</v>
+        <v>16621.22</v>
       </c>
       <c r="L50" s="57" t="n">
-        <v>16554.81</v>
+        <v>16555.54</v>
       </c>
       <c r="M50" s="57" t="n">
-        <v>16587.64</v>
+        <v>16588.38</v>
       </c>
       <c r="N50" s="57" t="n">
         <v>102601.87</v>
@@ -5538,7 +5538,7 @@
         </is>
       </c>
       <c r="C51" s="55" t="n">
-        <v>13.4991</v>
+        <v>13.4942</v>
       </c>
       <c r="D51" s="54" t="n">
         <v>27.4</v>
@@ -5564,13 +5564,13 @@
         <v>0.171</v>
       </c>
       <c r="K51" s="57" t="n">
-        <v>6738.56</v>
+        <v>6738.86</v>
       </c>
       <c r="L51" s="57" t="n">
-        <v>6525.33</v>
+        <v>6525.62</v>
       </c>
       <c r="M51" s="57" t="n">
-        <v>6631.94</v>
+        <v>6632.24</v>
       </c>
       <c r="N51" s="57" t="n">
         <v>55618.3</v>
@@ -5591,7 +5591,7 @@
         </is>
       </c>
       <c r="C52" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D52" s="50" t="n">
         <v>62</v>
@@ -5617,13 +5617,13 @@
         <v>1</v>
       </c>
       <c r="K52" s="53" t="n">
-        <v>402862.69</v>
+        <v>402865.22</v>
       </c>
       <c r="L52" s="53" t="n">
-        <v>397878.28</v>
+        <v>397880.78</v>
       </c>
       <c r="M52" s="53" t="n">
-        <v>400370.48</v>
+        <v>400373</v>
       </c>
       <c r="N52" s="53" t="n">
         <v>1235846.98</v>
@@ -5644,7 +5644,7 @@
         </is>
       </c>
       <c r="C53" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D53" s="50" t="n">
         <v>62</v>
@@ -5670,13 +5670,13 @@
         <v>0.826</v>
       </c>
       <c r="K53" s="53" t="n">
-        <v>302440.9</v>
+        <v>302442.81</v>
       </c>
       <c r="L53" s="53" t="n">
-        <v>303421.79</v>
+        <v>303423.69</v>
       </c>
       <c r="M53" s="53" t="n">
-        <v>302931.34</v>
+        <v>302933.25</v>
       </c>
       <c r="N53" s="53" t="n">
         <v>966614.62</v>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="C54" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D54" s="50" t="n">
         <v>62</v>
@@ -5723,13 +5723,13 @@
         <v>0.608</v>
       </c>
       <c r="K54" s="53" t="n">
-        <v>211618.83</v>
+        <v>211620.16</v>
       </c>
       <c r="L54" s="53" t="n">
-        <v>211491.17</v>
+        <v>211492.5</v>
       </c>
       <c r="M54" s="53" t="n">
-        <v>211555</v>
+        <v>211556.33</v>
       </c>
       <c r="N54" s="53" t="n">
         <v>814528.73</v>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="C55" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D55" s="50" t="n">
         <v>62</v>
@@ -5776,13 +5776,13 @@
         <v>0.5679999999999999</v>
       </c>
       <c r="K55" s="53" t="n">
-        <v>128651.93</v>
+        <v>128652.74</v>
       </c>
       <c r="L55" s="53" t="n">
-        <v>128935.5</v>
+        <v>128936.31</v>
       </c>
       <c r="M55" s="53" t="n">
-        <v>128793.71</v>
+        <v>128794.52</v>
       </c>
       <c r="N55" s="53" t="n">
         <v>629160.42</v>
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="C56" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D56" s="50" t="n">
         <v>62</v>
@@ -5829,13 +5829,13 @@
         <v>0.348</v>
       </c>
       <c r="K56" s="53" t="n">
-        <v>62359.26</v>
+        <v>62359.65</v>
       </c>
       <c r="L56" s="53" t="n">
-        <v>62067.93</v>
+        <v>62068.32</v>
       </c>
       <c r="M56" s="53" t="n">
-        <v>62213.59</v>
+        <v>62213.99</v>
       </c>
       <c r="N56" s="53" t="n">
         <v>393652.55</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="C57" s="51" t="n">
-        <v>13.6906</v>
+        <v>13.68</v>
       </c>
       <c r="D57" s="50" t="n">
         <v>62</v>
@@ -5882,13 +5882,13 @@
         <v>0.173</v>
       </c>
       <c r="K57" s="53" t="n">
-        <v>31847.9</v>
+        <v>31848.1</v>
       </c>
       <c r="L57" s="53" t="n">
-        <v>31871.95</v>
+        <v>31872.15</v>
       </c>
       <c r="M57" s="53" t="n">
-        <v>31859.93</v>
+        <v>31860.13</v>
       </c>
       <c r="N57" s="53" t="n">
         <v>158144.69</v>
@@ -5909,7 +5909,7 @@
         </is>
       </c>
       <c r="C58" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D58" s="54" t="n">
         <v>90.8</v>
@@ -5935,13 +5935,13 @@
         <v>0.955</v>
       </c>
       <c r="K58" s="57" t="n">
-        <v>406409.7</v>
+        <v>406414.54</v>
       </c>
       <c r="L58" s="57" t="n">
-        <v>406955.96</v>
+        <v>406960.81</v>
       </c>
       <c r="M58" s="57" t="n">
-        <v>406682.83</v>
+        <v>406687.67</v>
       </c>
       <c r="N58" s="57" t="n">
         <v>975967.71</v>
@@ -5962,7 +5962,7 @@
         </is>
       </c>
       <c r="C59" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D59" s="54" t="n">
         <v>90.8</v>
@@ -5988,13 +5988,13 @@
         <v>0.821</v>
       </c>
       <c r="K59" s="57" t="n">
-        <v>301673.59</v>
+        <v>301677.19</v>
       </c>
       <c r="L59" s="57" t="n">
-        <v>299789.98</v>
+        <v>299793.55</v>
       </c>
       <c r="M59" s="57" t="n">
-        <v>300731.79</v>
+        <v>300735.37</v>
       </c>
       <c r="N59" s="57" t="n">
         <v>737350.79</v>
@@ -6015,7 +6015,7 @@
         </is>
       </c>
       <c r="C60" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D60" s="54" t="n">
         <v>90.8</v>
@@ -6041,13 +6041,13 @@
         <v>0.68</v>
       </c>
       <c r="K60" s="57" t="n">
-        <v>204625.47</v>
+        <v>204627.91</v>
       </c>
       <c r="L60" s="57" t="n">
-        <v>204695.47</v>
+        <v>204697.91</v>
       </c>
       <c r="M60" s="57" t="n">
-        <v>204660.47</v>
+        <v>204662.91</v>
       </c>
       <c r="N60" s="57" t="n">
         <v>498733.87</v>
@@ -6068,7 +6068,7 @@
         </is>
       </c>
       <c r="C61" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D61" s="54" t="n">
         <v>90.8</v>
@@ -6094,13 +6094,13 @@
         <v>0.453</v>
       </c>
       <c r="K61" s="57" t="n">
-        <v>123825.98</v>
+        <v>123827.46</v>
       </c>
       <c r="L61" s="57" t="n">
-        <v>124342.27</v>
+        <v>124343.75</v>
       </c>
       <c r="M61" s="57" t="n">
-        <v>124084.12</v>
+        <v>124085.6</v>
       </c>
       <c r="N61" s="57" t="n">
         <v>337463.42</v>
@@ -6121,7 +6121,7 @@
         </is>
       </c>
       <c r="C62" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D62" s="54" t="n">
         <v>90.8</v>
@@ -6147,13 +6147,13 @@
         <v>0.318</v>
       </c>
       <c r="K62" s="57" t="n">
-        <v>49450.58</v>
+        <v>49451.17</v>
       </c>
       <c r="L62" s="57" t="n">
-        <v>49391.65</v>
+        <v>49392.24</v>
       </c>
       <c r="M62" s="57" t="n">
-        <v>49421.12</v>
+        <v>49421.7</v>
       </c>
       <c r="N62" s="57" t="n">
         <v>212357.39</v>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="C63" s="55" t="n">
-        <v>13.5373</v>
+        <v>13.5288</v>
       </c>
       <c r="D63" s="54" t="n">
         <v>90.8</v>
@@ -6200,13 +6200,13 @@
         <v>0.091</v>
       </c>
       <c r="K63" s="57" t="n">
-        <v>5439.4</v>
+        <v>5439.47</v>
       </c>
       <c r="L63" s="57" t="n">
-        <v>5475.27</v>
+        <v>5475.34</v>
       </c>
       <c r="M63" s="57" t="n">
-        <v>5457.34</v>
+        <v>5457.4</v>
       </c>
       <c r="N63" s="57" t="n">
         <v>14501.09</v>
@@ -6227,7 +6227,7 @@
         </is>
       </c>
       <c r="C64" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D64" s="50" t="n">
         <v>98.5</v>
@@ -6253,13 +6253,13 @@
         <v>0.908</v>
       </c>
       <c r="K64" s="53" t="n">
-        <v>169749.39</v>
+        <v>169752.1</v>
       </c>
       <c r="L64" s="53" t="n">
-        <v>169776.54</v>
+        <v>169779.25</v>
       </c>
       <c r="M64" s="53" t="n">
-        <v>169762.96</v>
+        <v>169765.67</v>
       </c>
       <c r="N64" s="53" t="n">
         <v>509626.79</v>
@@ -6280,7 +6280,7 @@
         </is>
       </c>
       <c r="C65" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D65" s="50" t="n">
         <v>98.5</v>
@@ -6306,13 +6306,13 @@
         <v>0.774</v>
       </c>
       <c r="K65" s="53" t="n">
-        <v>111553.53</v>
+        <v>111555.32</v>
       </c>
       <c r="L65" s="53" t="n">
-        <v>111165.46</v>
+        <v>111167.24</v>
       </c>
       <c r="M65" s="53" t="n">
-        <v>111359.5</v>
+        <v>111361.28</v>
       </c>
       <c r="N65" s="53" t="n">
         <v>351103.88</v>
@@ -6333,7 +6333,7 @@
         </is>
       </c>
       <c r="C66" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D66" s="50" t="n">
         <v>98.5</v>
@@ -6359,13 +6359,13 @@
         <v>0.589</v>
       </c>
       <c r="K66" s="53" t="n">
-        <v>62474.9</v>
+        <v>62475.9</v>
       </c>
       <c r="L66" s="53" t="n">
-        <v>62829.26</v>
+        <v>62830.27</v>
       </c>
       <c r="M66" s="53" t="n">
-        <v>62652.08</v>
+        <v>62653.08</v>
       </c>
       <c r="N66" s="53" t="n">
         <v>192580.96</v>
@@ -6386,7 +6386,7 @@
         </is>
       </c>
       <c r="C67" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D67" s="50" t="n">
         <v>98.5</v>
@@ -6412,13 +6412,13 @@
         <v>0.367</v>
       </c>
       <c r="K67" s="53" t="n">
-        <v>26746.11</v>
+        <v>26746.54</v>
       </c>
       <c r="L67" s="53" t="n">
-        <v>26945.37</v>
+        <v>26945.8</v>
       </c>
       <c r="M67" s="53" t="n">
-        <v>26845.74</v>
+        <v>26846.17</v>
       </c>
       <c r="N67" s="53" t="n">
         <v>116932.34</v>
@@ -6439,7 +6439,7 @@
         </is>
       </c>
       <c r="C68" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D68" s="50" t="n">
         <v>98.5</v>
@@ -6465,13 +6465,13 @@
         <v>0.138</v>
       </c>
       <c r="K68" s="53" t="n">
-        <v>6295.75</v>
+        <v>6295.85</v>
       </c>
       <c r="L68" s="53" t="n">
-        <v>6447.09</v>
+        <v>6447.19</v>
       </c>
       <c r="M68" s="53" t="n">
-        <v>6371.42</v>
+        <v>6371.52</v>
       </c>
       <c r="N68" s="53" t="n">
         <v>18552.24</v>
@@ -6492,7 +6492,7 @@
         </is>
       </c>
       <c r="C69" s="51" t="n">
-        <v>13.438</v>
+        <v>13.4304</v>
       </c>
       <c r="D69" s="50" t="n">
         <v>98.5</v>
@@ -6518,13 +6518,13 @@
         <v>0.091</v>
       </c>
       <c r="K69" s="53" t="n">
-        <v>3728.67</v>
+        <v>3728.73</v>
       </c>
       <c r="L69" s="53" t="n">
-        <v>3722.2</v>
+        <v>3722.26</v>
       </c>
       <c r="M69" s="53" t="n">
-        <v>3725.44</v>
+        <v>3725.5</v>
       </c>
       <c r="N69" s="53" t="n">
         <v>3805.76</v>
@@ -6545,7 +6545,7 @@
         </is>
       </c>
       <c r="C70" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D70" s="54" t="n">
         <v>127</v>
@@ -6571,13 +6571,13 @@
         <v>0.908</v>
       </c>
       <c r="K70" s="57" t="n">
-        <v>189875.55</v>
+        <v>189879.67</v>
       </c>
       <c r="L70" s="57" t="n">
-        <v>190802.69</v>
+        <v>190806.83</v>
       </c>
       <c r="M70" s="57" t="n">
-        <v>190339.12</v>
+        <v>190343.25</v>
       </c>
       <c r="N70" s="57" t="n">
         <v>488636.67</v>
@@ -6598,7 +6598,7 @@
         </is>
       </c>
       <c r="C71" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D71" s="54" t="n">
         <v>127</v>
@@ -6624,13 +6624,13 @@
         <v>0.8169999999999999</v>
       </c>
       <c r="K71" s="57" t="n">
-        <v>137663.79</v>
+        <v>137666.78</v>
       </c>
       <c r="L71" s="57" t="n">
-        <v>138624.46</v>
+        <v>138627.46</v>
       </c>
       <c r="M71" s="57" t="n">
-        <v>138144.12</v>
+        <v>138147.12</v>
       </c>
       <c r="N71" s="57" t="n">
         <v>393056.4</v>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="C72" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D72" s="54" t="n">
         <v>127</v>
@@ -6677,13 +6677,13 @@
         <v>0.6820000000000001</v>
       </c>
       <c r="K72" s="57" t="n">
-        <v>87017.31</v>
+        <v>87019.2</v>
       </c>
       <c r="L72" s="57" t="n">
-        <v>87721.50999999999</v>
+        <v>87723.41</v>
       </c>
       <c r="M72" s="57" t="n">
-        <v>87369.41</v>
+        <v>87371.3</v>
       </c>
       <c r="N72" s="57" t="n">
         <v>297476.13</v>
@@ -6704,7 +6704,7 @@
         </is>
       </c>
       <c r="C73" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D73" s="54" t="n">
         <v>127</v>
@@ -6730,13 +6730,13 @@
         <v>0.458</v>
       </c>
       <c r="K73" s="57" t="n">
-        <v>41564.9</v>
+        <v>41565.8</v>
       </c>
       <c r="L73" s="57" t="n">
-        <v>41498.24</v>
+        <v>41499.14</v>
       </c>
       <c r="M73" s="57" t="n">
-        <v>41531.57</v>
+        <v>41532.47</v>
       </c>
       <c r="N73" s="57" t="n">
         <v>181279.06</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C74" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D74" s="54" t="n">
         <v>127</v>
@@ -6783,13 +6783,13 @@
         <v>0.181</v>
       </c>
       <c r="K74" s="57" t="n">
-        <v>12961.34</v>
+        <v>12961.62</v>
       </c>
       <c r="L74" s="57" t="n">
-        <v>12818.57</v>
+        <v>12818.85</v>
       </c>
       <c r="M74" s="57" t="n">
-        <v>12889.95</v>
+        <v>12890.23</v>
       </c>
       <c r="N74" s="57" t="n">
         <v>100943.44</v>
@@ -6810,7 +6810,7 @@
         </is>
       </c>
       <c r="C75" s="55" t="n">
-        <v>13.402</v>
+        <v>13.3945</v>
       </c>
       <c r="D75" s="54" t="n">
         <v>127</v>
@@ -6836,13 +6836,13 @@
         <v>0.089</v>
       </c>
       <c r="K75" s="57" t="n">
-        <v>4498.39</v>
+        <v>4498.49</v>
       </c>
       <c r="L75" s="57" t="n">
-        <v>4388.58</v>
+        <v>4388.68</v>
       </c>
       <c r="M75" s="57" t="n">
-        <v>4443.49</v>
+        <v>4443.59</v>
       </c>
       <c r="N75" s="57" t="n">
         <v>10735.32</v>

</xml_diff>